<commit_message>
Refresh portal status workbook: Briefs 09 and 12, WP08.1h done; business settings live
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/BEE-portal-status.xlsx
+++ b/docs/tracking/BEE-portal-status.xlsx
@@ -586,17 +586,17 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Administration</t>
+          <t>administration</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin</t>
+          <t>business_setting_manage</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -606,7 +606,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>WP08.1h / Brief 12; frontend after backend merge. Provisional business numbers (efficiency cap, report age, tolerances, certificate validity).</t>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: See every business number and the value in force; Propose a change from a date; Approve or reject a colleague's proposal; Withdraw your own proposal.</t>
         </is>
       </c>
     </row>
@@ -5810,7 +5810,7 @@
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -6059,11 +6059,11 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11">
@@ -6134,11 +6134,11 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Pending (blocked)</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14">
@@ -6659,11 +6659,11 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E34" s="3" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
     </row>
     <row r="35">

</xml_diff>

<commit_message>
Refresh portal status workbook: Briefs 09 and 12, WP08.1h done; business settings live (#42)
Co-authored-by: Sameer Khanna <sameerkhanna@Sameers-MacBook-Pro.local>
Co-authored-by: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/BEE-portal-status.xlsx
+++ b/docs/tracking/BEE-portal-status.xlsx
@@ -586,17 +586,17 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Administration</t>
+          <t>administration</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin</t>
+          <t>business_setting_manage</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>Planned</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -606,7 +606,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>WP08.1h / Brief 12; frontend after backend merge. Provisional business numbers (efficiency cap, report age, tolerances, certificate validity).</t>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: See every business number and the value in force; Propose a change from a date; Approve or reject a colleague's proposal; Withdraw your own proposal.</t>
         </is>
       </c>
     </row>
@@ -5810,7 +5810,7 @@
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -6059,11 +6059,11 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11">
@@ -6134,11 +6134,11 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Pending (blocked)</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14">
@@ -6659,11 +6659,11 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E34" s="3" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
     </row>
     <row r="35">

</xml_diff>

<commit_message>
Accept WP05.1d evidence gates as a local activity; refresh status workbook
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/BEE-portal-status.xlsx
+++ b/docs/tracking/BEE-portal-status.xlsx
@@ -6309,11 +6309,11 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E20" s="3" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
Accept WP05.1d; plan WP04.2b registration (#43)
* Accept WP05.1d evidence gates as a local activity; refresh status workbook

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

* Plan WP04.2b brand and agency registration with the owner's default answers

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

---------

Co-authored-by: Sameer Khanna <sameerkhanna@Sameers-MacBook-Pro.local>
Co-authored-by: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/BEE-portal-status.xlsx
+++ b/docs/tracking/BEE-portal-status.xlsx
@@ -6309,11 +6309,11 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E20" s="3" t="n">
-        <v>70</v>
+        <v>100</v>
       </c>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
Refresh portal status workbook: WP04.2b-1, WP04.2b-2, Briefs 13 and 14 done; four live registration screens
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/BEE-portal-status.xlsx
+++ b/docs/tracking/BEE-portal-status.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G145"/>
+  <dimension ref="A1:G149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -5127,27 +5127,27 @@
     <row r="128">
       <c r="A128" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/brand-withdrawal</t>
+          <t>registrations/new</t>
         </is>
       </c>
       <c r="B128" s="3" t="inlineStr">
         <is>
-          <t>Brand withdrawal</t>
+          <t>New registration request</t>
         </is>
       </c>
       <c r="C128" s="3" t="inlineStr">
         <is>
-          <t>Withdrawal</t>
+          <t>registrations</t>
         </is>
       </c>
       <c r="D128" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E128" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F128" s="3" t="inlineStr">
@@ -5157,130 +5157,130 @@
       </c>
       <c r="G128" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: File a brand request; Ask to act for a brand; Save a draft.</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/deposit-release</t>
+          <t>registrations/request</t>
         </is>
       </c>
       <c r="B129" s="3" t="inlineStr">
         <is>
-          <t>Deposit release</t>
+          <t>Registration request</t>
         </is>
       </c>
       <c r="C129" s="3" t="inlineStr">
         <is>
-          <t>Withdrawal</t>
+          <t>registrations</t>
         </is>
       </c>
       <c r="D129" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E129" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F129" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G129" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: See the request; Upload the trade licence; See the fee and submit; Follow the request until Programme review; Recommend or return; Approve, return or reject; See why it was returned and resubmit.</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/dues-verification</t>
+          <t>registrations/requests</t>
         </is>
       </c>
       <c r="B130" s="3" t="inlineStr">
         <is>
-          <t>Dues verification</t>
+          <t>Registration requests</t>
         </is>
       </c>
       <c r="C130" s="3" t="inlineStr">
         <is>
-          <t>Withdrawal</t>
+          <t>registrations</t>
         </is>
       </c>
       <c r="D130" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance</t>
+          <t>manufacturer, agency</t>
         </is>
       </c>
       <c r="E130" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F130" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G130" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: List your registration requests; Open a request; Start a new request.</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/model-withdrawal</t>
+          <t>registrations/reviews</t>
         </is>
       </c>
       <c r="B131" s="3" t="inlineStr">
         <is>
-          <t>Model withdrawal</t>
+          <t>Registration reviews</t>
         </is>
       </c>
       <c r="C131" s="3" t="inlineStr">
         <is>
-          <t>Withdrawal</t>
+          <t>registrations</t>
         </is>
       </c>
       <c r="D131" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance</t>
+          <t>programme, director</t>
         </is>
       </c>
       <c r="E131" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F131" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G131" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: List requests waiting for you; Recommend or return; Approve, return or reject; Read the trail.</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/revocation-initiation</t>
+          <t>withdrawal/brand-withdrawal</t>
         </is>
       </c>
       <c r="B132" s="3" t="inlineStr">
         <is>
-          <t>Revocation initiation</t>
+          <t>Brand withdrawal</t>
         </is>
       </c>
       <c r="C132" s="3" t="inlineStr">
@@ -5300,7 +5300,7 @@
       </c>
       <c r="F132" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G132" s="3" t="inlineStr">
@@ -5312,12 +5312,12 @@
     <row r="133">
       <c r="A133" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/withdrawal-approval</t>
+          <t>withdrawal/deposit-release</t>
         </is>
       </c>
       <c r="B133" s="3" t="inlineStr">
         <is>
-          <t>Withdrawal approval</t>
+          <t>Deposit release</t>
         </is>
       </c>
       <c r="C133" s="3" t="inlineStr">
@@ -5349,12 +5349,12 @@
     <row r="134">
       <c r="A134" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/withdrawal-letter</t>
+          <t>withdrawal/dues-verification</t>
         </is>
       </c>
       <c r="B134" s="3" t="inlineStr">
         <is>
-          <t>Withdrawal letter</t>
+          <t>Dues verification</t>
         </is>
       </c>
       <c r="C134" s="3" t="inlineStr">
@@ -5386,12 +5386,12 @@
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/withdrawal-scrutiny</t>
+          <t>withdrawal/model-withdrawal</t>
         </is>
       </c>
       <c r="B135" s="3" t="inlineStr">
         <is>
-          <t>Withdrawal scrutiny</t>
+          <t>Model withdrawal</t>
         </is>
       </c>
       <c r="C135" s="3" t="inlineStr">
@@ -5423,27 +5423,27 @@
     <row r="136">
       <c r="A136" s="3" t="inlineStr">
         <is>
-          <t>workflow/application-review</t>
+          <t>withdrawal/revocation-initiation</t>
         </is>
       </c>
       <c r="B136" s="3" t="inlineStr">
         <is>
-          <t>Application review</t>
+          <t>Revocation initiation</t>
         </is>
       </c>
       <c r="C136" s="3" t="inlineStr">
         <is>
-          <t>Workflow</t>
+          <t>Withdrawal</t>
         </is>
       </c>
       <c r="D136" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance</t>
         </is>
       </c>
       <c r="E136" s="3" t="inlineStr">
         <is>
-          <t>Live – BEE service</t>
+          <t>Prototype (preview/sample data)</t>
         </is>
       </c>
       <c r="F136" s="3" t="inlineStr">
@@ -5453,29 +5453,29 @@
       </c>
       <c r="G136" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu by role or permission. Capabilities today: List the applications in progress; Link to your next action; Link to the history.</t>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
         <is>
-          <t>workflow/approval-note</t>
+          <t>withdrawal/withdrawal-approval</t>
         </is>
       </c>
       <c r="B137" s="3" t="inlineStr">
         <is>
-          <t>Approval note</t>
+          <t>Withdrawal approval</t>
         </is>
       </c>
       <c r="C137" s="3" t="inlineStr">
         <is>
-          <t>Workflow</t>
+          <t>Withdrawal</t>
         </is>
       </c>
       <c r="D137" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance</t>
         </is>
       </c>
       <c r="E137" s="3" t="inlineStr">
@@ -5497,22 +5497,22 @@
     <row r="138">
       <c r="A138" s="3" t="inlineStr">
         <is>
-          <t>workflow/checklist</t>
+          <t>withdrawal/withdrawal-letter</t>
         </is>
       </c>
       <c r="B138" s="3" t="inlineStr">
         <is>
-          <t>Checklist</t>
+          <t>Withdrawal letter</t>
         </is>
       </c>
       <c r="C138" s="3" t="inlineStr">
         <is>
-          <t>Workflow</t>
+          <t>Withdrawal</t>
         </is>
       </c>
       <c r="D138" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance</t>
         </is>
       </c>
       <c r="E138" s="3" t="inlineStr">
@@ -5534,22 +5534,22 @@
     <row r="139">
       <c r="A139" s="3" t="inlineStr">
         <is>
-          <t>workflow/clarification-and-return</t>
+          <t>withdrawal/withdrawal-scrutiny</t>
         </is>
       </c>
       <c r="B139" s="3" t="inlineStr">
         <is>
-          <t>Clarification and return</t>
+          <t>Withdrawal scrutiny</t>
         </is>
       </c>
       <c r="C139" s="3" t="inlineStr">
         <is>
-          <t>Workflow</t>
+          <t>Withdrawal</t>
         </is>
       </c>
       <c r="D139" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance</t>
         </is>
       </c>
       <c r="E139" s="3" t="inlineStr">
@@ -5571,12 +5571,12 @@
     <row r="140">
       <c r="A140" s="3" t="inlineStr">
         <is>
-          <t>workflow/delegation-and-reassignment</t>
+          <t>workflow/application-review</t>
         </is>
       </c>
       <c r="B140" s="3" t="inlineStr">
         <is>
-          <t>Delegation and reassignment</t>
+          <t>Application review</t>
         </is>
       </c>
       <c r="C140" s="3" t="inlineStr">
@@ -5591,7 +5591,7 @@
       </c>
       <c r="E140" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F140" s="3" t="inlineStr">
@@ -5601,19 +5601,19 @@
       </c>
       <c r="G140" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t xml:space="preserve"> Spring menu by role or permission. Capabilities today: List the applications in progress; Link to your next action; Link to the history.</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="3" t="inlineStr">
         <is>
-          <t>workflow/escalation-dashboard</t>
+          <t>workflow/approval-note</t>
         </is>
       </c>
       <c r="B141" s="3" t="inlineStr">
         <is>
-          <t>Escalation dashboard</t>
+          <t>Approval note</t>
         </is>
       </c>
       <c r="C141" s="3" t="inlineStr">
@@ -5628,66 +5628,66 @@
       </c>
       <c r="E141" s="3" t="inlineStr">
         <is>
-          <t>Live – BEE service</t>
+          <t>Prototype (preview/sample data)</t>
         </is>
       </c>
       <c r="F141" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G141" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu by role or permission. Capabilities today: Count the applications waiting at each stage (no time limits are set yet).</t>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="3" t="inlineStr">
         <is>
-          <t>workflow/my-approvals</t>
+          <t>workflow/checklist</t>
         </is>
       </c>
       <c r="B142" s="3" t="inlineStr">
         <is>
-          <t>My approvals</t>
+          <t>Checklist</t>
         </is>
       </c>
       <c r="C142" s="3" t="inlineStr">
         <is>
-          <t>workflow</t>
+          <t>Workflow</t>
         </is>
       </c>
       <c r="D142" s="3" t="inlineStr">
         <is>
-          <t>director, secretary</t>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
         </is>
       </c>
       <c r="E142" s="3" t="inlineStr">
         <is>
-          <t>Live – BEE service</t>
+          <t>Prototype (preview/sample data)</t>
         </is>
       </c>
       <c r="F142" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G142" s="3" t="inlineStr">
         <is>
-          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: List the applications waiting for your decision; Open the approval screen.</t>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="3" t="inlineStr">
         <is>
-          <t>workflow/personal-inbox</t>
+          <t>workflow/clarification-and-return</t>
         </is>
       </c>
       <c r="B143" s="3" t="inlineStr">
         <is>
-          <t>Personal inbox</t>
+          <t>Clarification and return</t>
         </is>
       </c>
       <c r="C143" s="3" t="inlineStr">
@@ -5702,29 +5702,29 @@
       </c>
       <c r="E143" s="3" t="inlineStr">
         <is>
-          <t>Live – BEE service</t>
+          <t>Prototype (preview/sample data)</t>
         </is>
       </c>
       <c r="F143" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G143" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu roles include: manufacturer, agency, finance, iame, reviewer, programme, director, secretary. Capabilities today: List the applications waiting for you; Open the screen where each is done.</t>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="3" t="inlineStr">
         <is>
-          <t>workflow/team-queue</t>
+          <t>workflow/delegation-and-reassignment</t>
         </is>
       </c>
       <c r="B144" s="3" t="inlineStr">
         <is>
-          <t>Team queue</t>
+          <t>Delegation and reassignment</t>
         </is>
       </c>
       <c r="C144" s="3" t="inlineStr">
@@ -5756,35 +5756,183 @@
     <row r="145">
       <c r="A145" s="3" t="inlineStr">
         <is>
+          <t>workflow/escalation-dashboard</t>
+        </is>
+      </c>
+      <c r="B145" s="3" t="inlineStr">
+        <is>
+          <t>Escalation dashboard</t>
+        </is>
+      </c>
+      <c r="C145" s="3" t="inlineStr">
+        <is>
+          <t>Workflow</t>
+        </is>
+      </c>
+      <c r="D145" s="3" t="inlineStr">
+        <is>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
+        </is>
+      </c>
+      <c r="E145" s="3" t="inlineStr">
+        <is>
+          <t>Live – BEE service</t>
+        </is>
+      </c>
+      <c r="F145" s="3" t="inlineStr">
+        <is>
+          <t>keep</t>
+        </is>
+      </c>
+      <c r="G145" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Spring menu by role or permission. Capabilities today: Count the applications waiting at each stage (no time limits are set yet).</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="3" t="inlineStr">
+        <is>
+          <t>workflow/my-approvals</t>
+        </is>
+      </c>
+      <c r="B146" s="3" t="inlineStr">
+        <is>
+          <t>My approvals</t>
+        </is>
+      </c>
+      <c r="C146" s="3" t="inlineStr">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="D146" s="3" t="inlineStr">
+        <is>
+          <t>director, secretary</t>
+        </is>
+      </c>
+      <c r="E146" s="3" t="inlineStr">
+        <is>
+          <t>Live – BEE service</t>
+        </is>
+      </c>
+      <c r="F146" s="3" t="inlineStr">
+        <is>
+          <t>keep</t>
+        </is>
+      </c>
+      <c r="G146" s="3" t="inlineStr">
+        <is>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: List the applications waiting for your decision; Open the approval screen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="3" t="inlineStr">
+        <is>
+          <t>workflow/personal-inbox</t>
+        </is>
+      </c>
+      <c r="B147" s="3" t="inlineStr">
+        <is>
+          <t>Personal inbox</t>
+        </is>
+      </c>
+      <c r="C147" s="3" t="inlineStr">
+        <is>
+          <t>Workflow</t>
+        </is>
+      </c>
+      <c r="D147" s="3" t="inlineStr">
+        <is>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
+        </is>
+      </c>
+      <c r="E147" s="3" t="inlineStr">
+        <is>
+          <t>Live – BEE service</t>
+        </is>
+      </c>
+      <c r="F147" s="3" t="inlineStr">
+        <is>
+          <t>keep</t>
+        </is>
+      </c>
+      <c r="G147" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Spring menu roles include: manufacturer, agency, finance, iame, reviewer, programme, director, secretary. Capabilities today: List the applications waiting for you; Open the screen where each is done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="3" t="inlineStr">
+        <is>
+          <t>workflow/team-queue</t>
+        </is>
+      </c>
+      <c r="B148" s="3" t="inlineStr">
+        <is>
+          <t>Team queue</t>
+        </is>
+      </c>
+      <c r="C148" s="3" t="inlineStr">
+        <is>
+          <t>Workflow</t>
+        </is>
+      </c>
+      <c r="D148" s="3" t="inlineStr">
+        <is>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
+        </is>
+      </c>
+      <c r="E148" s="3" t="inlineStr">
+        <is>
+          <t>Prototype (preview/sample data)</t>
+        </is>
+      </c>
+      <c r="F148" s="3" t="inlineStr">
+        <is>
+          <t>merge</t>
+        </is>
+      </c>
+      <c r="G148" s="3" t="inlineStr">
+        <is>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="3" t="inlineStr">
+        <is>
           <t>workflow/workflow-history</t>
         </is>
       </c>
-      <c r="B145" s="3" t="inlineStr">
+      <c r="B149" s="3" t="inlineStr">
         <is>
           <t>Workflow history</t>
         </is>
       </c>
-      <c r="C145" s="3" t="inlineStr">
+      <c r="C149" s="3" t="inlineStr">
         <is>
           <t>Workflow</t>
         </is>
       </c>
-      <c r="D145" s="3" t="inlineStr">
+      <c r="D149" s="3" t="inlineStr">
         <is>
           <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
         </is>
       </c>
-      <c r="E145" s="3" t="inlineStr">
+      <c r="E149" s="3" t="inlineStr">
         <is>
           <t>Live – BEE service</t>
         </is>
       </c>
-      <c r="F145" s="3" t="inlineStr">
-        <is>
-          <t>merge</t>
-        </is>
-      </c>
-      <c r="G145" s="3" t="inlineStr">
+      <c r="F149" s="3" t="inlineStr">
+        <is>
+          <t>merge</t>
+        </is>
+      </c>
+      <c r="G149" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve"> Spring menu by role or permission. Capabilities today: Choose an application; Read its steps as you are allowed to see them.</t>
         </is>
@@ -5804,7 +5952,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6144,42 +6292,42 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Work package</t>
+          <t>Cursor brief</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>WP02</t>
+          <t>BRIEF-13</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Identity, session, MFA, model-application policy</t>
+          <t>Registration applicant screens (list, form, request, licence, fee)</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Work package</t>
+          <t>Cursor brief</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>WP03</t>
+          <t>BRIEF-14</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>OpenAPI contract, BFF, contract tests</t>
+          <t>Registration review screens and applicant's returned path</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -6199,12 +6347,12 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>WP04</t>
+          <t>WP02</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Masters and brand authorisation</t>
+          <t>Identity, session, MFA, model-application policy</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -6213,7 +6361,7 @@
         </is>
       </c>
       <c r="E16" s="3" t="n">
-        <v>60</v>
+        <v>75</v>
       </c>
     </row>
     <row r="17">
@@ -6224,12 +6372,12 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>WP05.1a</t>
+          <t>WP03</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Read-only model applications UI</t>
+          <t>OpenAPI contract, BFF, contract tests</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -6249,21 +6397,21 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>WP05.1b</t>
+          <t>WP04</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Draft create/edit</t>
+          <t>Masters and brand authorisation</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="E18" s="3" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
     </row>
     <row r="19">
@@ -6274,12 +6422,12 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>WP05.1c</t>
+          <t>WP04.2b-1</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Draft submission</t>
+          <t>Registration: file, trade-licence PDF, fee, Finance confirmation</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -6299,12 +6447,12 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>WP05.1d</t>
+          <t>WP04.2b-2</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Submit-time evidence gates</t>
+          <t>Registration: recommend, approve, return, reject, resubmit; register entry</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -6324,21 +6472,21 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>WP06.1a</t>
+          <t>WP04.2b-2b</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Document intake and storage</t>
+          <t>Revocation and closure of a brand or authorisation by a second person</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E21" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -6349,17 +6497,17 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>WP06.2</t>
+          <t>WP04.2b-3</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Blob retention, orphans, limits (BL-001–003)</t>
+          <t>Model submit uses the registered brand (brand id)</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="E22" s="3" t="n">
@@ -6374,12 +6522,12 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>WP07.1a</t>
+          <t>WP05.1a</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Finance fee confirmation</t>
+          <t>Read-only model applications UI</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -6399,12 +6547,12 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>WP07.1b–f</t>
+          <t>WP05.1b</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>IAME, Reviewer, Rating, Director, Secretary stages</t>
+          <t>Draft create/edit</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -6424,12 +6572,12 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>WP07.1g–h</t>
+          <t>WP05.1c</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Return, resubmit, rejection</t>
+          <t>Draft submission</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -6449,12 +6597,12 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>WP07.1i–k</t>
+          <t>WP05.1d</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>History, inbox, workflow views</t>
+          <t>Submit-time evidence gates</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -6474,12 +6622,12 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>WP08.1a</t>
+          <t>WP06.1a</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Fee rule administration</t>
+          <t>Document intake and storage</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -6499,21 +6647,21 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>WP08.1b</t>
+          <t>WP06.2</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Tax line on fee rules</t>
+          <t>Blob retention, orphans, limits (BL-001–003)</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E28" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -6524,12 +6672,12 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>WP08.1c</t>
+          <t>WP07.1a</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Rating schemes administration</t>
+          <t>Finance fee confirmation</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -6549,12 +6697,12 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>WP08.1d</t>
+          <t>WP07.1b–f</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Permission-based admin menu</t>
+          <t>IAME, Reviewer, Rating, Director, Secretary stages</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -6574,12 +6722,12 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>WP08.1e</t>
+          <t>WP07.1g–h</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Fee confirmation correction proposals</t>
+          <t>Return, resubmit, rejection</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -6599,12 +6747,12 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>WP08.1f</t>
+          <t>WP07.1i–k</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Fee reversal</t>
+          <t>History, inbox, workflow views</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -6624,12 +6772,12 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>WP08.1g</t>
+          <t>WP08.1a</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Born-pending and notification proof</t>
+          <t>Fee rule administration</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -6649,12 +6797,12 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>WP08.1h</t>
+          <t>WP08.1b</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Business settings (propose/approve numbers)</t>
+          <t>Tax line on fee rules</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -6674,12 +6822,12 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>WP09.1a</t>
+          <t>WP08.1c</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Certificate record</t>
+          <t>Rating schemes administration</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -6699,12 +6847,12 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>WP09.1b</t>
+          <t>WP08.1d</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Printable certificate and label</t>
+          <t>Permission-based admin menu</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -6724,12 +6872,12 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>WP09.1c</t>
+          <t>WP08.1e</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Public verification page</t>
+          <t>Fee confirmation correction proposals</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -6749,12 +6897,12 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>WP09.1d</t>
+          <t>WP08.1f</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Verification rate limit</t>
+          <t>Fee reversal</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -6774,12 +6922,12 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>WP10.1a</t>
+          <t>WP08.1g</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>In-portal notifications (API)</t>
+          <t>Born-pending and notification proof</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -6799,12 +6947,12 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>WP10.1b</t>
+          <t>WP08.1h</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Notification bell and page</t>
+          <t>Business settings (propose/approve numbers)</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -6824,37 +6972,37 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>WP11</t>
+          <t>WP09.1a</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>AI demonstrations (local)</t>
+          <t>Certificate record</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E41" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>Platform</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>WP01</t>
+          <t>WP09.1b</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Documentation and design evidence</t>
+          <t>Printable certificate and label</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -6869,75 +7017,225 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>Backlog theme</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>BL-024/025</t>
+          <t>WP09.1c</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Feature template and OpenAPI split</t>
+          <t>Public verification page</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E43" s="3" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>Backlog theme</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>BL-040–042</t>
+          <t>WP09.1d</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+          <t>Verification rate limit</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E44" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
+          <t>Work package</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>WP10.1a</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>In-portal notifications (API)</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>Work package</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>WP10.1b</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>Notification bell and page</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>Work package</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>WP11</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>AI demonstrations (local)</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>WP01</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>Documentation and design evidence</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>Backlog theme</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>BL-024/025</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>Feature template and OpenAPI split</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>Backlog theme</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>BL-040–042</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
           <t>Owner decision</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
+      <c r="B51" s="3" t="inlineStr">
         <is>
           <t>D10</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr">
+      <c r="C51" s="3" t="inlineStr">
         <is>
           <t>Provisional local rules for notifications (portal only)</t>
         </is>
       </c>
-      <c r="D45" s="3" t="inlineStr">
+      <c r="D51" s="3" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
-      <c r="E45" s="3" t="n">
+      <c r="E51" s="3" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Refresh portal status workbook: WP04.2b-1, WP04.2b-2, Briefs 13 and 14 done; four live registration screens (#48)
Co-authored-by: Sameer Khanna <sameerkhanna@Sameers-MacBook-Pro.local>
Co-authored-by: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/BEE-portal-status.xlsx
+++ b/docs/tracking/BEE-portal-status.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G145"/>
+  <dimension ref="A1:G149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -5127,27 +5127,27 @@
     <row r="128">
       <c r="A128" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/brand-withdrawal</t>
+          <t>registrations/new</t>
         </is>
       </c>
       <c r="B128" s="3" t="inlineStr">
         <is>
-          <t>Brand withdrawal</t>
+          <t>New registration request</t>
         </is>
       </c>
       <c r="C128" s="3" t="inlineStr">
         <is>
-          <t>Withdrawal</t>
+          <t>registrations</t>
         </is>
       </c>
       <c r="D128" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E128" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F128" s="3" t="inlineStr">
@@ -5157,130 +5157,130 @@
       </c>
       <c r="G128" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: File a brand request; Ask to act for a brand; Save a draft.</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/deposit-release</t>
+          <t>registrations/request</t>
         </is>
       </c>
       <c r="B129" s="3" t="inlineStr">
         <is>
-          <t>Deposit release</t>
+          <t>Registration request</t>
         </is>
       </c>
       <c r="C129" s="3" t="inlineStr">
         <is>
-          <t>Withdrawal</t>
+          <t>registrations</t>
         </is>
       </c>
       <c r="D129" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E129" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F129" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G129" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: See the request; Upload the trade licence; See the fee and submit; Follow the request until Programme review; Recommend or return; Approve, return or reject; See why it was returned and resubmit.</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/dues-verification</t>
+          <t>registrations/requests</t>
         </is>
       </c>
       <c r="B130" s="3" t="inlineStr">
         <is>
-          <t>Dues verification</t>
+          <t>Registration requests</t>
         </is>
       </c>
       <c r="C130" s="3" t="inlineStr">
         <is>
-          <t>Withdrawal</t>
+          <t>registrations</t>
         </is>
       </c>
       <c r="D130" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance</t>
+          <t>manufacturer, agency</t>
         </is>
       </c>
       <c r="E130" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F130" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G130" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: List your registration requests; Open a request; Start a new request.</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/model-withdrawal</t>
+          <t>registrations/reviews</t>
         </is>
       </c>
       <c r="B131" s="3" t="inlineStr">
         <is>
-          <t>Model withdrawal</t>
+          <t>Registration reviews</t>
         </is>
       </c>
       <c r="C131" s="3" t="inlineStr">
         <is>
-          <t>Withdrawal</t>
+          <t>registrations</t>
         </is>
       </c>
       <c r="D131" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance</t>
+          <t>programme, director</t>
         </is>
       </c>
       <c r="E131" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F131" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G131" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: List requests waiting for you; Recommend or return; Approve, return or reject; Read the trail.</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/revocation-initiation</t>
+          <t>withdrawal/brand-withdrawal</t>
         </is>
       </c>
       <c r="B132" s="3" t="inlineStr">
         <is>
-          <t>Revocation initiation</t>
+          <t>Brand withdrawal</t>
         </is>
       </c>
       <c r="C132" s="3" t="inlineStr">
@@ -5300,7 +5300,7 @@
       </c>
       <c r="F132" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G132" s="3" t="inlineStr">
@@ -5312,12 +5312,12 @@
     <row r="133">
       <c r="A133" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/withdrawal-approval</t>
+          <t>withdrawal/deposit-release</t>
         </is>
       </c>
       <c r="B133" s="3" t="inlineStr">
         <is>
-          <t>Withdrawal approval</t>
+          <t>Deposit release</t>
         </is>
       </c>
       <c r="C133" s="3" t="inlineStr">
@@ -5349,12 +5349,12 @@
     <row r="134">
       <c r="A134" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/withdrawal-letter</t>
+          <t>withdrawal/dues-verification</t>
         </is>
       </c>
       <c r="B134" s="3" t="inlineStr">
         <is>
-          <t>Withdrawal letter</t>
+          <t>Dues verification</t>
         </is>
       </c>
       <c r="C134" s="3" t="inlineStr">
@@ -5386,12 +5386,12 @@
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/withdrawal-scrutiny</t>
+          <t>withdrawal/model-withdrawal</t>
         </is>
       </c>
       <c r="B135" s="3" t="inlineStr">
         <is>
-          <t>Withdrawal scrutiny</t>
+          <t>Model withdrawal</t>
         </is>
       </c>
       <c r="C135" s="3" t="inlineStr">
@@ -5423,27 +5423,27 @@
     <row r="136">
       <c r="A136" s="3" t="inlineStr">
         <is>
-          <t>workflow/application-review</t>
+          <t>withdrawal/revocation-initiation</t>
         </is>
       </c>
       <c r="B136" s="3" t="inlineStr">
         <is>
-          <t>Application review</t>
+          <t>Revocation initiation</t>
         </is>
       </c>
       <c r="C136" s="3" t="inlineStr">
         <is>
-          <t>Workflow</t>
+          <t>Withdrawal</t>
         </is>
       </c>
       <c r="D136" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance</t>
         </is>
       </c>
       <c r="E136" s="3" t="inlineStr">
         <is>
-          <t>Live – BEE service</t>
+          <t>Prototype (preview/sample data)</t>
         </is>
       </c>
       <c r="F136" s="3" t="inlineStr">
@@ -5453,29 +5453,29 @@
       </c>
       <c r="G136" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu by role or permission. Capabilities today: List the applications in progress; Link to your next action; Link to the history.</t>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
         <is>
-          <t>workflow/approval-note</t>
+          <t>withdrawal/withdrawal-approval</t>
         </is>
       </c>
       <c r="B137" s="3" t="inlineStr">
         <is>
-          <t>Approval note</t>
+          <t>Withdrawal approval</t>
         </is>
       </c>
       <c r="C137" s="3" t="inlineStr">
         <is>
-          <t>Workflow</t>
+          <t>Withdrawal</t>
         </is>
       </c>
       <c r="D137" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance</t>
         </is>
       </c>
       <c r="E137" s="3" t="inlineStr">
@@ -5497,22 +5497,22 @@
     <row r="138">
       <c r="A138" s="3" t="inlineStr">
         <is>
-          <t>workflow/checklist</t>
+          <t>withdrawal/withdrawal-letter</t>
         </is>
       </c>
       <c r="B138" s="3" t="inlineStr">
         <is>
-          <t>Checklist</t>
+          <t>Withdrawal letter</t>
         </is>
       </c>
       <c r="C138" s="3" t="inlineStr">
         <is>
-          <t>Workflow</t>
+          <t>Withdrawal</t>
         </is>
       </c>
       <c r="D138" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance</t>
         </is>
       </c>
       <c r="E138" s="3" t="inlineStr">
@@ -5534,22 +5534,22 @@
     <row r="139">
       <c r="A139" s="3" t="inlineStr">
         <is>
-          <t>workflow/clarification-and-return</t>
+          <t>withdrawal/withdrawal-scrutiny</t>
         </is>
       </c>
       <c r="B139" s="3" t="inlineStr">
         <is>
-          <t>Clarification and return</t>
+          <t>Withdrawal scrutiny</t>
         </is>
       </c>
       <c r="C139" s="3" t="inlineStr">
         <is>
-          <t>Workflow</t>
+          <t>Withdrawal</t>
         </is>
       </c>
       <c r="D139" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance</t>
         </is>
       </c>
       <c r="E139" s="3" t="inlineStr">
@@ -5571,12 +5571,12 @@
     <row r="140">
       <c r="A140" s="3" t="inlineStr">
         <is>
-          <t>workflow/delegation-and-reassignment</t>
+          <t>workflow/application-review</t>
         </is>
       </c>
       <c r="B140" s="3" t="inlineStr">
         <is>
-          <t>Delegation and reassignment</t>
+          <t>Application review</t>
         </is>
       </c>
       <c r="C140" s="3" t="inlineStr">
@@ -5591,7 +5591,7 @@
       </c>
       <c r="E140" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F140" s="3" t="inlineStr">
@@ -5601,19 +5601,19 @@
       </c>
       <c r="G140" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t xml:space="preserve"> Spring menu by role or permission. Capabilities today: List the applications in progress; Link to your next action; Link to the history.</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="3" t="inlineStr">
         <is>
-          <t>workflow/escalation-dashboard</t>
+          <t>workflow/approval-note</t>
         </is>
       </c>
       <c r="B141" s="3" t="inlineStr">
         <is>
-          <t>Escalation dashboard</t>
+          <t>Approval note</t>
         </is>
       </c>
       <c r="C141" s="3" t="inlineStr">
@@ -5628,66 +5628,66 @@
       </c>
       <c r="E141" s="3" t="inlineStr">
         <is>
-          <t>Live – BEE service</t>
+          <t>Prototype (preview/sample data)</t>
         </is>
       </c>
       <c r="F141" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G141" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu by role or permission. Capabilities today: Count the applications waiting at each stage (no time limits are set yet).</t>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="3" t="inlineStr">
         <is>
-          <t>workflow/my-approvals</t>
+          <t>workflow/checklist</t>
         </is>
       </c>
       <c r="B142" s="3" t="inlineStr">
         <is>
-          <t>My approvals</t>
+          <t>Checklist</t>
         </is>
       </c>
       <c r="C142" s="3" t="inlineStr">
         <is>
-          <t>workflow</t>
+          <t>Workflow</t>
         </is>
       </c>
       <c r="D142" s="3" t="inlineStr">
         <is>
-          <t>director, secretary</t>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
         </is>
       </c>
       <c r="E142" s="3" t="inlineStr">
         <is>
-          <t>Live – BEE service</t>
+          <t>Prototype (preview/sample data)</t>
         </is>
       </c>
       <c r="F142" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G142" s="3" t="inlineStr">
         <is>
-          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: List the applications waiting for your decision; Open the approval screen.</t>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="3" t="inlineStr">
         <is>
-          <t>workflow/personal-inbox</t>
+          <t>workflow/clarification-and-return</t>
         </is>
       </c>
       <c r="B143" s="3" t="inlineStr">
         <is>
-          <t>Personal inbox</t>
+          <t>Clarification and return</t>
         </is>
       </c>
       <c r="C143" s="3" t="inlineStr">
@@ -5702,29 +5702,29 @@
       </c>
       <c r="E143" s="3" t="inlineStr">
         <is>
-          <t>Live – BEE service</t>
+          <t>Prototype (preview/sample data)</t>
         </is>
       </c>
       <c r="F143" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G143" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu roles include: manufacturer, agency, finance, iame, reviewer, programme, director, secretary. Capabilities today: List the applications waiting for you; Open the screen where each is done.</t>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="3" t="inlineStr">
         <is>
-          <t>workflow/team-queue</t>
+          <t>workflow/delegation-and-reassignment</t>
         </is>
       </c>
       <c r="B144" s="3" t="inlineStr">
         <is>
-          <t>Team queue</t>
+          <t>Delegation and reassignment</t>
         </is>
       </c>
       <c r="C144" s="3" t="inlineStr">
@@ -5756,35 +5756,183 @@
     <row r="145">
       <c r="A145" s="3" t="inlineStr">
         <is>
+          <t>workflow/escalation-dashboard</t>
+        </is>
+      </c>
+      <c r="B145" s="3" t="inlineStr">
+        <is>
+          <t>Escalation dashboard</t>
+        </is>
+      </c>
+      <c r="C145" s="3" t="inlineStr">
+        <is>
+          <t>Workflow</t>
+        </is>
+      </c>
+      <c r="D145" s="3" t="inlineStr">
+        <is>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
+        </is>
+      </c>
+      <c r="E145" s="3" t="inlineStr">
+        <is>
+          <t>Live – BEE service</t>
+        </is>
+      </c>
+      <c r="F145" s="3" t="inlineStr">
+        <is>
+          <t>keep</t>
+        </is>
+      </c>
+      <c r="G145" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Spring menu by role or permission. Capabilities today: Count the applications waiting at each stage (no time limits are set yet).</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="3" t="inlineStr">
+        <is>
+          <t>workflow/my-approvals</t>
+        </is>
+      </c>
+      <c r="B146" s="3" t="inlineStr">
+        <is>
+          <t>My approvals</t>
+        </is>
+      </c>
+      <c r="C146" s="3" t="inlineStr">
+        <is>
+          <t>workflow</t>
+        </is>
+      </c>
+      <c r="D146" s="3" t="inlineStr">
+        <is>
+          <t>director, secretary</t>
+        </is>
+      </c>
+      <c r="E146" s="3" t="inlineStr">
+        <is>
+          <t>Live – BEE service</t>
+        </is>
+      </c>
+      <c r="F146" s="3" t="inlineStr">
+        <is>
+          <t>keep</t>
+        </is>
+      </c>
+      <c r="G146" s="3" t="inlineStr">
+        <is>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: List the applications waiting for your decision; Open the approval screen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="3" t="inlineStr">
+        <is>
+          <t>workflow/personal-inbox</t>
+        </is>
+      </c>
+      <c r="B147" s="3" t="inlineStr">
+        <is>
+          <t>Personal inbox</t>
+        </is>
+      </c>
+      <c r="C147" s="3" t="inlineStr">
+        <is>
+          <t>Workflow</t>
+        </is>
+      </c>
+      <c r="D147" s="3" t="inlineStr">
+        <is>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
+        </is>
+      </c>
+      <c r="E147" s="3" t="inlineStr">
+        <is>
+          <t>Live – BEE service</t>
+        </is>
+      </c>
+      <c r="F147" s="3" t="inlineStr">
+        <is>
+          <t>keep</t>
+        </is>
+      </c>
+      <c r="G147" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> Spring menu roles include: manufacturer, agency, finance, iame, reviewer, programme, director, secretary. Capabilities today: List the applications waiting for you; Open the screen where each is done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="3" t="inlineStr">
+        <is>
+          <t>workflow/team-queue</t>
+        </is>
+      </c>
+      <c r="B148" s="3" t="inlineStr">
+        <is>
+          <t>Team queue</t>
+        </is>
+      </c>
+      <c r="C148" s="3" t="inlineStr">
+        <is>
+          <t>Workflow</t>
+        </is>
+      </c>
+      <c r="D148" s="3" t="inlineStr">
+        <is>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
+        </is>
+      </c>
+      <c r="E148" s="3" t="inlineStr">
+        <is>
+          <t>Prototype (preview/sample data)</t>
+        </is>
+      </c>
+      <c r="F148" s="3" t="inlineStr">
+        <is>
+          <t>merge</t>
+        </is>
+      </c>
+      <c r="G148" s="3" t="inlineStr">
+        <is>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="3" t="inlineStr">
+        <is>
           <t>workflow/workflow-history</t>
         </is>
       </c>
-      <c r="B145" s="3" t="inlineStr">
+      <c r="B149" s="3" t="inlineStr">
         <is>
           <t>Workflow history</t>
         </is>
       </c>
-      <c r="C145" s="3" t="inlineStr">
+      <c r="C149" s="3" t="inlineStr">
         <is>
           <t>Workflow</t>
         </is>
       </c>
-      <c r="D145" s="3" t="inlineStr">
+      <c r="D149" s="3" t="inlineStr">
         <is>
           <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
         </is>
       </c>
-      <c r="E145" s="3" t="inlineStr">
+      <c r="E149" s="3" t="inlineStr">
         <is>
           <t>Live – BEE service</t>
         </is>
       </c>
-      <c r="F145" s="3" t="inlineStr">
-        <is>
-          <t>merge</t>
-        </is>
-      </c>
-      <c r="G145" s="3" t="inlineStr">
+      <c r="F149" s="3" t="inlineStr">
+        <is>
+          <t>merge</t>
+        </is>
+      </c>
+      <c r="G149" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve"> Spring menu by role or permission. Capabilities today: Choose an application; Read its steps as you are allowed to see them.</t>
         </is>
@@ -5804,7 +5952,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6144,42 +6292,42 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Work package</t>
+          <t>Cursor brief</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>WP02</t>
+          <t>BRIEF-13</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Identity, session, MFA, model-application policy</t>
+          <t>Registration applicant screens (list, form, request, licence, fee)</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Work package</t>
+          <t>Cursor brief</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>WP03</t>
+          <t>BRIEF-14</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>OpenAPI contract, BFF, contract tests</t>
+          <t>Registration review screens and applicant's returned path</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
@@ -6199,12 +6347,12 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>WP04</t>
+          <t>WP02</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Masters and brand authorisation</t>
+          <t>Identity, session, MFA, model-application policy</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -6213,7 +6361,7 @@
         </is>
       </c>
       <c r="E16" s="3" t="n">
-        <v>60</v>
+        <v>75</v>
       </c>
     </row>
     <row r="17">
@@ -6224,12 +6372,12 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>WP05.1a</t>
+          <t>WP03</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Read-only model applications UI</t>
+          <t>OpenAPI contract, BFF, contract tests</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
@@ -6249,21 +6397,21 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>WP05.1b</t>
+          <t>WP04</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Draft create/edit</t>
+          <t>Masters and brand authorisation</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="E18" s="3" t="n">
-        <v>100</v>
+        <v>80</v>
       </c>
     </row>
     <row r="19">
@@ -6274,12 +6422,12 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>WP05.1c</t>
+          <t>WP04.2b-1</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Draft submission</t>
+          <t>Registration: file, trade-licence PDF, fee, Finance confirmation</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -6299,12 +6447,12 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>WP05.1d</t>
+          <t>WP04.2b-2</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Submit-time evidence gates</t>
+          <t>Registration: recommend, approve, return, reject, resubmit; register entry</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -6324,21 +6472,21 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>WP06.1a</t>
+          <t>WP04.2b-2b</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Document intake and storage</t>
+          <t>Revocation and closure of a brand or authorisation by a second person</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E21" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -6349,17 +6497,17 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>WP06.2</t>
+          <t>WP04.2b-3</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Blob retention, orphans, limits (BL-001–003)</t>
+          <t>Model submit uses the registered brand (brand id)</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="E22" s="3" t="n">
@@ -6374,12 +6522,12 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>WP07.1a</t>
+          <t>WP05.1a</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Finance fee confirmation</t>
+          <t>Read-only model applications UI</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -6399,12 +6547,12 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>WP07.1b–f</t>
+          <t>WP05.1b</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>IAME, Reviewer, Rating, Director, Secretary stages</t>
+          <t>Draft create/edit</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -6424,12 +6572,12 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>WP07.1g–h</t>
+          <t>WP05.1c</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Return, resubmit, rejection</t>
+          <t>Draft submission</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -6449,12 +6597,12 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>WP07.1i–k</t>
+          <t>WP05.1d</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>History, inbox, workflow views</t>
+          <t>Submit-time evidence gates</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -6474,12 +6622,12 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>WP08.1a</t>
+          <t>WP06.1a</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Fee rule administration</t>
+          <t>Document intake and storage</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -6499,21 +6647,21 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>WP08.1b</t>
+          <t>WP06.2</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Tax line on fee rules</t>
+          <t>Blob retention, orphans, limits (BL-001–003)</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E28" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="29">
@@ -6524,12 +6672,12 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>WP08.1c</t>
+          <t>WP07.1a</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Rating schemes administration</t>
+          <t>Finance fee confirmation</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -6549,12 +6697,12 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>WP08.1d</t>
+          <t>WP07.1b–f</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Permission-based admin menu</t>
+          <t>IAME, Reviewer, Rating, Director, Secretary stages</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -6574,12 +6722,12 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>WP08.1e</t>
+          <t>WP07.1g–h</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Fee confirmation correction proposals</t>
+          <t>Return, resubmit, rejection</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -6599,12 +6747,12 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>WP08.1f</t>
+          <t>WP07.1i–k</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Fee reversal</t>
+          <t>History, inbox, workflow views</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -6624,12 +6772,12 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>WP08.1g</t>
+          <t>WP08.1a</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Born-pending and notification proof</t>
+          <t>Fee rule administration</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -6649,12 +6797,12 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>WP08.1h</t>
+          <t>WP08.1b</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Business settings (propose/approve numbers)</t>
+          <t>Tax line on fee rules</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -6674,12 +6822,12 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>WP09.1a</t>
+          <t>WP08.1c</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Certificate record</t>
+          <t>Rating schemes administration</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -6699,12 +6847,12 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>WP09.1b</t>
+          <t>WP08.1d</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Printable certificate and label</t>
+          <t>Permission-based admin menu</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -6724,12 +6872,12 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>WP09.1c</t>
+          <t>WP08.1e</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Public verification page</t>
+          <t>Fee confirmation correction proposals</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -6749,12 +6897,12 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>WP09.1d</t>
+          <t>WP08.1f</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Verification rate limit</t>
+          <t>Fee reversal</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -6774,12 +6922,12 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>WP10.1a</t>
+          <t>WP08.1g</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>In-portal notifications (API)</t>
+          <t>Born-pending and notification proof</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -6799,12 +6947,12 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>WP10.1b</t>
+          <t>WP08.1h</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Notification bell and page</t>
+          <t>Business settings (propose/approve numbers)</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -6824,37 +6972,37 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>WP11</t>
+          <t>WP09.1a</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>AI demonstrations (local)</t>
+          <t>Certificate record</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E41" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>Platform</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>WP01</t>
+          <t>WP09.1b</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Documentation and design evidence</t>
+          <t>Printable certificate and label</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -6869,75 +7017,225 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>Backlog theme</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>BL-024/025</t>
+          <t>WP09.1c</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Feature template and OpenAPI split</t>
+          <t>Public verification page</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E43" s="3" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>Backlog theme</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>BL-040–042</t>
+          <t>WP09.1d</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+          <t>Verification rate limit</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E44" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
+          <t>Work package</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>WP10.1a</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>In-portal notifications (API)</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>Work package</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>WP10.1b</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>Notification bell and page</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>Work package</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>WP11</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>AI demonstrations (local)</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>WP01</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>Documentation and design evidence</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>Backlog theme</t>
+        </is>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>BL-024/025</t>
+        </is>
+      </c>
+      <c r="C49" s="3" t="inlineStr">
+        <is>
+          <t>Feature template and OpenAPI split</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>Backlog theme</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>BL-040–042</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
           <t>Owner decision</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
+      <c r="B51" s="3" t="inlineStr">
         <is>
           <t>D10</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr">
+      <c r="C51" s="3" t="inlineStr">
         <is>
           <t>Provisional local rules for notifications (portal only)</t>
         </is>
       </c>
-      <c r="D45" s="3" t="inlineStr">
+      <c r="D51" s="3" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
-      <c r="E45" s="3" t="n">
+      <c r="E51" s="3" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
WP04.2b-3: live proof that the register feeds the model flow; workbook; BL-181
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/BEE-portal-status.xlsx
+++ b/docs/tracking/BEE-portal-status.xlsx
@@ -6411,7 +6411,7 @@
         </is>
       </c>
       <c r="E18" s="3" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
     </row>
     <row r="19">
@@ -6502,16 +6502,16 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Model submit uses the registered brand (brand id)</t>
+          <t>Model flow uses the registered brand (brand id); live proof of the chain</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E22" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="23">

</xml_diff>

<commit_message>
WP04.2b-3: the register feeds the model flow (live proof) (#49)
* WP04.2b-3: live proof that the register feeds the model flow; workbook; BL-181

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

* WP04.2b-3: correct the doc wording on edit (review nit)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

---------

Co-authored-by: Sameer Khanna <sameerkhanna@Sameers-MacBook-Pro.local>
Co-authored-by: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/BEE-portal-status.xlsx
+++ b/docs/tracking/BEE-portal-status.xlsx
@@ -6411,7 +6411,7 @@
         </is>
       </c>
       <c r="E18" s="3" t="n">
-        <v>80</v>
+        <v>90</v>
       </c>
     </row>
     <row r="19">
@@ -6502,16 +6502,16 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Model submit uses the registered brand (brand id)</t>
+          <t>Model flow uses the registered brand (brand id); live proof of the chain</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E22" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="23">

</xml_diff>

<commit_message>
Review fixes for Brief 15: re-read after a stale refusal, no panel carry-over between rows, note only with a rejection, no dead reload button, table captions; BL-185 done, BL-187; workbook
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/BEE-portal-status.xlsx
+++ b/docs/tracking/BEE-portal-status.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G149"/>
+  <dimension ref="A1:G150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -5164,12 +5164,12 @@
     <row r="129">
       <c r="A129" s="3" t="inlineStr">
         <is>
-          <t>registrations/request</t>
+          <t>registrations/register</t>
         </is>
       </c>
       <c r="B129" s="3" t="inlineStr">
         <is>
-          <t>Registration request</t>
+          <t>Register</t>
         </is>
       </c>
       <c r="C129" s="3" t="inlineStr">
@@ -5179,7 +5179,7 @@
       </c>
       <c r="D129" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>programme, director</t>
         </is>
       </c>
       <c r="E129" s="3" t="inlineStr">
@@ -5194,19 +5194,19 @@
       </c>
       <c r="G129" s="3" t="inlineStr">
         <is>
-          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: See the request; Upload the trade licence; See the fee and submit; Follow the request until Programme review; Recommend or return; Approve, return or reject; See why it was returned and resubmit.</t>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: See registered brands and authorisations; Propose a closure or revocation; Approve, reject or withdraw a proposal; Read the history.</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="3" t="inlineStr">
         <is>
-          <t>registrations/requests</t>
+          <t>registrations/request</t>
         </is>
       </c>
       <c r="B130" s="3" t="inlineStr">
         <is>
-          <t>Registration requests</t>
+          <t>Registration request</t>
         </is>
       </c>
       <c r="C130" s="3" t="inlineStr">
@@ -5216,7 +5216,7 @@
       </c>
       <c r="D130" s="3" t="inlineStr">
         <is>
-          <t>manufacturer, agency</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E130" s="3" t="inlineStr">
@@ -5231,19 +5231,19 @@
       </c>
       <c r="G130" s="3" t="inlineStr">
         <is>
-          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: List your registration requests; Open a request; Start a new request.</t>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: See the request; Upload the trade licence; See the fee and submit; Follow the request until Programme review; Recommend or return; Approve, return or reject; See why it was returned and resubmit.</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="3" t="inlineStr">
         <is>
-          <t>registrations/reviews</t>
+          <t>registrations/requests</t>
         </is>
       </c>
       <c r="B131" s="3" t="inlineStr">
         <is>
-          <t>Registration reviews</t>
+          <t>Registration requests</t>
         </is>
       </c>
       <c r="C131" s="3" t="inlineStr">
@@ -5253,7 +5253,7 @@
       </c>
       <c r="D131" s="3" t="inlineStr">
         <is>
-          <t>programme, director</t>
+          <t>manufacturer, agency</t>
         </is>
       </c>
       <c r="E131" s="3" t="inlineStr">
@@ -5268,34 +5268,34 @@
       </c>
       <c r="G131" s="3" t="inlineStr">
         <is>
-          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: List requests waiting for you; Recommend or return; Approve, return or reject; Read the trail.</t>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: List your registration requests; Open a request; Start a new request.</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/brand-withdrawal</t>
+          <t>registrations/reviews</t>
         </is>
       </c>
       <c r="B132" s="3" t="inlineStr">
         <is>
-          <t>Brand withdrawal</t>
+          <t>Registration reviews</t>
         </is>
       </c>
       <c r="C132" s="3" t="inlineStr">
         <is>
-          <t>Withdrawal</t>
+          <t>registrations</t>
         </is>
       </c>
       <c r="D132" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance</t>
+          <t>programme, director</t>
         </is>
       </c>
       <c r="E132" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F132" s="3" t="inlineStr">
@@ -5305,19 +5305,19 @@
       </c>
       <c r="G132" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: List requests waiting for you; Recommend or return; Approve, return or reject; Read the trail.</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/deposit-release</t>
+          <t>withdrawal/brand-withdrawal</t>
         </is>
       </c>
       <c r="B133" s="3" t="inlineStr">
         <is>
-          <t>Deposit release</t>
+          <t>Brand withdrawal</t>
         </is>
       </c>
       <c r="C133" s="3" t="inlineStr">
@@ -5337,7 +5337,7 @@
       </c>
       <c r="F133" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G133" s="3" t="inlineStr">
@@ -5349,12 +5349,12 @@
     <row r="134">
       <c r="A134" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/dues-verification</t>
+          <t>withdrawal/deposit-release</t>
         </is>
       </c>
       <c r="B134" s="3" t="inlineStr">
         <is>
-          <t>Dues verification</t>
+          <t>Deposit release</t>
         </is>
       </c>
       <c r="C134" s="3" t="inlineStr">
@@ -5386,12 +5386,12 @@
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/model-withdrawal</t>
+          <t>withdrawal/dues-verification</t>
         </is>
       </c>
       <c r="B135" s="3" t="inlineStr">
         <is>
-          <t>Model withdrawal</t>
+          <t>Dues verification</t>
         </is>
       </c>
       <c r="C135" s="3" t="inlineStr">
@@ -5423,12 +5423,12 @@
     <row r="136">
       <c r="A136" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/revocation-initiation</t>
+          <t>withdrawal/model-withdrawal</t>
         </is>
       </c>
       <c r="B136" s="3" t="inlineStr">
         <is>
-          <t>Revocation initiation</t>
+          <t>Model withdrawal</t>
         </is>
       </c>
       <c r="C136" s="3" t="inlineStr">
@@ -5460,12 +5460,12 @@
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/withdrawal-approval</t>
+          <t>withdrawal/revocation-initiation</t>
         </is>
       </c>
       <c r="B137" s="3" t="inlineStr">
         <is>
-          <t>Withdrawal approval</t>
+          <t>Revocation initiation</t>
         </is>
       </c>
       <c r="C137" s="3" t="inlineStr">
@@ -5497,12 +5497,12 @@
     <row r="138">
       <c r="A138" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/withdrawal-letter</t>
+          <t>withdrawal/withdrawal-approval</t>
         </is>
       </c>
       <c r="B138" s="3" t="inlineStr">
         <is>
-          <t>Withdrawal letter</t>
+          <t>Withdrawal approval</t>
         </is>
       </c>
       <c r="C138" s="3" t="inlineStr">
@@ -5534,12 +5534,12 @@
     <row r="139">
       <c r="A139" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/withdrawal-scrutiny</t>
+          <t>withdrawal/withdrawal-letter</t>
         </is>
       </c>
       <c r="B139" s="3" t="inlineStr">
         <is>
-          <t>Withdrawal scrutiny</t>
+          <t>Withdrawal letter</t>
         </is>
       </c>
       <c r="C139" s="3" t="inlineStr">
@@ -5571,27 +5571,27 @@
     <row r="140">
       <c r="A140" s="3" t="inlineStr">
         <is>
-          <t>workflow/application-review</t>
+          <t>withdrawal/withdrawal-scrutiny</t>
         </is>
       </c>
       <c r="B140" s="3" t="inlineStr">
         <is>
-          <t>Application review</t>
+          <t>Withdrawal scrutiny</t>
         </is>
       </c>
       <c r="C140" s="3" t="inlineStr">
         <is>
-          <t>Workflow</t>
+          <t>Withdrawal</t>
         </is>
       </c>
       <c r="D140" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance</t>
         </is>
       </c>
       <c r="E140" s="3" t="inlineStr">
         <is>
-          <t>Live – BEE service</t>
+          <t>Prototype (preview/sample data)</t>
         </is>
       </c>
       <c r="F140" s="3" t="inlineStr">
@@ -5601,19 +5601,19 @@
       </c>
       <c r="G140" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu by role or permission. Capabilities today: List the applications in progress; Link to your next action; Link to the history.</t>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="3" t="inlineStr">
         <is>
-          <t>workflow/approval-note</t>
+          <t>workflow/application-review</t>
         </is>
       </c>
       <c r="B141" s="3" t="inlineStr">
         <is>
-          <t>Approval note</t>
+          <t>Application review</t>
         </is>
       </c>
       <c r="C141" s="3" t="inlineStr">
@@ -5628,7 +5628,7 @@
       </c>
       <c r="E141" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F141" s="3" t="inlineStr">
@@ -5638,19 +5638,19 @@
       </c>
       <c r="G141" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t xml:space="preserve"> Spring menu by role or permission. Capabilities today: List the applications in progress; Link to your next action; Link to the history.</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="3" t="inlineStr">
         <is>
-          <t>workflow/checklist</t>
+          <t>workflow/approval-note</t>
         </is>
       </c>
       <c r="B142" s="3" t="inlineStr">
         <is>
-          <t>Checklist</t>
+          <t>Approval note</t>
         </is>
       </c>
       <c r="C142" s="3" t="inlineStr">
@@ -5682,12 +5682,12 @@
     <row r="143">
       <c r="A143" s="3" t="inlineStr">
         <is>
-          <t>workflow/clarification-and-return</t>
+          <t>workflow/checklist</t>
         </is>
       </c>
       <c r="B143" s="3" t="inlineStr">
         <is>
-          <t>Clarification and return</t>
+          <t>Checklist</t>
         </is>
       </c>
       <c r="C143" s="3" t="inlineStr">
@@ -5719,12 +5719,12 @@
     <row r="144">
       <c r="A144" s="3" t="inlineStr">
         <is>
-          <t>workflow/delegation-and-reassignment</t>
+          <t>workflow/clarification-and-return</t>
         </is>
       </c>
       <c r="B144" s="3" t="inlineStr">
         <is>
-          <t>Delegation and reassignment</t>
+          <t>Clarification and return</t>
         </is>
       </c>
       <c r="C144" s="3" t="inlineStr">
@@ -5756,12 +5756,12 @@
     <row r="145">
       <c r="A145" s="3" t="inlineStr">
         <is>
-          <t>workflow/escalation-dashboard</t>
+          <t>workflow/delegation-and-reassignment</t>
         </is>
       </c>
       <c r="B145" s="3" t="inlineStr">
         <is>
-          <t>Escalation dashboard</t>
+          <t>Delegation and reassignment</t>
         </is>
       </c>
       <c r="C145" s="3" t="inlineStr">
@@ -5776,39 +5776,39 @@
       </c>
       <c r="E145" s="3" t="inlineStr">
         <is>
-          <t>Live – BEE service</t>
+          <t>Prototype (preview/sample data)</t>
         </is>
       </c>
       <c r="F145" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G145" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu by role or permission. Capabilities today: Count the applications waiting at each stage (no time limits are set yet).</t>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="3" t="inlineStr">
         <is>
-          <t>workflow/my-approvals</t>
+          <t>workflow/escalation-dashboard</t>
         </is>
       </c>
       <c r="B146" s="3" t="inlineStr">
         <is>
-          <t>My approvals</t>
+          <t>Escalation dashboard</t>
         </is>
       </c>
       <c r="C146" s="3" t="inlineStr">
         <is>
-          <t>workflow</t>
+          <t>Workflow</t>
         </is>
       </c>
       <c r="D146" s="3" t="inlineStr">
         <is>
-          <t>director, secretary</t>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
         </is>
       </c>
       <c r="E146" s="3" t="inlineStr">
@@ -5823,29 +5823,29 @@
       </c>
       <c r="G146" s="3" t="inlineStr">
         <is>
-          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: List the applications waiting for your decision; Open the approval screen.</t>
+          <t xml:space="preserve"> Spring menu by role or permission. Capabilities today: Count the applications waiting at each stage (no time limits are set yet).</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="3" t="inlineStr">
         <is>
-          <t>workflow/personal-inbox</t>
+          <t>workflow/my-approvals</t>
         </is>
       </c>
       <c r="B147" s="3" t="inlineStr">
         <is>
-          <t>Personal inbox</t>
+          <t>My approvals</t>
         </is>
       </c>
       <c r="C147" s="3" t="inlineStr">
         <is>
-          <t>Workflow</t>
+          <t>workflow</t>
         </is>
       </c>
       <c r="D147" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
+          <t>director, secretary</t>
         </is>
       </c>
       <c r="E147" s="3" t="inlineStr">
@@ -5860,19 +5860,19 @@
       </c>
       <c r="G147" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu roles include: manufacturer, agency, finance, iame, reviewer, programme, director, secretary. Capabilities today: List the applications waiting for you; Open the screen where each is done.</t>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: List the applications waiting for your decision; Open the approval screen.</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="3" t="inlineStr">
         <is>
-          <t>workflow/team-queue</t>
+          <t>workflow/personal-inbox</t>
         </is>
       </c>
       <c r="B148" s="3" t="inlineStr">
         <is>
-          <t>Team queue</t>
+          <t>Personal inbox</t>
         </is>
       </c>
       <c r="C148" s="3" t="inlineStr">
@@ -5887,52 +5887,89 @@
       </c>
       <c r="E148" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F148" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G148" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t xml:space="preserve"> Spring menu roles include: manufacturer, agency, finance, iame, reviewer, programme, director, secretary. Capabilities today: List the applications waiting for you; Open the screen where each is done.</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="3" t="inlineStr">
         <is>
+          <t>workflow/team-queue</t>
+        </is>
+      </c>
+      <c r="B149" s="3" t="inlineStr">
+        <is>
+          <t>Team queue</t>
+        </is>
+      </c>
+      <c r="C149" s="3" t="inlineStr">
+        <is>
+          <t>Workflow</t>
+        </is>
+      </c>
+      <c r="D149" s="3" t="inlineStr">
+        <is>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
+        </is>
+      </c>
+      <c r="E149" s="3" t="inlineStr">
+        <is>
+          <t>Prototype (preview/sample data)</t>
+        </is>
+      </c>
+      <c r="F149" s="3" t="inlineStr">
+        <is>
+          <t>merge</t>
+        </is>
+      </c>
+      <c r="G149" s="3" t="inlineStr">
+        <is>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="3" t="inlineStr">
+        <is>
           <t>workflow/workflow-history</t>
         </is>
       </c>
-      <c r="B149" s="3" t="inlineStr">
+      <c r="B150" s="3" t="inlineStr">
         <is>
           <t>Workflow history</t>
         </is>
       </c>
-      <c r="C149" s="3" t="inlineStr">
+      <c r="C150" s="3" t="inlineStr">
         <is>
           <t>Workflow</t>
         </is>
       </c>
-      <c r="D149" s="3" t="inlineStr">
+      <c r="D150" s="3" t="inlineStr">
         <is>
           <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
         </is>
       </c>
-      <c r="E149" s="3" t="inlineStr">
+      <c r="E150" s="3" t="inlineStr">
         <is>
           <t>Live – BEE service</t>
         </is>
       </c>
-      <c r="F149" s="3" t="inlineStr">
-        <is>
-          <t>merge</t>
-        </is>
-      </c>
-      <c r="G149" s="3" t="inlineStr">
+      <c r="F150" s="3" t="inlineStr">
+        <is>
+          <t>merge</t>
+        </is>
+      </c>
+      <c r="G150" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve"> Spring menu by role or permission. Capabilities today: Choose an application; Read its steps as you are allowed to see them.</t>
         </is>
@@ -5952,7 +5989,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6342,26 +6379,26 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Work package</t>
+          <t>Cursor brief</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>WP02</t>
+          <t>BRIEF-15</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Identity, session, MFA, model-application policy</t>
+          <t>Register screen: propose and decide closing or revoking an entry</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
     </row>
     <row r="17">
@@ -6372,21 +6409,21 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>WP03</t>
+          <t>WP02</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>OpenAPI contract, BFF, contract tests</t>
+          <t>Identity, session, MFA, model-application policy</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
     </row>
     <row r="18">
@@ -6397,21 +6434,21 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>WP04</t>
+          <t>WP03</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Masters and brand authorisation</t>
+          <t>OpenAPI contract, BFF, contract tests</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E18" s="3" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="19">
@@ -6422,21 +6459,21 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>WP04.2b-1</t>
+          <t>WP04</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Registration: file, trade-licence PDF, fee, Finance confirmation</t>
+          <t>Masters and brand authorisation</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="E19" s="3" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
     </row>
     <row r="20">
@@ -6447,12 +6484,12 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>WP04.2b-2</t>
+          <t>WP04.2b-1</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Registration: recommend, approve, return, reject, resubmit; register entry</t>
+          <t>Registration: file, trade-licence PDF, fee, Finance confirmation</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -6472,21 +6509,21 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>WP04.2b-2b</t>
+          <t>WP04.2b-2</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Revocation and closure of a brand or authorisation by a second person</t>
+          <t>Registration: recommend, approve, return, reject, resubmit; register entry</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E21" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="22">
@@ -6497,12 +6534,12 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>WP04.2b-3</t>
+          <t>WP04.2b-2b</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Model flow uses the registered brand (brand id); live proof of the chain</t>
+          <t>Revocation and closure of a brand or authorisation by a second person</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -6522,12 +6559,12 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>WP05.1a</t>
+          <t>WP04.2b-3</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Read-only model applications UI</t>
+          <t>Model flow uses the registered brand (brand id); live proof of the chain</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -6547,12 +6584,12 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>WP05.1b</t>
+          <t>WP05.1a</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Draft create/edit</t>
+          <t>Read-only model applications UI</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -6572,12 +6609,12 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>WP05.1c</t>
+          <t>WP05.1b</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Draft submission</t>
+          <t>Draft create/edit</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -6597,12 +6634,12 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>WP05.1d</t>
+          <t>WP05.1c</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Submit-time evidence gates</t>
+          <t>Draft submission</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -6622,12 +6659,12 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>WP06.1a</t>
+          <t>WP05.1d</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Document intake and storage</t>
+          <t>Submit-time evidence gates</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -6647,21 +6684,21 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>WP06.2</t>
+          <t>WP06.1a</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Blob retention, orphans, limits (BL-001–003)</t>
+          <t>Document intake and storage</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E28" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="29">
@@ -6672,21 +6709,21 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>WP07.1a</t>
+          <t>WP06.2</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Finance fee confirmation</t>
+          <t>Blob retention, orphans, limits (BL-001–003)</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E29" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -6697,12 +6734,12 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>WP07.1b–f</t>
+          <t>WP07.1a</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>IAME, Reviewer, Rating, Director, Secretary stages</t>
+          <t>Finance fee confirmation</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -6722,12 +6759,12 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>WP07.1g–h</t>
+          <t>WP07.1b–f</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Return, resubmit, rejection</t>
+          <t>IAME, Reviewer, Rating, Director, Secretary stages</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -6747,12 +6784,12 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>WP07.1i–k</t>
+          <t>WP07.1g–h</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>History, inbox, workflow views</t>
+          <t>Return, resubmit, rejection</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -6772,12 +6809,12 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>WP08.1a</t>
+          <t>WP07.1i–k</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Fee rule administration</t>
+          <t>History, inbox, workflow views</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -6797,12 +6834,12 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>WP08.1b</t>
+          <t>WP08.1a</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Tax line on fee rules</t>
+          <t>Fee rule administration</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -6822,12 +6859,12 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>WP08.1c</t>
+          <t>WP08.1b</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Rating schemes administration</t>
+          <t>Tax line on fee rules</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -6847,12 +6884,12 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>WP08.1d</t>
+          <t>WP08.1c</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Permission-based admin menu</t>
+          <t>Rating schemes administration</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -6872,12 +6909,12 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>WP08.1e</t>
+          <t>WP08.1d</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Fee confirmation correction proposals</t>
+          <t>Permission-based admin menu</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -6897,12 +6934,12 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>WP08.1f</t>
+          <t>WP08.1e</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Fee reversal</t>
+          <t>Fee confirmation correction proposals</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -6922,12 +6959,12 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>WP08.1g</t>
+          <t>WP08.1f</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Born-pending and notification proof</t>
+          <t>Fee reversal</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -6947,12 +6984,12 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>WP08.1h</t>
+          <t>WP08.1g</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Business settings (propose/approve numbers)</t>
+          <t>Born-pending and notification proof</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -6972,12 +7009,12 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>WP09.1a</t>
+          <t>WP08.1h</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Certificate record</t>
+          <t>Business settings (propose/approve numbers)</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -6997,12 +7034,12 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>WP09.1b</t>
+          <t>WP09.1a</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Printable certificate and label</t>
+          <t>Certificate record</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -7022,12 +7059,12 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>WP09.1c</t>
+          <t>WP09.1b</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Public verification page</t>
+          <t>Printable certificate and label</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -7047,12 +7084,12 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>WP09.1d</t>
+          <t>WP09.1c</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Verification rate limit</t>
+          <t>Public verification page</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -7072,12 +7109,12 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>WP10.1a</t>
+          <t>WP09.1d</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>In-portal notifications (API)</t>
+          <t>Verification rate limit</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -7097,12 +7134,12 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>WP10.1b</t>
+          <t>WP10.1a</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Notification bell and page</t>
+          <t>In-portal notifications (API)</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -7122,71 +7159,71 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>WP11</t>
+          <t>WP10.1b</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>AI demonstrations (local)</t>
+          <t>Notification bell and page</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E47" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>Platform</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>WP01</t>
+          <t>WP11</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Documentation and design evidence</t>
+          <t>AI demonstrations (local)</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E48" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>Backlog theme</t>
+          <t>Platform</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>BL-024/025</t>
+          <t>WP01</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Feature template and OpenAPI split</t>
+          <t>Documentation and design evidence</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E49" s="3" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
     </row>
     <row r="50">
@@ -7197,45 +7234,70 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>BL-040–042</t>
+          <t>BL-024/025</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+          <t>Feature template and OpenAPI split</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="E50" s="3" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
+          <t>Backlog theme</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>BL-040–042</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
           <t>Owner decision</t>
         </is>
       </c>
-      <c r="B51" s="3" t="inlineStr">
+      <c r="B52" s="3" t="inlineStr">
         <is>
           <t>D10</t>
         </is>
       </c>
-      <c r="C51" s="3" t="inlineStr">
+      <c r="C52" s="3" t="inlineStr">
         <is>
           <t>Provisional local rules for notifications (portal only)</t>
         </is>
       </c>
-      <c r="D51" s="3" t="inlineStr">
+      <c r="D52" s="3" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
-      <c r="E51" s="3" t="n">
+      <c r="E52" s="3" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Brief 15: the register screen (propose and decide closing or revoking an entry) (#51)
* Hand over Brief 15 (register revocation screen) to Cursor

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

* Brief 15: let Programme propose a register closure and the Director decide it.

The screen offers the controls the API allows, and it shows Spring's refusal when the person may not take the step.

Co-authored-by: Cursor <cursoragent@cursor.com>

* Review fixes for Brief 15: re-read after a stale refusal, no panel carry-over between rows, note only with a rejection, no dead reload button, table captions; BL-185 done, BL-187; workbook

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

---------

Co-authored-by: Sameer Khanna <sameerkhanna@Sameers-MacBook-Pro.local>
Co-authored-by: Claude Sonnet 5.5 <noreply@anthropic.com>
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/BEE-portal-status.xlsx
+++ b/docs/tracking/BEE-portal-status.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G149"/>
+  <dimension ref="A1:G150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -5164,12 +5164,12 @@
     <row r="129">
       <c r="A129" s="3" t="inlineStr">
         <is>
-          <t>registrations/request</t>
+          <t>registrations/register</t>
         </is>
       </c>
       <c r="B129" s="3" t="inlineStr">
         <is>
-          <t>Registration request</t>
+          <t>Register</t>
         </is>
       </c>
       <c r="C129" s="3" t="inlineStr">
@@ -5179,7 +5179,7 @@
       </c>
       <c r="D129" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>programme, director</t>
         </is>
       </c>
       <c r="E129" s="3" t="inlineStr">
@@ -5194,19 +5194,19 @@
       </c>
       <c r="G129" s="3" t="inlineStr">
         <is>
-          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: See the request; Upload the trade licence; See the fee and submit; Follow the request until Programme review; Recommend or return; Approve, return or reject; See why it was returned and resubmit.</t>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: See registered brands and authorisations; Propose a closure or revocation; Approve, reject or withdraw a proposal; Read the history.</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="3" t="inlineStr">
         <is>
-          <t>registrations/requests</t>
+          <t>registrations/request</t>
         </is>
       </c>
       <c r="B130" s="3" t="inlineStr">
         <is>
-          <t>Registration requests</t>
+          <t>Registration request</t>
         </is>
       </c>
       <c r="C130" s="3" t="inlineStr">
@@ -5216,7 +5216,7 @@
       </c>
       <c r="D130" s="3" t="inlineStr">
         <is>
-          <t>manufacturer, agency</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E130" s="3" t="inlineStr">
@@ -5231,19 +5231,19 @@
       </c>
       <c r="G130" s="3" t="inlineStr">
         <is>
-          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: List your registration requests; Open a request; Start a new request.</t>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: See the request; Upload the trade licence; See the fee and submit; Follow the request until Programme review; Recommend or return; Approve, return or reject; See why it was returned and resubmit.</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="3" t="inlineStr">
         <is>
-          <t>registrations/reviews</t>
+          <t>registrations/requests</t>
         </is>
       </c>
       <c r="B131" s="3" t="inlineStr">
         <is>
-          <t>Registration reviews</t>
+          <t>Registration requests</t>
         </is>
       </c>
       <c r="C131" s="3" t="inlineStr">
@@ -5253,7 +5253,7 @@
       </c>
       <c r="D131" s="3" t="inlineStr">
         <is>
-          <t>programme, director</t>
+          <t>manufacturer, agency</t>
         </is>
       </c>
       <c r="E131" s="3" t="inlineStr">
@@ -5268,34 +5268,34 @@
       </c>
       <c r="G131" s="3" t="inlineStr">
         <is>
-          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: List requests waiting for you; Recommend or return; Approve, return or reject; Read the trail.</t>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: List your registration requests; Open a request; Start a new request.</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/brand-withdrawal</t>
+          <t>registrations/reviews</t>
         </is>
       </c>
       <c r="B132" s="3" t="inlineStr">
         <is>
-          <t>Brand withdrawal</t>
+          <t>Registration reviews</t>
         </is>
       </c>
       <c r="C132" s="3" t="inlineStr">
         <is>
-          <t>Withdrawal</t>
+          <t>registrations</t>
         </is>
       </c>
       <c r="D132" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance</t>
+          <t>programme, director</t>
         </is>
       </c>
       <c r="E132" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F132" s="3" t="inlineStr">
@@ -5305,19 +5305,19 @@
       </c>
       <c r="G132" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: List requests waiting for you; Recommend or return; Approve, return or reject; Read the trail.</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/deposit-release</t>
+          <t>withdrawal/brand-withdrawal</t>
         </is>
       </c>
       <c r="B133" s="3" t="inlineStr">
         <is>
-          <t>Deposit release</t>
+          <t>Brand withdrawal</t>
         </is>
       </c>
       <c r="C133" s="3" t="inlineStr">
@@ -5337,7 +5337,7 @@
       </c>
       <c r="F133" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G133" s="3" t="inlineStr">
@@ -5349,12 +5349,12 @@
     <row r="134">
       <c r="A134" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/dues-verification</t>
+          <t>withdrawal/deposit-release</t>
         </is>
       </c>
       <c r="B134" s="3" t="inlineStr">
         <is>
-          <t>Dues verification</t>
+          <t>Deposit release</t>
         </is>
       </c>
       <c r="C134" s="3" t="inlineStr">
@@ -5386,12 +5386,12 @@
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/model-withdrawal</t>
+          <t>withdrawal/dues-verification</t>
         </is>
       </c>
       <c r="B135" s="3" t="inlineStr">
         <is>
-          <t>Model withdrawal</t>
+          <t>Dues verification</t>
         </is>
       </c>
       <c r="C135" s="3" t="inlineStr">
@@ -5423,12 +5423,12 @@
     <row r="136">
       <c r="A136" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/revocation-initiation</t>
+          <t>withdrawal/model-withdrawal</t>
         </is>
       </c>
       <c r="B136" s="3" t="inlineStr">
         <is>
-          <t>Revocation initiation</t>
+          <t>Model withdrawal</t>
         </is>
       </c>
       <c r="C136" s="3" t="inlineStr">
@@ -5460,12 +5460,12 @@
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/withdrawal-approval</t>
+          <t>withdrawal/revocation-initiation</t>
         </is>
       </c>
       <c r="B137" s="3" t="inlineStr">
         <is>
-          <t>Withdrawal approval</t>
+          <t>Revocation initiation</t>
         </is>
       </c>
       <c r="C137" s="3" t="inlineStr">
@@ -5497,12 +5497,12 @@
     <row r="138">
       <c r="A138" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/withdrawal-letter</t>
+          <t>withdrawal/withdrawal-approval</t>
         </is>
       </c>
       <c r="B138" s="3" t="inlineStr">
         <is>
-          <t>Withdrawal letter</t>
+          <t>Withdrawal approval</t>
         </is>
       </c>
       <c r="C138" s="3" t="inlineStr">
@@ -5534,12 +5534,12 @@
     <row r="139">
       <c r="A139" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/withdrawal-scrutiny</t>
+          <t>withdrawal/withdrawal-letter</t>
         </is>
       </c>
       <c r="B139" s="3" t="inlineStr">
         <is>
-          <t>Withdrawal scrutiny</t>
+          <t>Withdrawal letter</t>
         </is>
       </c>
       <c r="C139" s="3" t="inlineStr">
@@ -5571,27 +5571,27 @@
     <row r="140">
       <c r="A140" s="3" t="inlineStr">
         <is>
-          <t>workflow/application-review</t>
+          <t>withdrawal/withdrawal-scrutiny</t>
         </is>
       </c>
       <c r="B140" s="3" t="inlineStr">
         <is>
-          <t>Application review</t>
+          <t>Withdrawal scrutiny</t>
         </is>
       </c>
       <c r="C140" s="3" t="inlineStr">
         <is>
-          <t>Workflow</t>
+          <t>Withdrawal</t>
         </is>
       </c>
       <c r="D140" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance</t>
         </is>
       </c>
       <c r="E140" s="3" t="inlineStr">
         <is>
-          <t>Live – BEE service</t>
+          <t>Prototype (preview/sample data)</t>
         </is>
       </c>
       <c r="F140" s="3" t="inlineStr">
@@ -5601,19 +5601,19 @@
       </c>
       <c r="G140" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu by role or permission. Capabilities today: List the applications in progress; Link to your next action; Link to the history.</t>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="3" t="inlineStr">
         <is>
-          <t>workflow/approval-note</t>
+          <t>workflow/application-review</t>
         </is>
       </c>
       <c r="B141" s="3" t="inlineStr">
         <is>
-          <t>Approval note</t>
+          <t>Application review</t>
         </is>
       </c>
       <c r="C141" s="3" t="inlineStr">
@@ -5628,7 +5628,7 @@
       </c>
       <c r="E141" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F141" s="3" t="inlineStr">
@@ -5638,19 +5638,19 @@
       </c>
       <c r="G141" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t xml:space="preserve"> Spring menu by role or permission. Capabilities today: List the applications in progress; Link to your next action; Link to the history.</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="3" t="inlineStr">
         <is>
-          <t>workflow/checklist</t>
+          <t>workflow/approval-note</t>
         </is>
       </c>
       <c r="B142" s="3" t="inlineStr">
         <is>
-          <t>Checklist</t>
+          <t>Approval note</t>
         </is>
       </c>
       <c r="C142" s="3" t="inlineStr">
@@ -5682,12 +5682,12 @@
     <row r="143">
       <c r="A143" s="3" t="inlineStr">
         <is>
-          <t>workflow/clarification-and-return</t>
+          <t>workflow/checklist</t>
         </is>
       </c>
       <c r="B143" s="3" t="inlineStr">
         <is>
-          <t>Clarification and return</t>
+          <t>Checklist</t>
         </is>
       </c>
       <c r="C143" s="3" t="inlineStr">
@@ -5719,12 +5719,12 @@
     <row r="144">
       <c r="A144" s="3" t="inlineStr">
         <is>
-          <t>workflow/delegation-and-reassignment</t>
+          <t>workflow/clarification-and-return</t>
         </is>
       </c>
       <c r="B144" s="3" t="inlineStr">
         <is>
-          <t>Delegation and reassignment</t>
+          <t>Clarification and return</t>
         </is>
       </c>
       <c r="C144" s="3" t="inlineStr">
@@ -5756,12 +5756,12 @@
     <row r="145">
       <c r="A145" s="3" t="inlineStr">
         <is>
-          <t>workflow/escalation-dashboard</t>
+          <t>workflow/delegation-and-reassignment</t>
         </is>
       </c>
       <c r="B145" s="3" t="inlineStr">
         <is>
-          <t>Escalation dashboard</t>
+          <t>Delegation and reassignment</t>
         </is>
       </c>
       <c r="C145" s="3" t="inlineStr">
@@ -5776,39 +5776,39 @@
       </c>
       <c r="E145" s="3" t="inlineStr">
         <is>
-          <t>Live – BEE service</t>
+          <t>Prototype (preview/sample data)</t>
         </is>
       </c>
       <c r="F145" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G145" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu by role or permission. Capabilities today: Count the applications waiting at each stage (no time limits are set yet).</t>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="3" t="inlineStr">
         <is>
-          <t>workflow/my-approvals</t>
+          <t>workflow/escalation-dashboard</t>
         </is>
       </c>
       <c r="B146" s="3" t="inlineStr">
         <is>
-          <t>My approvals</t>
+          <t>Escalation dashboard</t>
         </is>
       </c>
       <c r="C146" s="3" t="inlineStr">
         <is>
-          <t>workflow</t>
+          <t>Workflow</t>
         </is>
       </c>
       <c r="D146" s="3" t="inlineStr">
         <is>
-          <t>director, secretary</t>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
         </is>
       </c>
       <c r="E146" s="3" t="inlineStr">
@@ -5823,29 +5823,29 @@
       </c>
       <c r="G146" s="3" t="inlineStr">
         <is>
-          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: List the applications waiting for your decision; Open the approval screen.</t>
+          <t xml:space="preserve"> Spring menu by role or permission. Capabilities today: Count the applications waiting at each stage (no time limits are set yet).</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="3" t="inlineStr">
         <is>
-          <t>workflow/personal-inbox</t>
+          <t>workflow/my-approvals</t>
         </is>
       </c>
       <c r="B147" s="3" t="inlineStr">
         <is>
-          <t>Personal inbox</t>
+          <t>My approvals</t>
         </is>
       </c>
       <c r="C147" s="3" t="inlineStr">
         <is>
-          <t>Workflow</t>
+          <t>workflow</t>
         </is>
       </c>
       <c r="D147" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
+          <t>director, secretary</t>
         </is>
       </c>
       <c r="E147" s="3" t="inlineStr">
@@ -5860,19 +5860,19 @@
       </c>
       <c r="G147" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu roles include: manufacturer, agency, finance, iame, reviewer, programme, director, secretary. Capabilities today: List the applications waiting for you; Open the screen where each is done.</t>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: List the applications waiting for your decision; Open the approval screen.</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="3" t="inlineStr">
         <is>
-          <t>workflow/team-queue</t>
+          <t>workflow/personal-inbox</t>
         </is>
       </c>
       <c r="B148" s="3" t="inlineStr">
         <is>
-          <t>Team queue</t>
+          <t>Personal inbox</t>
         </is>
       </c>
       <c r="C148" s="3" t="inlineStr">
@@ -5887,52 +5887,89 @@
       </c>
       <c r="E148" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F148" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G148" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t xml:space="preserve"> Spring menu roles include: manufacturer, agency, finance, iame, reviewer, programme, director, secretary. Capabilities today: List the applications waiting for you; Open the screen where each is done.</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="3" t="inlineStr">
         <is>
+          <t>workflow/team-queue</t>
+        </is>
+      </c>
+      <c r="B149" s="3" t="inlineStr">
+        <is>
+          <t>Team queue</t>
+        </is>
+      </c>
+      <c r="C149" s="3" t="inlineStr">
+        <is>
+          <t>Workflow</t>
+        </is>
+      </c>
+      <c r="D149" s="3" t="inlineStr">
+        <is>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
+        </is>
+      </c>
+      <c r="E149" s="3" t="inlineStr">
+        <is>
+          <t>Prototype (preview/sample data)</t>
+        </is>
+      </c>
+      <c r="F149" s="3" t="inlineStr">
+        <is>
+          <t>merge</t>
+        </is>
+      </c>
+      <c r="G149" s="3" t="inlineStr">
+        <is>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="3" t="inlineStr">
+        <is>
           <t>workflow/workflow-history</t>
         </is>
       </c>
-      <c r="B149" s="3" t="inlineStr">
+      <c r="B150" s="3" t="inlineStr">
         <is>
           <t>Workflow history</t>
         </is>
       </c>
-      <c r="C149" s="3" t="inlineStr">
+      <c r="C150" s="3" t="inlineStr">
         <is>
           <t>Workflow</t>
         </is>
       </c>
-      <c r="D149" s="3" t="inlineStr">
+      <c r="D150" s="3" t="inlineStr">
         <is>
           <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
         </is>
       </c>
-      <c r="E149" s="3" t="inlineStr">
+      <c r="E150" s="3" t="inlineStr">
         <is>
           <t>Live – BEE service</t>
         </is>
       </c>
-      <c r="F149" s="3" t="inlineStr">
-        <is>
-          <t>merge</t>
-        </is>
-      </c>
-      <c r="G149" s="3" t="inlineStr">
+      <c r="F150" s="3" t="inlineStr">
+        <is>
+          <t>merge</t>
+        </is>
+      </c>
+      <c r="G150" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve"> Spring menu by role or permission. Capabilities today: Choose an application; Read its steps as you are allowed to see them.</t>
         </is>
@@ -5952,7 +5989,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6342,26 +6379,26 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>Work package</t>
+          <t>Cursor brief</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>WP02</t>
+          <t>BRIEF-15</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Identity, session, MFA, model-application policy</t>
+          <t>Register screen: propose and decide closing or revoking an entry</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
     </row>
     <row r="17">
@@ -6372,21 +6409,21 @@
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>WP03</t>
+          <t>WP02</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>OpenAPI contract, BFF, contract tests</t>
+          <t>Identity, session, MFA, model-application policy</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
     </row>
     <row r="18">
@@ -6397,21 +6434,21 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>WP04</t>
+          <t>WP03</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Masters and brand authorisation</t>
+          <t>OpenAPI contract, BFF, contract tests</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E18" s="3" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="19">
@@ -6422,21 +6459,21 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>WP04.2b-1</t>
+          <t>WP04</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Registration: file, trade-licence PDF, fee, Finance confirmation</t>
+          <t>Masters and brand authorisation</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="E19" s="3" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
     </row>
     <row r="20">
@@ -6447,12 +6484,12 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>WP04.2b-2</t>
+          <t>WP04.2b-1</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Registration: recommend, approve, return, reject, resubmit; register entry</t>
+          <t>Registration: file, trade-licence PDF, fee, Finance confirmation</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -6472,21 +6509,21 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>WP04.2b-2b</t>
+          <t>WP04.2b-2</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Revocation and closure of a brand or authorisation by a second person</t>
+          <t>Registration: recommend, approve, return, reject, resubmit; register entry</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E21" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="22">
@@ -6497,12 +6534,12 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>WP04.2b-3</t>
+          <t>WP04.2b-2b</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Model flow uses the registered brand (brand id); live proof of the chain</t>
+          <t>Revocation and closure of a brand or authorisation by a second person</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -6522,12 +6559,12 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>WP05.1a</t>
+          <t>WP04.2b-3</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Read-only model applications UI</t>
+          <t>Model flow uses the registered brand (brand id); live proof of the chain</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -6547,12 +6584,12 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>WP05.1b</t>
+          <t>WP05.1a</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Draft create/edit</t>
+          <t>Read-only model applications UI</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -6572,12 +6609,12 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>WP05.1c</t>
+          <t>WP05.1b</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Draft submission</t>
+          <t>Draft create/edit</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -6597,12 +6634,12 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>WP05.1d</t>
+          <t>WP05.1c</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Submit-time evidence gates</t>
+          <t>Draft submission</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -6622,12 +6659,12 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>WP06.1a</t>
+          <t>WP05.1d</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Document intake and storage</t>
+          <t>Submit-time evidence gates</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -6647,21 +6684,21 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>WP06.2</t>
+          <t>WP06.1a</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Blob retention, orphans, limits (BL-001–003)</t>
+          <t>Document intake and storage</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E28" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="29">
@@ -6672,21 +6709,21 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>WP07.1a</t>
+          <t>WP06.2</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Finance fee confirmation</t>
+          <t>Blob retention, orphans, limits (BL-001–003)</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E29" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -6697,12 +6734,12 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>WP07.1b–f</t>
+          <t>WP07.1a</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>IAME, Reviewer, Rating, Director, Secretary stages</t>
+          <t>Finance fee confirmation</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -6722,12 +6759,12 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>WP07.1g–h</t>
+          <t>WP07.1b–f</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Return, resubmit, rejection</t>
+          <t>IAME, Reviewer, Rating, Director, Secretary stages</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -6747,12 +6784,12 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>WP07.1i–k</t>
+          <t>WP07.1g–h</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>History, inbox, workflow views</t>
+          <t>Return, resubmit, rejection</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -6772,12 +6809,12 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>WP08.1a</t>
+          <t>WP07.1i–k</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Fee rule administration</t>
+          <t>History, inbox, workflow views</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -6797,12 +6834,12 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>WP08.1b</t>
+          <t>WP08.1a</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Tax line on fee rules</t>
+          <t>Fee rule administration</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -6822,12 +6859,12 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>WP08.1c</t>
+          <t>WP08.1b</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Rating schemes administration</t>
+          <t>Tax line on fee rules</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -6847,12 +6884,12 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>WP08.1d</t>
+          <t>WP08.1c</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Permission-based admin menu</t>
+          <t>Rating schemes administration</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -6872,12 +6909,12 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>WP08.1e</t>
+          <t>WP08.1d</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Fee confirmation correction proposals</t>
+          <t>Permission-based admin menu</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -6897,12 +6934,12 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>WP08.1f</t>
+          <t>WP08.1e</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Fee reversal</t>
+          <t>Fee confirmation correction proposals</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -6922,12 +6959,12 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>WP08.1g</t>
+          <t>WP08.1f</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Born-pending and notification proof</t>
+          <t>Fee reversal</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -6947,12 +6984,12 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>WP08.1h</t>
+          <t>WP08.1g</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Business settings (propose/approve numbers)</t>
+          <t>Born-pending and notification proof</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -6972,12 +7009,12 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>WP09.1a</t>
+          <t>WP08.1h</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Certificate record</t>
+          <t>Business settings (propose/approve numbers)</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -6997,12 +7034,12 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>WP09.1b</t>
+          <t>WP09.1a</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Printable certificate and label</t>
+          <t>Certificate record</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -7022,12 +7059,12 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>WP09.1c</t>
+          <t>WP09.1b</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Public verification page</t>
+          <t>Printable certificate and label</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -7047,12 +7084,12 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>WP09.1d</t>
+          <t>WP09.1c</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Verification rate limit</t>
+          <t>Public verification page</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -7072,12 +7109,12 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>WP10.1a</t>
+          <t>WP09.1d</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>In-portal notifications (API)</t>
+          <t>Verification rate limit</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -7097,12 +7134,12 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>WP10.1b</t>
+          <t>WP10.1a</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Notification bell and page</t>
+          <t>In-portal notifications (API)</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -7122,71 +7159,71 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>WP11</t>
+          <t>WP10.1b</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>AI demonstrations (local)</t>
+          <t>Notification bell and page</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E47" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>Platform</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>WP01</t>
+          <t>WP11</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Documentation and design evidence</t>
+          <t>AI demonstrations (local)</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E48" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>Backlog theme</t>
+          <t>Platform</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>BL-024/025</t>
+          <t>WP01</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Feature template and OpenAPI split</t>
+          <t>Documentation and design evidence</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E49" s="3" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
     </row>
     <row r="50">
@@ -7197,45 +7234,70 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>BL-040–042</t>
+          <t>BL-024/025</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+          <t>Feature template and OpenAPI split</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="E50" s="3" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
+          <t>Backlog theme</t>
+        </is>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>BL-040–042</t>
+        </is>
+      </c>
+      <c r="C51" s="3" t="inlineStr">
+        <is>
+          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
           <t>Owner decision</t>
         </is>
       </c>
-      <c r="B51" s="3" t="inlineStr">
+      <c r="B52" s="3" t="inlineStr">
         <is>
           <t>D10</t>
         </is>
       </c>
-      <c r="C51" s="3" t="inlineStr">
+      <c r="C52" s="3" t="inlineStr">
         <is>
           <t>Provisional local rules for notifications (portal only)</t>
         </is>
       </c>
-      <c r="D51" s="3" t="inlineStr">
+      <c r="D52" s="3" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
-      <c r="E51" s="3" t="n">
+      <c r="E52" s="3" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
WP04 accepted as a local package: gate 2025/0 recorded; workbook
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/BEE-portal-status.xlsx
+++ b/docs/tracking/BEE-portal-status.xlsx
@@ -5989,7 +5989,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6464,16 +6464,16 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Masters and brand authorisation</t>
+          <t>Registration and master data (package accepted 14 Oct 2026)</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E19" s="3" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="20">
@@ -6484,12 +6484,12 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>WP04.2b-1</t>
+          <t>WP04.3</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Registration: file, trade-licence PDF, fee, Finance confirmation</t>
+          <t>Audit trail for the register, name reuse, audit and validation tests</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -6509,12 +6509,12 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>WP04.2b-2</t>
+          <t>WP04.2b-1</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Registration: recommend, approve, return, reject, resubmit; register entry</t>
+          <t>Registration: file, trade-licence PDF, fee, Finance confirmation</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -6534,12 +6534,12 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>WP04.2b-2b</t>
+          <t>WP04.2b-2</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Revocation and closure of a brand or authorisation by a second person</t>
+          <t>Registration: recommend, approve, return, reject, resubmit; register entry</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -6559,12 +6559,12 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>WP04.2b-3</t>
+          <t>WP04.2b-2b</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Model flow uses the registered brand (brand id); live proof of the chain</t>
+          <t>Revocation and closure of a brand or authorisation by a second person</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -6584,12 +6584,12 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>WP05.1a</t>
+          <t>WP04.2b-3</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Read-only model applications UI</t>
+          <t>Model flow uses the registered brand (brand id); live proof of the chain</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -6609,12 +6609,12 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>WP05.1b</t>
+          <t>WP05.1a</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Draft create/edit</t>
+          <t>Read-only model applications UI</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -6634,12 +6634,12 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>WP05.1c</t>
+          <t>WP05.1b</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Draft submission</t>
+          <t>Draft create/edit</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -6659,12 +6659,12 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>WP05.1d</t>
+          <t>WP05.1c</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Submit-time evidence gates</t>
+          <t>Draft submission</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -6684,12 +6684,12 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>WP06.1a</t>
+          <t>WP05.1d</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Document intake and storage</t>
+          <t>Submit-time evidence gates</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -6709,21 +6709,21 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>WP06.2</t>
+          <t>WP06.1a</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Blob retention, orphans, limits (BL-001–003)</t>
+          <t>Document intake and storage</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E29" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="30">
@@ -6734,21 +6734,21 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>WP07.1a</t>
+          <t>WP06.2</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Finance fee confirmation</t>
+          <t>Blob retention, orphans, limits (BL-001–003)</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E30" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -6759,12 +6759,12 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>WP07.1b–f</t>
+          <t>WP07.1a</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>IAME, Reviewer, Rating, Director, Secretary stages</t>
+          <t>Finance fee confirmation</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -6784,12 +6784,12 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>WP07.1g–h</t>
+          <t>WP07.1b–f</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Return, resubmit, rejection</t>
+          <t>IAME, Reviewer, Rating, Director, Secretary stages</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -6809,12 +6809,12 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>WP07.1i–k</t>
+          <t>WP07.1g–h</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>History, inbox, workflow views</t>
+          <t>Return, resubmit, rejection</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -6834,12 +6834,12 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>WP08.1a</t>
+          <t>WP07.1i–k</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Fee rule administration</t>
+          <t>History, inbox, workflow views</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -6859,12 +6859,12 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>WP08.1b</t>
+          <t>WP08.1a</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Tax line on fee rules</t>
+          <t>Fee rule administration</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -6884,12 +6884,12 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>WP08.1c</t>
+          <t>WP08.1b</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Rating schemes administration</t>
+          <t>Tax line on fee rules</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -6909,12 +6909,12 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>WP08.1d</t>
+          <t>WP08.1c</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Permission-based admin menu</t>
+          <t>Rating schemes administration</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -6934,12 +6934,12 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>WP08.1e</t>
+          <t>WP08.1d</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Fee confirmation correction proposals</t>
+          <t>Permission-based admin menu</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -6959,12 +6959,12 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>WP08.1f</t>
+          <t>WP08.1e</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Fee reversal</t>
+          <t>Fee confirmation correction proposals</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -6984,12 +6984,12 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>WP08.1g</t>
+          <t>WP08.1f</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Born-pending and notification proof</t>
+          <t>Fee reversal</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -7009,12 +7009,12 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>WP08.1h</t>
+          <t>WP08.1g</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Business settings (propose/approve numbers)</t>
+          <t>Born-pending and notification proof</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -7034,12 +7034,12 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>WP09.1a</t>
+          <t>WP08.1h</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Certificate record</t>
+          <t>Business settings (propose/approve numbers)</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -7059,12 +7059,12 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>WP09.1b</t>
+          <t>WP09.1a</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Printable certificate and label</t>
+          <t>Certificate record</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -7084,12 +7084,12 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>WP09.1c</t>
+          <t>WP09.1b</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Public verification page</t>
+          <t>Printable certificate and label</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -7109,12 +7109,12 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>WP09.1d</t>
+          <t>WP09.1c</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Verification rate limit</t>
+          <t>Public verification page</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -7134,12 +7134,12 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>WP10.1a</t>
+          <t>WP09.1d</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>In-portal notifications (API)</t>
+          <t>Verification rate limit</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -7159,12 +7159,12 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>WP10.1b</t>
+          <t>WP10.1a</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Notification bell and page</t>
+          <t>In-portal notifications (API)</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
@@ -7184,71 +7184,71 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>WP11</t>
+          <t>WP10.1b</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>AI demonstrations (local)</t>
+          <t>Notification bell and page</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E48" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>Platform</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>WP01</t>
+          <t>WP11</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Documentation and design evidence</t>
+          <t>AI demonstrations (local)</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E49" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>Backlog theme</t>
+          <t>Platform</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>BL-024/025</t>
+          <t>WP01</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Feature template and OpenAPI split</t>
+          <t>Documentation and design evidence</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E50" s="3" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
     </row>
     <row r="51">
@@ -7259,45 +7259,70 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>BL-040–042</t>
+          <t>BL-024/025</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+          <t>Feature template and OpenAPI split</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="E51" s="3" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
+          <t>Backlog theme</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>BL-040–042</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
           <t>Owner decision</t>
         </is>
       </c>
-      <c r="B52" s="3" t="inlineStr">
+      <c r="B53" s="3" t="inlineStr">
         <is>
           <t>D10</t>
         </is>
       </c>
-      <c r="C52" s="3" t="inlineStr">
+      <c r="C53" s="3" t="inlineStr">
         <is>
           <t>Provisional local rules for notifications (portal only)</t>
         </is>
       </c>
-      <c r="D52" s="3" t="inlineStr">
+      <c r="D53" s="3" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
-      <c r="E52" s="3" t="n">
+      <c r="E53" s="3" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
WP04 package review: audit trail, name reuse, expired period, WP04.3 evidence; WP04 accepted (#52)
* WP04 package review: audit trail (V47), name reuse after revocation (V47, V48), expired period at approval, WP04.3 evidence, status documents; contract 0.31.0

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

* WP04 package review: stronger audit test, second review recorded, BL-191

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

* WP04 accepted as a local package: gate 2025/0 recorded; workbook

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

---------

Co-authored-by: Sameer Khanna <sameerkhanna@Sameers-MacBook-Pro.local>
Co-authored-by: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/BEE-portal-status.xlsx
+++ b/docs/tracking/BEE-portal-status.xlsx
@@ -5989,7 +5989,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6464,16 +6464,16 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Masters and brand authorisation</t>
+          <t>Registration and master data (package accepted 14 Oct 2026)</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E19" s="3" t="n">
-        <v>90</v>
+        <v>100</v>
       </c>
     </row>
     <row r="20">
@@ -6484,12 +6484,12 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>WP04.2b-1</t>
+          <t>WP04.3</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Registration: file, trade-licence PDF, fee, Finance confirmation</t>
+          <t>Audit trail for the register, name reuse, audit and validation tests</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
@@ -6509,12 +6509,12 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>WP04.2b-2</t>
+          <t>WP04.2b-1</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Registration: recommend, approve, return, reject, resubmit; register entry</t>
+          <t>Registration: file, trade-licence PDF, fee, Finance confirmation</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
@@ -6534,12 +6534,12 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>WP04.2b-2b</t>
+          <t>WP04.2b-2</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Revocation and closure of a brand or authorisation by a second person</t>
+          <t>Registration: recommend, approve, return, reject, resubmit; register entry</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -6559,12 +6559,12 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>WP04.2b-3</t>
+          <t>WP04.2b-2b</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Model flow uses the registered brand (brand id); live proof of the chain</t>
+          <t>Revocation and closure of a brand or authorisation by a second person</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -6584,12 +6584,12 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>WP05.1a</t>
+          <t>WP04.2b-3</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Read-only model applications UI</t>
+          <t>Model flow uses the registered brand (brand id); live proof of the chain</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -6609,12 +6609,12 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>WP05.1b</t>
+          <t>WP05.1a</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Draft create/edit</t>
+          <t>Read-only model applications UI</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -6634,12 +6634,12 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>WP05.1c</t>
+          <t>WP05.1b</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Draft submission</t>
+          <t>Draft create/edit</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -6659,12 +6659,12 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>WP05.1d</t>
+          <t>WP05.1c</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Submit-time evidence gates</t>
+          <t>Draft submission</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -6684,12 +6684,12 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>WP06.1a</t>
+          <t>WP05.1d</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Document intake and storage</t>
+          <t>Submit-time evidence gates</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -6709,21 +6709,21 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>WP06.2</t>
+          <t>WP06.1a</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Blob retention, orphans, limits (BL-001–003)</t>
+          <t>Document intake and storage</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E29" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="30">
@@ -6734,21 +6734,21 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>WP07.1a</t>
+          <t>WP06.2</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Finance fee confirmation</t>
+          <t>Blob retention, orphans, limits (BL-001–003)</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E30" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31">
@@ -6759,12 +6759,12 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>WP07.1b–f</t>
+          <t>WP07.1a</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>IAME, Reviewer, Rating, Director, Secretary stages</t>
+          <t>Finance fee confirmation</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -6784,12 +6784,12 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>WP07.1g–h</t>
+          <t>WP07.1b–f</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Return, resubmit, rejection</t>
+          <t>IAME, Reviewer, Rating, Director, Secretary stages</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -6809,12 +6809,12 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>WP07.1i–k</t>
+          <t>WP07.1g–h</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>History, inbox, workflow views</t>
+          <t>Return, resubmit, rejection</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -6834,12 +6834,12 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>WP08.1a</t>
+          <t>WP07.1i–k</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Fee rule administration</t>
+          <t>History, inbox, workflow views</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -6859,12 +6859,12 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>WP08.1b</t>
+          <t>WP08.1a</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Tax line on fee rules</t>
+          <t>Fee rule administration</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -6884,12 +6884,12 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>WP08.1c</t>
+          <t>WP08.1b</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Rating schemes administration</t>
+          <t>Tax line on fee rules</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -6909,12 +6909,12 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>WP08.1d</t>
+          <t>WP08.1c</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Permission-based admin menu</t>
+          <t>Rating schemes administration</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -6934,12 +6934,12 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>WP08.1e</t>
+          <t>WP08.1d</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Fee confirmation correction proposals</t>
+          <t>Permission-based admin menu</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -6959,12 +6959,12 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>WP08.1f</t>
+          <t>WP08.1e</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Fee reversal</t>
+          <t>Fee confirmation correction proposals</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -6984,12 +6984,12 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>WP08.1g</t>
+          <t>WP08.1f</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Born-pending and notification proof</t>
+          <t>Fee reversal</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -7009,12 +7009,12 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>WP08.1h</t>
+          <t>WP08.1g</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Business settings (propose/approve numbers)</t>
+          <t>Born-pending and notification proof</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -7034,12 +7034,12 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>WP09.1a</t>
+          <t>WP08.1h</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Certificate record</t>
+          <t>Business settings (propose/approve numbers)</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -7059,12 +7059,12 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>WP09.1b</t>
+          <t>WP09.1a</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Printable certificate and label</t>
+          <t>Certificate record</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -7084,12 +7084,12 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>WP09.1c</t>
+          <t>WP09.1b</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Public verification page</t>
+          <t>Printable certificate and label</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -7109,12 +7109,12 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>WP09.1d</t>
+          <t>WP09.1c</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Verification rate limit</t>
+          <t>Public verification page</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -7134,12 +7134,12 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>WP10.1a</t>
+          <t>WP09.1d</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>In-portal notifications (API)</t>
+          <t>Verification rate limit</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -7159,12 +7159,12 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>WP10.1b</t>
+          <t>WP10.1a</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Notification bell and page</t>
+          <t>In-portal notifications (API)</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
@@ -7184,71 +7184,71 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>WP11</t>
+          <t>WP10.1b</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>AI demonstrations (local)</t>
+          <t>Notification bell and page</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E48" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>Platform</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>WP01</t>
+          <t>WP11</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Documentation and design evidence</t>
+          <t>AI demonstrations (local)</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E49" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>Backlog theme</t>
+          <t>Platform</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>BL-024/025</t>
+          <t>WP01</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Feature template and OpenAPI split</t>
+          <t>Documentation and design evidence</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E50" s="3" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
     </row>
     <row r="51">
@@ -7259,45 +7259,70 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>BL-040–042</t>
+          <t>BL-024/025</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+          <t>Feature template and OpenAPI split</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="E51" s="3" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
+          <t>Backlog theme</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>BL-040–042</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
           <t>Owner decision</t>
         </is>
       </c>
-      <c r="B52" s="3" t="inlineStr">
+      <c r="B53" s="3" t="inlineStr">
         <is>
           <t>D10</t>
         </is>
       </c>
-      <c r="C52" s="3" t="inlineStr">
+      <c r="C53" s="3" t="inlineStr">
         <is>
           <t>Provisional local rules for notifications (portal only)</t>
         </is>
       </c>
-      <c r="D52" s="3" t="inlineStr">
+      <c r="D53" s="3" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
-      <c r="E52" s="3" t="n">
+      <c r="E53" s="3" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
WP02.4: gate 2063/0 recorded; workbook (WP02 slices, WP04 order)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/BEE-portal-status.xlsx
+++ b/docs/tracking/BEE-portal-status.xlsx
@@ -5989,7 +5989,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6423,7 +6423,7 @@
         </is>
       </c>
       <c r="E17" s="3" t="n">
-        <v>75</v>
+        <v>85</v>
       </c>
     </row>
     <row r="18">
@@ -6434,12 +6434,12 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>WP03</t>
+          <t>WP02.4a</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>OpenAPI contract, BFF, contract tests</t>
+          <t>Keycloak brute-force detection (temporary lockout)</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -6459,12 +6459,12 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>WP04</t>
+          <t>WP02.4b</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Registration and master data (package accepted 14 Oct 2026)</t>
+          <t>Complete denial evidence: cases N1 to N10 and A7</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -6484,21 +6484,21 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>WP04.3</t>
+          <t>WP02.4c</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Audit trail for the register, name reuse, audit and validation tests</t>
+          <t>Delegation (maker-checker, expiry, revocation, audit)</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="E20" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -6509,21 +6509,21 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>WP04.2b-1</t>
+          <t>WP02.5</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Registration: file, trade-licence PDF, fee, Finance confirmation</t>
+          <t>Escalation (R12): waits for BEE's time limits per stage (B14)</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E21" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -6534,12 +6534,12 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>WP04.2b-2</t>
+          <t>WP03</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Registration: recommend, approve, return, reject, resubmit; register entry</t>
+          <t>OpenAPI contract, BFF, contract tests</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -6559,12 +6559,12 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>WP04.2b-2b</t>
+          <t>WP04</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Revocation and closure of a brand or authorisation by a second person</t>
+          <t>Registration and master data (package accepted 14 Oct 2026)</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -6584,12 +6584,12 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>WP04.2b-3</t>
+          <t>WP04.2b-1</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Model flow uses the registered brand (brand id); live proof of the chain</t>
+          <t>Registration: file, trade-licence PDF, fee, Finance confirmation</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -6609,12 +6609,12 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>WP05.1a</t>
+          <t>WP04.2b-2</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Read-only model applications UI</t>
+          <t>Registration: recommend, approve, return, reject, resubmit; register entry</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -6634,12 +6634,12 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>WP05.1b</t>
+          <t>WP04.2b-2b</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Draft create/edit</t>
+          <t>Revocation and closure of a brand or authorisation by a second person</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -6659,12 +6659,12 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>WP05.1c</t>
+          <t>WP04.2b-3</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Draft submission</t>
+          <t>Model flow uses the registered brand (brand id); live proof of the chain</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -6684,12 +6684,12 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>WP05.1d</t>
+          <t>WP04.3</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Submit-time evidence gates</t>
+          <t>Audit trail for the register, name reuse, audit and validation tests</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -6709,12 +6709,12 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>WP06.1a</t>
+          <t>WP05.1a</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Document intake and storage</t>
+          <t>Read-only model applications UI</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -6734,21 +6734,21 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>WP06.2</t>
+          <t>WP05.1b</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Blob retention, orphans, limits (BL-001–003)</t>
+          <t>Draft create/edit</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E30" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="31">
@@ -6759,12 +6759,12 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>WP07.1a</t>
+          <t>WP05.1c</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Finance fee confirmation</t>
+          <t>Draft submission</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -6784,12 +6784,12 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>WP07.1b–f</t>
+          <t>WP05.1d</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>IAME, Reviewer, Rating, Director, Secretary stages</t>
+          <t>Submit-time evidence gates</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -6809,12 +6809,12 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>WP07.1g–h</t>
+          <t>WP06.1a</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Return, resubmit, rejection</t>
+          <t>Document intake and storage</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -6834,21 +6834,21 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>WP07.1i–k</t>
+          <t>WP06.2</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>History, inbox, workflow views</t>
+          <t>Blob retention, orphans, limits (BL-001–003)</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E34" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -6859,12 +6859,12 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>WP08.1a</t>
+          <t>WP07.1a</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Fee rule administration</t>
+          <t>Finance fee confirmation</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -6884,12 +6884,12 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>WP08.1b</t>
+          <t>WP07.1b–f</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Tax line on fee rules</t>
+          <t>IAME, Reviewer, Rating, Director, Secretary stages</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -6909,12 +6909,12 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>WP08.1c</t>
+          <t>WP07.1g–h</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Rating schemes administration</t>
+          <t>Return, resubmit, rejection</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -6934,12 +6934,12 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>WP08.1d</t>
+          <t>WP07.1i–k</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Permission-based admin menu</t>
+          <t>History, inbox, workflow views</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -6959,12 +6959,12 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>WP08.1e</t>
+          <t>WP08.1a</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Fee confirmation correction proposals</t>
+          <t>Fee rule administration</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -6984,12 +6984,12 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>WP08.1f</t>
+          <t>WP08.1b</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Fee reversal</t>
+          <t>Tax line on fee rules</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -7009,12 +7009,12 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>WP08.1g</t>
+          <t>WP08.1c</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Born-pending and notification proof</t>
+          <t>Rating schemes administration</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -7034,12 +7034,12 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>WP08.1h</t>
+          <t>WP08.1d</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Business settings (propose/approve numbers)</t>
+          <t>Permission-based admin menu</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -7059,12 +7059,12 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>WP09.1a</t>
+          <t>WP08.1e</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Certificate record</t>
+          <t>Fee confirmation correction proposals</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -7084,12 +7084,12 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>WP09.1b</t>
+          <t>WP08.1f</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Printable certificate and label</t>
+          <t>Fee reversal</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -7109,12 +7109,12 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>WP09.1c</t>
+          <t>WP08.1g</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Public verification page</t>
+          <t>Born-pending and notification proof</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -7134,12 +7134,12 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>WP09.1d</t>
+          <t>WP08.1h</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Verification rate limit</t>
+          <t>Business settings (propose/approve numbers)</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -7159,12 +7159,12 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>WP10.1a</t>
+          <t>WP09.1a</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>In-portal notifications (API)</t>
+          <t>Certificate record</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
@@ -7184,12 +7184,12 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>WP10.1b</t>
+          <t>WP09.1b</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Notification bell and page</t>
+          <t>Printable certificate and label</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
@@ -7209,37 +7209,37 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>WP11</t>
+          <t>WP09.1c</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>AI demonstrations (local)</t>
+          <t>Public verification page</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E49" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>Platform</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>WP01</t>
+          <t>WP09.1d</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Documentation and design evidence</t>
+          <t>Verification rate limit</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
@@ -7254,75 +7254,175 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>Backlog theme</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>BL-024/025</t>
+          <t>WP10.1a</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Feature template and OpenAPI split</t>
+          <t>In-portal notifications (API)</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E51" s="3" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>Backlog theme</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>BL-040–042</t>
+          <t>WP10.1b</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+          <t>Notification bell and page</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E52" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
+          <t>Work package</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>WP11</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>AI demonstrations (local)</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>WP01</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>Documentation and design evidence</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>Backlog theme</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>BL-024/025</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>Feature template and OpenAPI split</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>Backlog theme</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>BL-040–042</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
           <t>Owner decision</t>
         </is>
       </c>
-      <c r="B53" s="3" t="inlineStr">
+      <c r="B57" s="3" t="inlineStr">
         <is>
           <t>D10</t>
         </is>
       </c>
-      <c r="C53" s="3" t="inlineStr">
+      <c r="C57" s="3" t="inlineStr">
         <is>
           <t>Provisional local rules for notifications (portal only)</t>
         </is>
       </c>
-      <c r="D53" s="3" t="inlineStr">
+      <c r="D57" s="3" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
-      <c r="E53" s="3" t="n">
+      <c r="E57" s="3" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
WP02.4: Keycloak brute-force detection and the complete denial suite (N1-N10, A7) (#53)
* WP02.4: Keycloak brute-force detection, the complete denial suite (N1 to N10, A7), evidence note

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

* WP02.3 note: gaps closed by WP02.4

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

* WP02.4 review fixes: a 401 is not a denial, controls for the suite, crash recovery, realm policy in the docker start path, honest N6/N7 wording; BL-192

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

* WP02.4: drop an unused eslint-disable line

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

* WP02.4: gate 2063/0 recorded; workbook (WP02 slices, WP04 order)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

---------

Co-authored-by: Sameer Khanna <sameerkhanna@Sameers-MacBook-Pro.local>
Co-authored-by: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/BEE-portal-status.xlsx
+++ b/docs/tracking/BEE-portal-status.xlsx
@@ -5989,7 +5989,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6423,7 +6423,7 @@
         </is>
       </c>
       <c r="E17" s="3" t="n">
-        <v>75</v>
+        <v>85</v>
       </c>
     </row>
     <row r="18">
@@ -6434,12 +6434,12 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>WP03</t>
+          <t>WP02.4a</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>OpenAPI contract, BFF, contract tests</t>
+          <t>Keycloak brute-force detection (temporary lockout)</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -6459,12 +6459,12 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>WP04</t>
+          <t>WP02.4b</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Registration and master data (package accepted 14 Oct 2026)</t>
+          <t>Complete denial evidence: cases N1 to N10 and A7</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -6484,21 +6484,21 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>WP04.3</t>
+          <t>WP02.4c</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Audit trail for the register, name reuse, audit and validation tests</t>
+          <t>Delegation (maker-checker, expiry, revocation, audit)</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="E20" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21">
@@ -6509,21 +6509,21 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>WP04.2b-1</t>
+          <t>WP02.5</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Registration: file, trade-licence PDF, fee, Finance confirmation</t>
+          <t>Escalation (R12): waits for BEE's time limits per stage (B14)</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E21" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -6534,12 +6534,12 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>WP04.2b-2</t>
+          <t>WP03</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Registration: recommend, approve, return, reject, resubmit; register entry</t>
+          <t>OpenAPI contract, BFF, contract tests</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -6559,12 +6559,12 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>WP04.2b-2b</t>
+          <t>WP04</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Revocation and closure of a brand or authorisation by a second person</t>
+          <t>Registration and master data (package accepted 14 Oct 2026)</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -6584,12 +6584,12 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>WP04.2b-3</t>
+          <t>WP04.2b-1</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Model flow uses the registered brand (brand id); live proof of the chain</t>
+          <t>Registration: file, trade-licence PDF, fee, Finance confirmation</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -6609,12 +6609,12 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>WP05.1a</t>
+          <t>WP04.2b-2</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Read-only model applications UI</t>
+          <t>Registration: recommend, approve, return, reject, resubmit; register entry</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -6634,12 +6634,12 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>WP05.1b</t>
+          <t>WP04.2b-2b</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Draft create/edit</t>
+          <t>Revocation and closure of a brand or authorisation by a second person</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -6659,12 +6659,12 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>WP05.1c</t>
+          <t>WP04.2b-3</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Draft submission</t>
+          <t>Model flow uses the registered brand (brand id); live proof of the chain</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -6684,12 +6684,12 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>WP05.1d</t>
+          <t>WP04.3</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Submit-time evidence gates</t>
+          <t>Audit trail for the register, name reuse, audit and validation tests</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -6709,12 +6709,12 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>WP06.1a</t>
+          <t>WP05.1a</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Document intake and storage</t>
+          <t>Read-only model applications UI</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -6734,21 +6734,21 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>WP06.2</t>
+          <t>WP05.1b</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Blob retention, orphans, limits (BL-001–003)</t>
+          <t>Draft create/edit</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E30" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="31">
@@ -6759,12 +6759,12 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>WP07.1a</t>
+          <t>WP05.1c</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Finance fee confirmation</t>
+          <t>Draft submission</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -6784,12 +6784,12 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>WP07.1b–f</t>
+          <t>WP05.1d</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>IAME, Reviewer, Rating, Director, Secretary stages</t>
+          <t>Submit-time evidence gates</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -6809,12 +6809,12 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>WP07.1g–h</t>
+          <t>WP06.1a</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Return, resubmit, rejection</t>
+          <t>Document intake and storage</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -6834,21 +6834,21 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>WP07.1i–k</t>
+          <t>WP06.2</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>History, inbox, workflow views</t>
+          <t>Blob retention, orphans, limits (BL-001–003)</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E34" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
@@ -6859,12 +6859,12 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>WP08.1a</t>
+          <t>WP07.1a</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Fee rule administration</t>
+          <t>Finance fee confirmation</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -6884,12 +6884,12 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>WP08.1b</t>
+          <t>WP07.1b–f</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Tax line on fee rules</t>
+          <t>IAME, Reviewer, Rating, Director, Secretary stages</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -6909,12 +6909,12 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>WP08.1c</t>
+          <t>WP07.1g–h</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Rating schemes administration</t>
+          <t>Return, resubmit, rejection</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -6934,12 +6934,12 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>WP08.1d</t>
+          <t>WP07.1i–k</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Permission-based admin menu</t>
+          <t>History, inbox, workflow views</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -6959,12 +6959,12 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>WP08.1e</t>
+          <t>WP08.1a</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Fee confirmation correction proposals</t>
+          <t>Fee rule administration</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -6984,12 +6984,12 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>WP08.1f</t>
+          <t>WP08.1b</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Fee reversal</t>
+          <t>Tax line on fee rules</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -7009,12 +7009,12 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>WP08.1g</t>
+          <t>WP08.1c</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Born-pending and notification proof</t>
+          <t>Rating schemes administration</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -7034,12 +7034,12 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>WP08.1h</t>
+          <t>WP08.1d</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Business settings (propose/approve numbers)</t>
+          <t>Permission-based admin menu</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -7059,12 +7059,12 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>WP09.1a</t>
+          <t>WP08.1e</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Certificate record</t>
+          <t>Fee confirmation correction proposals</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -7084,12 +7084,12 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>WP09.1b</t>
+          <t>WP08.1f</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Printable certificate and label</t>
+          <t>Fee reversal</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -7109,12 +7109,12 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>WP09.1c</t>
+          <t>WP08.1g</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Public verification page</t>
+          <t>Born-pending and notification proof</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -7134,12 +7134,12 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>WP09.1d</t>
+          <t>WP08.1h</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Verification rate limit</t>
+          <t>Business settings (propose/approve numbers)</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -7159,12 +7159,12 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>WP10.1a</t>
+          <t>WP09.1a</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>In-portal notifications (API)</t>
+          <t>Certificate record</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
@@ -7184,12 +7184,12 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>WP10.1b</t>
+          <t>WP09.1b</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Notification bell and page</t>
+          <t>Printable certificate and label</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
@@ -7209,37 +7209,37 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>WP11</t>
+          <t>WP09.1c</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>AI demonstrations (local)</t>
+          <t>Public verification page</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E49" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>Platform</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>WP01</t>
+          <t>WP09.1d</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Documentation and design evidence</t>
+          <t>Verification rate limit</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
@@ -7254,75 +7254,175 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>Backlog theme</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>BL-024/025</t>
+          <t>WP10.1a</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Feature template and OpenAPI split</t>
+          <t>In-portal notifications (API)</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E51" s="3" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>Backlog theme</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>BL-040–042</t>
+          <t>WP10.1b</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+          <t>Notification bell and page</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E52" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
+          <t>Work package</t>
+        </is>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>WP11</t>
+        </is>
+      </c>
+      <c r="C53" s="3" t="inlineStr">
+        <is>
+          <t>AI demonstrations (local)</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>WP01</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>Documentation and design evidence</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>Backlog theme</t>
+        </is>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>BL-024/025</t>
+        </is>
+      </c>
+      <c r="C55" s="3" t="inlineStr">
+        <is>
+          <t>Feature template and OpenAPI split</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>Backlog theme</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>BL-040–042</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
+        <is>
           <t>Owner decision</t>
         </is>
       </c>
-      <c r="B53" s="3" t="inlineStr">
+      <c r="B57" s="3" t="inlineStr">
         <is>
           <t>D10</t>
         </is>
       </c>
-      <c r="C53" s="3" t="inlineStr">
+      <c r="C57" s="3" t="inlineStr">
         <is>
           <t>Provisional local rules for notifications (portal only)</t>
         </is>
       </c>
-      <c r="D53" s="3" t="inlineStr">
+      <c r="D57" s="3" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
-      <c r="E53" s="3" t="n">
+      <c r="E57" s="3" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
WP02.4c: delegation of a stage role (V49, contract 0.32.0)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/BEE-portal-status.xlsx
+++ b/docs/tracking/BEE-portal-status.xlsx
@@ -5989,7 +5989,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6404,26 +6404,26 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Work package</t>
+          <t>Cursor brief</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>WP02</t>
+          <t>BRIEF-16</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Identity, session, MFA, model-application policy</t>
+          <t>Delegation screen (ask, approve, revoke, my delegations)</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
-        <v>85</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -6434,21 +6434,21 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>WP02.4a</t>
+          <t>WP02</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Keycloak brute-force detection (temporary lockout)</t>
+          <t>Identity, session, MFA, model-application policy</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="E18" s="3" t="n">
-        <v>100</v>
+        <v>92</v>
       </c>
     </row>
     <row r="19">
@@ -6459,12 +6459,12 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>WP02.4b</t>
+          <t>WP02.4a</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Complete denial evidence: cases N1 to N10 and A7</t>
+          <t>Keycloak brute-force detection (temporary lockout)</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -6484,21 +6484,21 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>WP02.4c</t>
+          <t>WP02.4b</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Delegation (maker-checker, expiry, revocation, audit)</t>
+          <t>Complete denial evidence: cases N1 to N10 and A7</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E20" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="21">
@@ -6509,21 +6509,21 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>WP02.5</t>
+          <t>WP02.4c</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Escalation (R12): waits for BEE's time limits per stage (B14)</t>
+          <t>Delegation (maker-checker, expiry, revocation, audit)</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E21" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="22">
@@ -6534,21 +6534,21 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>WP03</t>
+          <t>WP02.5</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>OpenAPI contract, BFF, contract tests</t>
+          <t>Escalation (R12): waits for BEE's time limits per stage (B14)</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E22" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -6559,12 +6559,12 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>WP04</t>
+          <t>WP03</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Registration and master data (package accepted 14 Oct 2026)</t>
+          <t>OpenAPI contract, BFF, contract tests</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -6584,12 +6584,12 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>WP04.2b-1</t>
+          <t>WP04</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Registration: file, trade-licence PDF, fee, Finance confirmation</t>
+          <t>Registration and master data (package accepted 14 Oct 2026)</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -6609,12 +6609,12 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>WP04.2b-2</t>
+          <t>WP04.2b-1</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Registration: recommend, approve, return, reject, resubmit; register entry</t>
+          <t>Registration: file, trade-licence PDF, fee, Finance confirmation</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -6634,12 +6634,12 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>WP04.2b-2b</t>
+          <t>WP04.2b-2</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Revocation and closure of a brand or authorisation by a second person</t>
+          <t>Registration: recommend, approve, return, reject, resubmit; register entry</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -6659,12 +6659,12 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>WP04.2b-3</t>
+          <t>WP04.2b-2b</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Model flow uses the registered brand (brand id); live proof of the chain</t>
+          <t>Revocation and closure of a brand or authorisation by a second person</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -6684,12 +6684,12 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>WP04.3</t>
+          <t>WP04.2b-3</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Audit trail for the register, name reuse, audit and validation tests</t>
+          <t>Model flow uses the registered brand (brand id); live proof of the chain</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -6709,12 +6709,12 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>WP05.1a</t>
+          <t>WP04.3</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Read-only model applications UI</t>
+          <t>Audit trail for the register, name reuse, audit and validation tests</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -6734,12 +6734,12 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>WP05.1b</t>
+          <t>WP05.1a</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Draft create/edit</t>
+          <t>Read-only model applications UI</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -6759,12 +6759,12 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>WP05.1c</t>
+          <t>WP05.1b</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Draft submission</t>
+          <t>Draft create/edit</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -6784,12 +6784,12 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>WP05.1d</t>
+          <t>WP05.1c</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Submit-time evidence gates</t>
+          <t>Draft submission</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -6809,12 +6809,12 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>WP06.1a</t>
+          <t>WP05.1d</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Document intake and storage</t>
+          <t>Submit-time evidence gates</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -6834,21 +6834,21 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>WP06.2</t>
+          <t>WP06.1a</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Blob retention, orphans, limits (BL-001–003)</t>
+          <t>Document intake and storage</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E34" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="35">
@@ -6859,21 +6859,21 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>WP07.1a</t>
+          <t>WP06.2</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Finance fee confirmation</t>
+          <t>Blob retention, orphans, limits (BL-001–003)</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E35" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -6884,12 +6884,12 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>WP07.1b–f</t>
+          <t>WP07.1a</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>IAME, Reviewer, Rating, Director, Secretary stages</t>
+          <t>Finance fee confirmation</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -6909,12 +6909,12 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>WP07.1g–h</t>
+          <t>WP07.1b–f</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Return, resubmit, rejection</t>
+          <t>IAME, Reviewer, Rating, Director, Secretary stages</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -6934,12 +6934,12 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>WP07.1i–k</t>
+          <t>WP07.1g–h</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>History, inbox, workflow views</t>
+          <t>Return, resubmit, rejection</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -6959,12 +6959,12 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>WP08.1a</t>
+          <t>WP07.1i–k</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Fee rule administration</t>
+          <t>History, inbox, workflow views</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -6984,12 +6984,12 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>WP08.1b</t>
+          <t>WP08.1a</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Tax line on fee rules</t>
+          <t>Fee rule administration</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -7009,12 +7009,12 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>WP08.1c</t>
+          <t>WP08.1b</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Rating schemes administration</t>
+          <t>Tax line on fee rules</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -7034,12 +7034,12 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>WP08.1d</t>
+          <t>WP08.1c</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Permission-based admin menu</t>
+          <t>Rating schemes administration</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -7059,12 +7059,12 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>WP08.1e</t>
+          <t>WP08.1d</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Fee confirmation correction proposals</t>
+          <t>Permission-based admin menu</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -7084,12 +7084,12 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>WP08.1f</t>
+          <t>WP08.1e</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Fee reversal</t>
+          <t>Fee confirmation correction proposals</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -7109,12 +7109,12 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>WP08.1g</t>
+          <t>WP08.1f</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Born-pending and notification proof</t>
+          <t>Fee reversal</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -7134,12 +7134,12 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>WP08.1h</t>
+          <t>WP08.1g</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Business settings (propose/approve numbers)</t>
+          <t>Born-pending and notification proof</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -7159,12 +7159,12 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>WP09.1a</t>
+          <t>WP08.1h</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Certificate record</t>
+          <t>Business settings (propose/approve numbers)</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
@@ -7184,12 +7184,12 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>WP09.1b</t>
+          <t>WP09.1a</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Printable certificate and label</t>
+          <t>Certificate record</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
@@ -7209,12 +7209,12 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>WP09.1c</t>
+          <t>WP09.1b</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Public verification page</t>
+          <t>Printable certificate and label</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -7234,12 +7234,12 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>WP09.1d</t>
+          <t>WP09.1c</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Verification rate limit</t>
+          <t>Public verification page</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
@@ -7259,12 +7259,12 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>WP10.1a</t>
+          <t>WP09.1d</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>In-portal notifications (API)</t>
+          <t>Verification rate limit</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -7284,12 +7284,12 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>WP10.1b</t>
+          <t>WP10.1a</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Notification bell and page</t>
+          <t>In-portal notifications (API)</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -7309,71 +7309,71 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>WP11</t>
+          <t>WP10.1b</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>AI demonstrations (local)</t>
+          <t>Notification bell and page</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E53" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>Platform</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>WP01</t>
+          <t>WP11</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Documentation and design evidence</t>
+          <t>AI demonstrations (local)</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E54" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>Backlog theme</t>
+          <t>Platform</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>BL-024/025</t>
+          <t>WP01</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Feature template and OpenAPI split</t>
+          <t>Documentation and design evidence</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E55" s="3" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
     </row>
     <row r="56">
@@ -7384,45 +7384,70 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>BL-040–042</t>
+          <t>BL-024/025</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+          <t>Feature template and OpenAPI split</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="E56" s="3" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
+          <t>Backlog theme</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>BL-040–042</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
           <t>Owner decision</t>
         </is>
       </c>
-      <c r="B57" s="3" t="inlineStr">
+      <c r="B58" s="3" t="inlineStr">
         <is>
           <t>D10</t>
         </is>
       </c>
-      <c r="C57" s="3" t="inlineStr">
+      <c r="C58" s="3" t="inlineStr">
         <is>
           <t>Provisional local rules for notifications (portal only)</t>
         </is>
       </c>
-      <c r="D57" s="3" t="inlineStr">
+      <c r="D58" s="3" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
-      <c r="E57" s="3" t="n">
+      <c r="E58" s="3" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
WP02.4c: delegation of a stage role (Programme, Director, Finance) (#54)
* WP02.4c: delegation of a stage role (V49, contract 0.32.0)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

* WP02.4c review fixes: two-stage-role delegator and partner delegate refused (V50), permission before body; BL-198

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

* WP02.4c: keep the 502 responses on the runtime operations; the admin permission list now includes delegation_approve

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

* WP02.4c: second permission-list expectation in FeeRuleDatabaseTest

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

* WP02.4c: gate 2172/0 recorded

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

---------

Co-authored-by: Sameer Khanna <sameerkhanna@Sameers-MacBook-Pro.local>
Co-authored-by: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/BEE-portal-status.xlsx
+++ b/docs/tracking/BEE-portal-status.xlsx
@@ -5989,7 +5989,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E57"/>
+  <dimension ref="A1:E58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6404,26 +6404,26 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Work package</t>
+          <t>Cursor brief</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>WP02</t>
+          <t>BRIEF-16</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>Identity, session, MFA, model-application policy</t>
+          <t>Delegation screen (ask, approve, revoke, my delegations)</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Pending</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
-        <v>85</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -6434,21 +6434,21 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>WP02.4a</t>
+          <t>WP02</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Keycloak brute-force detection (temporary lockout)</t>
+          <t>Identity, session, MFA, model-application policy</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="E18" s="3" t="n">
-        <v>100</v>
+        <v>92</v>
       </c>
     </row>
     <row r="19">
@@ -6459,12 +6459,12 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>WP02.4b</t>
+          <t>WP02.4a</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>Complete denial evidence: cases N1 to N10 and A7</t>
+          <t>Keycloak brute-force detection (temporary lockout)</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
@@ -6484,21 +6484,21 @@
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>WP02.4c</t>
+          <t>WP02.4b</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Delegation (maker-checker, expiry, revocation, audit)</t>
+          <t>Complete denial evidence: cases N1 to N10 and A7</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E20" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="21">
@@ -6509,21 +6509,21 @@
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>WP02.5</t>
+          <t>WP02.4c</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Escalation (R12): waits for BEE's time limits per stage (B14)</t>
+          <t>Delegation (maker-checker, expiry, revocation, audit)</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E21" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="22">
@@ -6534,21 +6534,21 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>WP03</t>
+          <t>WP02.5</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>OpenAPI contract, BFF, contract tests</t>
+          <t>Escalation (R12): waits for BEE's time limits per stage (B14)</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E22" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="23">
@@ -6559,12 +6559,12 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>WP04</t>
+          <t>WP03</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Registration and master data (package accepted 14 Oct 2026)</t>
+          <t>OpenAPI contract, BFF, contract tests</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -6584,12 +6584,12 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>WP04.2b-1</t>
+          <t>WP04</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Registration: file, trade-licence PDF, fee, Finance confirmation</t>
+          <t>Registration and master data (package accepted 14 Oct 2026)</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -6609,12 +6609,12 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>WP04.2b-2</t>
+          <t>WP04.2b-1</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Registration: recommend, approve, return, reject, resubmit; register entry</t>
+          <t>Registration: file, trade-licence PDF, fee, Finance confirmation</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -6634,12 +6634,12 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>WP04.2b-2b</t>
+          <t>WP04.2b-2</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Revocation and closure of a brand or authorisation by a second person</t>
+          <t>Registration: recommend, approve, return, reject, resubmit; register entry</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -6659,12 +6659,12 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>WP04.2b-3</t>
+          <t>WP04.2b-2b</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Model flow uses the registered brand (brand id); live proof of the chain</t>
+          <t>Revocation and closure of a brand or authorisation by a second person</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
@@ -6684,12 +6684,12 @@
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>WP04.3</t>
+          <t>WP04.2b-3</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Audit trail for the register, name reuse, audit and validation tests</t>
+          <t>Model flow uses the registered brand (brand id); live proof of the chain</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -6709,12 +6709,12 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>WP05.1a</t>
+          <t>WP04.3</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Read-only model applications UI</t>
+          <t>Audit trail for the register, name reuse, audit and validation tests</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -6734,12 +6734,12 @@
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>WP05.1b</t>
+          <t>WP05.1a</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Draft create/edit</t>
+          <t>Read-only model applications UI</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -6759,12 +6759,12 @@
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>WP05.1c</t>
+          <t>WP05.1b</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Draft submission</t>
+          <t>Draft create/edit</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -6784,12 +6784,12 @@
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>WP05.1d</t>
+          <t>WP05.1c</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Submit-time evidence gates</t>
+          <t>Draft submission</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -6809,12 +6809,12 @@
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>WP06.1a</t>
+          <t>WP05.1d</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>Document intake and storage</t>
+          <t>Submit-time evidence gates</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
@@ -6834,21 +6834,21 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>WP06.2</t>
+          <t>WP06.1a</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Blob retention, orphans, limits (BL-001–003)</t>
+          <t>Document intake and storage</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E34" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="35">
@@ -6859,21 +6859,21 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>WP07.1a</t>
+          <t>WP06.2</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Finance fee confirmation</t>
+          <t>Blob retention, orphans, limits (BL-001–003)</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E35" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
@@ -6884,12 +6884,12 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>WP07.1b–f</t>
+          <t>WP07.1a</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>IAME, Reviewer, Rating, Director, Secretary stages</t>
+          <t>Finance fee confirmation</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
@@ -6909,12 +6909,12 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>WP07.1g–h</t>
+          <t>WP07.1b–f</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Return, resubmit, rejection</t>
+          <t>IAME, Reviewer, Rating, Director, Secretary stages</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -6934,12 +6934,12 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>WP07.1i–k</t>
+          <t>WP07.1g–h</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>History, inbox, workflow views</t>
+          <t>Return, resubmit, rejection</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -6959,12 +6959,12 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>WP08.1a</t>
+          <t>WP07.1i–k</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Fee rule administration</t>
+          <t>History, inbox, workflow views</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -6984,12 +6984,12 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>WP08.1b</t>
+          <t>WP08.1a</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Tax line on fee rules</t>
+          <t>Fee rule administration</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -7009,12 +7009,12 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>WP08.1c</t>
+          <t>WP08.1b</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Rating schemes administration</t>
+          <t>Tax line on fee rules</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -7034,12 +7034,12 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>WP08.1d</t>
+          <t>WP08.1c</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Permission-based admin menu</t>
+          <t>Rating schemes administration</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -7059,12 +7059,12 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>WP08.1e</t>
+          <t>WP08.1d</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Fee confirmation correction proposals</t>
+          <t>Permission-based admin menu</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -7084,12 +7084,12 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>WP08.1f</t>
+          <t>WP08.1e</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Fee reversal</t>
+          <t>Fee confirmation correction proposals</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -7109,12 +7109,12 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>WP08.1g</t>
+          <t>WP08.1f</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Born-pending and notification proof</t>
+          <t>Fee reversal</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -7134,12 +7134,12 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>WP08.1h</t>
+          <t>WP08.1g</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Business settings (propose/approve numbers)</t>
+          <t>Born-pending and notification proof</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -7159,12 +7159,12 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>WP09.1a</t>
+          <t>WP08.1h</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Certificate record</t>
+          <t>Business settings (propose/approve numbers)</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
@@ -7184,12 +7184,12 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>WP09.1b</t>
+          <t>WP09.1a</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Printable certificate and label</t>
+          <t>Certificate record</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
@@ -7209,12 +7209,12 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>WP09.1c</t>
+          <t>WP09.1b</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Public verification page</t>
+          <t>Printable certificate and label</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -7234,12 +7234,12 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>WP09.1d</t>
+          <t>WP09.1c</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Verification rate limit</t>
+          <t>Public verification page</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
@@ -7259,12 +7259,12 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>WP10.1a</t>
+          <t>WP09.1d</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>In-portal notifications (API)</t>
+          <t>Verification rate limit</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -7284,12 +7284,12 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>WP10.1b</t>
+          <t>WP10.1a</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Notification bell and page</t>
+          <t>In-portal notifications (API)</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -7309,71 +7309,71 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>WP11</t>
+          <t>WP10.1b</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>AI demonstrations (local)</t>
+          <t>Notification bell and page</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E53" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>Platform</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>WP01</t>
+          <t>WP11</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Documentation and design evidence</t>
+          <t>AI demonstrations (local)</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E54" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>Backlog theme</t>
+          <t>Platform</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>BL-024/025</t>
+          <t>WP01</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Feature template and OpenAPI split</t>
+          <t>Documentation and design evidence</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E55" s="3" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
     </row>
     <row r="56">
@@ -7384,45 +7384,70 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>BL-040–042</t>
+          <t>BL-024/025</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+          <t>Feature template and OpenAPI split</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="E56" s="3" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
+          <t>Backlog theme</t>
+        </is>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>BL-040–042</t>
+        </is>
+      </c>
+      <c r="C57" s="3" t="inlineStr">
+        <is>
+          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
           <t>Owner decision</t>
         </is>
       </c>
-      <c r="B57" s="3" t="inlineStr">
+      <c r="B58" s="3" t="inlineStr">
         <is>
           <t>D10</t>
         </is>
       </c>
-      <c r="C57" s="3" t="inlineStr">
+      <c r="C58" s="3" t="inlineStr">
         <is>
           <t>Provisional local rules for notifications (portal only)</t>
         </is>
       </c>
-      <c r="D57" s="3" t="inlineStr">
+      <c r="D58" s="3" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
-      <c r="E57" s="3" t="n">
+      <c r="E58" s="3" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Review fixes for Brief 16: date minimums, the ask form keeps its refusal until edited, the end date is shown as not included, persistent hints, alerts, captions; BL-193 done, BL-199; workbook
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/BEE-portal-status.xlsx
+++ b/docs/tracking/BEE-portal-status.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G150"/>
+  <dimension ref="A1:G151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -1464,49 +1464,49 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>documents/access-rights</t>
+          <t>delegations</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Access rights</t>
+          <t>Delegations</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Documents</t>
+          <t>delegations</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
+          <t>programme, director, finance, admin</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: Ask to delegate a role; Withdraw or revoke your delegation; Approve or reject a request; See what you hold and until when.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>documents/check-in-or-out</t>
+          <t>documents/access-rights</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Check in or out</t>
+          <t>Access rights</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -1538,12 +1538,12 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>documents/malware-quarantine</t>
+          <t>documents/check-in-or-out</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Malware quarantine</t>
+          <t>Check in or out</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
@@ -1575,12 +1575,12 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>documents/preview</t>
+          <t>documents/malware-quarantine</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Preview</t>
+          <t>Malware quarantine</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -1600,7 +1600,7 @@
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
@@ -1612,12 +1612,12 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>documents/repository</t>
+          <t>documents/preview</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Repository</t>
+          <t>Preview</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -1637,7 +1637,7 @@
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
@@ -1649,12 +1649,12 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>documents/retention-hold</t>
+          <t>documents/repository</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Retention hold</t>
+          <t>Repository</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -1674,7 +1674,7 @@
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
@@ -1686,12 +1686,12 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>documents/search</t>
+          <t>documents/retention-hold</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Search</t>
+          <t>Retention hold</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -1723,12 +1723,12 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>documents/version-history</t>
+          <t>documents/search</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Version history</t>
+          <t>Search</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -1760,22 +1760,22 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>enforcement/chain-of-custody</t>
+          <t>documents/version-history</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Chain of custody</t>
+          <t>Version history</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Enforcement</t>
+          <t>Documents</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary</t>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
@@ -1797,12 +1797,12 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>enforcement/challenge-test</t>
+          <t>enforcement/chain-of-custody</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Challenge test</t>
+          <t>Chain of custody</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -1822,7 +1822,7 @@
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
@@ -1834,12 +1834,12 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>enforcement/enforcement-decision</t>
+          <t>enforcement/challenge-test</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Enforcement decision</t>
+          <t>Challenge test</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -1871,12 +1871,12 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>enforcement/iame-or-sda-assignment</t>
+          <t>enforcement/enforcement-decision</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>IAME or SDA assignment</t>
+          <t>Enforcement decision</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
@@ -1896,7 +1896,7 @@
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
@@ -1908,12 +1908,12 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>enforcement/laboratory-assignment</t>
+          <t>enforcement/iame-or-sda-assignment</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Laboratory assignment</t>
+          <t>IAME or SDA assignment</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
@@ -1945,12 +1945,12 @@
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>enforcement/manufacturer-response</t>
+          <t>enforcement/laboratory-assignment</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Manufacturer response</t>
+          <t>Laboratory assignment</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
@@ -1970,7 +1970,7 @@
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
@@ -1982,12 +1982,12 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>enforcement/penalty-or-suspension</t>
+          <t>enforcement/manufacturer-response</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Penalty or suspension</t>
+          <t>Manufacturer response</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
@@ -2019,12 +2019,12 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>enforcement/result-scrutiny</t>
+          <t>enforcement/penalty-or-suspension</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>Result scrutiny</t>
+          <t>Penalty or suspension</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
@@ -2056,12 +2056,12 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>enforcement/sample-plan</t>
+          <t>enforcement/result-scrutiny</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Sample plan</t>
+          <t>Result scrutiny</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
@@ -2081,7 +2081,7 @@
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
@@ -2093,12 +2093,12 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>enforcement/sample-plan-approval</t>
+          <t>enforcement/sample-plan</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>Sample plan approval</t>
+          <t>Sample plan</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
@@ -2118,7 +2118,7 @@
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
@@ -2130,12 +2130,12 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>enforcement/sample-receipt</t>
+          <t>enforcement/sample-plan-approval</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Sample receipt</t>
+          <t>Sample plan approval</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
@@ -2167,12 +2167,12 @@
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>enforcement/show-cause</t>
+          <t>enforcement/sample-receipt</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>Show cause</t>
+          <t>Sample receipt</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -2204,12 +2204,12 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>enforcement/test-report</t>
+          <t>enforcement/show-cause</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Test report</t>
+          <t>Show cause</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
@@ -2241,12 +2241,12 @@
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>enforcement/test-result</t>
+          <t>enforcement/test-report</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>Test result</t>
+          <t>Test report</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
@@ -2278,22 +2278,22 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>finance/failed-or-duplicate-payments</t>
+          <t>enforcement/test-result</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Failed or duplicate payments</t>
+          <t>Test result</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Enforcement</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance, Auditor</t>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
@@ -2315,12 +2315,12 @@
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>finance/fee-and-penalty-ledger</t>
+          <t>finance/failed-or-duplicate-payments</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>Fee and penalty ledger</t>
+          <t>Failed or duplicate payments</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
@@ -2352,12 +2352,12 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>finance/finance-queue</t>
+          <t>finance/fee-and-penalty-ledger</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Finance queue</t>
+          <t>Fee and penalty ledger</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
@@ -2372,29 +2372,29 @@
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>Live – BEE service</t>
+          <t>Prototype (preview/sample data)</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu roles include: finance. Capabilities today: List fee-due applications; View fee and evidence; Confirm fee received.</t>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>finance/payment-reconciliation</t>
+          <t>finance/finance-queue</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>Payment reconciliation</t>
+          <t>Finance queue</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
@@ -2409,7 +2409,7 @@
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
@@ -2419,19 +2419,19 @@
       </c>
       <c r="G54" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t xml:space="preserve"> Spring menu roles include: finance. Capabilities today: List fee-due applications; View fee and evidence; Confirm fee received.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>finance/payment-verification</t>
+          <t>finance/payment-reconciliation</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>Payment verification</t>
+          <t>Payment reconciliation</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
@@ -2451,7 +2451,7 @@
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
@@ -2463,12 +2463,12 @@
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>finance/receipt</t>
+          <t>finance/payment-verification</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>Receipt</t>
+          <t>Payment verification</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>Live – BEE service</t>
+          <t>Prototype (preview/sample data)</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
@@ -2493,19 +2493,19 @@
       </c>
       <c r="G56" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Permission: fee_confirmation_correct. Capabilities today: See the fee confirmations and any correction; Propose a correction to a receipt reference or date; Approve or reject a colleague's correction; Withdraw your own correction.</t>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>finance/refund</t>
+          <t>finance/receipt</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>Refund</t>
+          <t>Receipt</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
@@ -2520,29 +2520,29 @@
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t xml:space="preserve"> Permission: fee_confirmation_correct. Capabilities today: See the fee confirmations and any correction; Propose a correction to a receipt reference or date; Approve or reject a colleague's correction; Withdraw your own correction.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>finance/security-deposit-ledger</t>
+          <t>finance/refund</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>Security deposit ledger</t>
+          <t>Refund</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
@@ -2574,12 +2574,12 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>finance/settlement</t>
+          <t>finance/security-deposit-ledger</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>Settlement</t>
+          <t>Security deposit ledger</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
@@ -2599,7 +2599,7 @@
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr">
@@ -2611,12 +2611,12 @@
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>finance/transaction-search</t>
+          <t>finance/settlement</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>Transaction search</t>
+          <t>Settlement</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
@@ -2636,7 +2636,7 @@
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G60" s="3" t="inlineStr">
@@ -2648,22 +2648,22 @@
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>helpdesk/agent-queue</t>
+          <t>finance/transaction-search</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>Agent queue</t>
+          <t>Transaction search</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>Helpdesk</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Helpdesk</t>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance, Auditor</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
@@ -2673,7 +2673,7 @@
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
@@ -2685,12 +2685,12 @@
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>helpdesk/assignment-and-escalation</t>
+          <t>helpdesk/agent-queue</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>Assignment and escalation</t>
+          <t>Agent queue</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
@@ -2722,12 +2722,12 @@
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>helpdesk/classification</t>
+          <t>helpdesk/assignment-and-escalation</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>Classification</t>
+          <t>Assignment and escalation</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
@@ -2759,12 +2759,12 @@
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>helpdesk/communication-history</t>
+          <t>helpdesk/classification</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>Communication history</t>
+          <t>Classification</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
@@ -2796,12 +2796,12 @@
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>helpdesk/feedback</t>
+          <t>helpdesk/communication-history</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>Feedback</t>
+          <t>Communication history</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
@@ -2833,12 +2833,12 @@
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>helpdesk/knowledge-base</t>
+          <t>helpdesk/feedback</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>Knowledge base</t>
+          <t>Feedback</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G66" s="3" t="inlineStr">
@@ -2870,12 +2870,12 @@
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>helpdesk/raise-ticket</t>
+          <t>helpdesk/knowledge-base</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>Raise ticket</t>
+          <t>Knowledge base</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
@@ -2907,12 +2907,12 @@
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>helpdesk/resolution-and-closure</t>
+          <t>helpdesk/raise-ticket</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>Resolution and closure</t>
+          <t>Raise ticket</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
@@ -2932,7 +2932,7 @@
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G68" s="3" t="inlineStr">
@@ -2944,12 +2944,12 @@
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>helpdesk/sla-dashboard</t>
+          <t>helpdesk/resolution-and-closure</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>SLA dashboard</t>
+          <t>Resolution and closure</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
@@ -2969,7 +2969,7 @@
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G69" s="3" t="inlineStr">
@@ -2981,12 +2981,12 @@
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>helpdesk/track-ticket</t>
+          <t>helpdesk/sla-dashboard</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>Track ticket</t>
+          <t>SLA dashboard</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
@@ -3006,7 +3006,7 @@
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G70" s="3" t="inlineStr">
@@ -3018,22 +3018,22 @@
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>identity/access-review</t>
+          <t>helpdesk/track-ticket</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>Access review</t>
+          <t>Track ticket</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>Helpdesk</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary</t>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Helpdesk</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
@@ -3055,12 +3055,12 @@
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>identity/delegation</t>
+          <t>identity/access-review</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>Delegation</t>
+          <t>Access review</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
@@ -3092,12 +3092,12 @@
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>identity/login-and-mfa</t>
+          <t>identity/delegation</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>Login and MFA</t>
+          <t>Delegation</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
@@ -3117,7 +3117,7 @@
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>retire</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G73" s="3" t="inlineStr">
@@ -3129,12 +3129,12 @@
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>identity/organisation-users</t>
+          <t>identity/login-and-mfa</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>Organisation users</t>
+          <t>Login and MFA</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
@@ -3154,7 +3154,7 @@
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>retire</t>
         </is>
       </c>
       <c r="G74" s="3" t="inlineStr">
@@ -3166,12 +3166,12 @@
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>identity/role-assignment</t>
+          <t>identity/organisation-users</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>Role assignment</t>
+          <t>Organisation users</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
@@ -3191,7 +3191,7 @@
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G75" s="3" t="inlineStr">
@@ -3203,12 +3203,12 @@
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>identity/user-profile</t>
+          <t>identity/role-assignment</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>User profile</t>
+          <t>Role assignment</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
@@ -3240,22 +3240,22 @@
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>mis-ai/chatbot-review</t>
+          <t>identity/user-profile</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>Chatbot review</t>
+          <t>User profile</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>MIS &amp; AI</t>
+          <t>Identity</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance, Auditor</t>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary</t>
         </is>
       </c>
       <c r="E77" s="3" t="inlineStr">
@@ -3277,12 +3277,12 @@
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>mis-ai/data-quality</t>
+          <t>mis-ai/chatbot-review</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>Data quality</t>
+          <t>Chatbot review</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
@@ -3302,7 +3302,7 @@
       </c>
       <c r="F78" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G78" s="3" t="inlineStr">
@@ -3314,12 +3314,12 @@
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>mis-ai/enforcement-dashboard</t>
+          <t>mis-ai/data-quality</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>Enforcement dashboard</t>
+          <t>Data quality</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
@@ -3351,12 +3351,12 @@
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>mis-ai/executive-mis</t>
+          <t>mis-ai/enforcement-dashboard</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>Executive MIS</t>
+          <t>Enforcement dashboard</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
@@ -3388,12 +3388,12 @@
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>mis-ai/extraction-review</t>
+          <t>mis-ai/executive-mis</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>Extraction review</t>
+          <t>Executive MIS</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
@@ -3413,7 +3413,7 @@
       </c>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G81" s="3" t="inlineStr">
@@ -3425,12 +3425,12 @@
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>mis-ai/helpdesk-dashboard</t>
+          <t>mis-ai/extraction-review</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>Helpdesk dashboard</t>
+          <t>Extraction review</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
@@ -3462,12 +3462,12 @@
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>mis-ai/model-dashboard</t>
+          <t>mis-ai/helpdesk-dashboard</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>Model dashboard</t>
+          <t>Helpdesk dashboard</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
@@ -3499,12 +3499,12 @@
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>mis-ai/model-monitoring</t>
+          <t>mis-ai/model-dashboard</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>Model monitoring</t>
+          <t>Model dashboard</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
@@ -3524,7 +3524,7 @@
       </c>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G84" s="3" t="inlineStr">
@@ -3536,12 +3536,12 @@
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>mis-ai/production-and-fee-dashboard</t>
+          <t>mis-ai/model-monitoring</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>Production and fee dashboard</t>
+          <t>Model monitoring</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
@@ -3561,7 +3561,7 @@
       </c>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G85" s="3" t="inlineStr">
@@ -3573,12 +3573,12 @@
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>mis-ai/production-anomaly</t>
+          <t>mis-ai/production-and-fee-dashboard</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>Production anomaly</t>
+          <t>Production and fee dashboard</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
@@ -3610,12 +3610,12 @@
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>mis-ai/rating-trends</t>
+          <t>mis-ai/production-anomaly</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>Rating trends</t>
+          <t>Production anomaly</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
@@ -3647,12 +3647,12 @@
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>mis-ai/registration-dashboard</t>
+          <t>mis-ai/rating-trends</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>Registration dashboard</t>
+          <t>Rating trends</t>
         </is>
       </c>
       <c r="C88" s="3" t="inlineStr">
@@ -3672,7 +3672,7 @@
       </c>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G88" s="3" t="inlineStr">
@@ -3684,12 +3684,12 @@
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>mis-ai/report-builder</t>
+          <t>mis-ai/registration-dashboard</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>Report builder</t>
+          <t>Registration dashboard</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
@@ -3721,12 +3721,12 @@
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>mis-ai/risk-scoring</t>
+          <t>mis-ai/report-builder</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>Risk scoring</t>
+          <t>Report builder</t>
         </is>
       </c>
       <c r="C90" s="3" t="inlineStr">
@@ -3746,7 +3746,7 @@
       </c>
       <c r="F90" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G90" s="3" t="inlineStr">
@@ -3758,12 +3758,12 @@
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>mis-ai/scheduled-reports</t>
+          <t>mis-ai/risk-scoring</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>Scheduled reports</t>
+          <t>Risk scoring</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
@@ -3795,22 +3795,22 @@
     <row r="92">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t>model-label/approval-letter</t>
+          <t>mis-ai/scheduled-reports</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>Approval letter</t>
+          <t>Scheduled reports</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>Model &amp; Label</t>
+          <t>MIS &amp; AI</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance, Helpdesk</t>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance, Auditor</t>
         </is>
       </c>
       <c r="E92" s="3" t="inlineStr">
@@ -3832,12 +3832,12 @@
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>model-label/approval-note</t>
+          <t>model-label/approval-letter</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>Approval note</t>
+          <t>Approval letter</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
@@ -3869,12 +3869,12 @@
     <row r="94">
       <c r="A94" s="3" t="inlineStr">
         <is>
-          <t>model-label/bee-scrutiny</t>
+          <t>model-label/approval-note</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>BEE scrutiny</t>
+          <t>Approval note</t>
         </is>
       </c>
       <c r="C94" s="3" t="inlineStr">
@@ -3889,29 +3889,29 @@
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>Live – BEE service</t>
+          <t>Prototype (preview/sample data)</t>
         </is>
       </c>
       <c r="F94" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G94" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu roles include: reviewer. Capabilities today: List assigned applications; View evidence and test reports; Forward to rating; Return to the applicant; Reject permanently; See the earlier steps and notes.</t>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>model-label/director-approval</t>
+          <t>model-label/bee-scrutiny</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>Director approval</t>
+          <t>BEE scrutiny</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
@@ -3936,19 +3936,19 @@
       </c>
       <c r="G95" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu roles include: director, secretary. Capabilities today: List applications awaiting your decision; View the rating, evidence and test reports; Recommend approval (Director); Give final approval (Secretary); Return to the applicant; Reject permanently; See the earlier steps and notes.</t>
+          <t xml:space="preserve"> Spring menu roles include: reviewer. Capabilities today: List assigned applications; View evidence and test reports; Forward to rating; Return to the applicant; Reject permanently; See the earlier steps and notes.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t>model-label/family-models</t>
+          <t>model-label/director-approval</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>Family models</t>
+          <t>Director approval</t>
         </is>
       </c>
       <c r="C96" s="3" t="inlineStr">
@@ -3963,29 +3963,29 @@
       </c>
       <c r="E96" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F96" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G96" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t xml:space="preserve"> Spring menu roles include: director, secretary. Capabilities today: List applications awaiting your decision; View the rating, evidence and test reports; Recommend approval (Director); Give final approval (Secretary); Return to the applicant; Reject permanently; See the earlier steps and notes.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>model-label/iame-scrutiny</t>
+          <t>model-label/family-models</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>IAME scrutiny</t>
+          <t>Family models</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
@@ -4000,29 +4000,29 @@
       </c>
       <c r="E97" s="3" t="inlineStr">
         <is>
-          <t>Live – BEE service</t>
+          <t>Prototype (preview/sample data)</t>
         </is>
       </c>
       <c r="F97" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G97" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu roles include: iame. Capabilities today: List assigned applications; View evidence and test reports; Record finding and forward; Return to the applicant; Reject permanently; See the earlier steps and notes.</t>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="3" t="inlineStr">
         <is>
-          <t>model-label/lab-accreditation</t>
+          <t>model-label/iame-scrutiny</t>
         </is>
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>Lab accreditation</t>
+          <t>IAME scrutiny</t>
         </is>
       </c>
       <c r="C98" s="3" t="inlineStr">
@@ -4037,29 +4037,29 @@
       </c>
       <c r="E98" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F98" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G98" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t xml:space="preserve"> Spring menu roles include: iame. Capabilities today: List assigned applications; View evidence and test reports; Record finding and forward; Return to the applicant; Reject permanently; See the earlier steps and notes.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t>model-label/label-details</t>
+          <t>model-label/lab-accreditation</t>
         </is>
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>Label details</t>
+          <t>Lab accreditation</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
@@ -4091,12 +4091,12 @@
     <row r="100">
       <c r="A100" s="3" t="inlineStr">
         <is>
-          <t>model-label/label-preview</t>
+          <t>model-label/label-details</t>
         </is>
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>Label preview</t>
+          <t>Label details</t>
         </is>
       </c>
       <c r="C100" s="3" t="inlineStr">
@@ -4111,29 +4111,29 @@
       </c>
       <c r="E100" s="3" t="inlineStr">
         <is>
-          <t>Live – BEE service</t>
+          <t>Prototype (preview/sample data)</t>
         </is>
       </c>
       <c r="F100" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G100" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu roles include: manufacturer, agency. Capabilities today: List your approved applications; Open the printable certificate and star label; Print or save as PDF; A QR code that opens the public verification page.</t>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>model-label/model-dashboard</t>
+          <t>model-label/label-preview</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>Model dashboard</t>
+          <t>Label preview</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
@@ -4158,19 +4158,19 @@
       </c>
       <c r="G101" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu roles include: manufacturer, agency. Capabilities today: List; View detail; Edit draft; Submit draft; See why it was returned; Edit and resubmit; See why it was rejected; See the history.</t>
+          <t xml:space="preserve"> Spring menu roles include: manufacturer, agency. Capabilities today: List your approved applications; Open the printable certificate and star label; Print or save as PDF; A QR code that opens the public verification page.</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="3" t="inlineStr">
         <is>
-          <t>model-label/model-documents</t>
+          <t>model-label/model-dashboard</t>
         </is>
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>Model documents</t>
+          <t>Model dashboard</t>
         </is>
       </c>
       <c r="C102" s="3" t="inlineStr">
@@ -4185,29 +4185,29 @@
       </c>
       <c r="E102" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F102" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G102" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t xml:space="preserve"> Spring menu roles include: manufacturer, agency. Capabilities today: List; View detail; Edit draft; Submit draft; See why it was returned; Edit and resubmit; See why it was rejected; See the history.</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>model-label/model-payment</t>
+          <t>model-label/model-documents</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>Model payment</t>
+          <t>Model documents</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
@@ -4227,7 +4227,7 @@
       </c>
       <c r="F103" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G103" s="3" t="inlineStr">
@@ -4239,12 +4239,12 @@
     <row r="104">
       <c r="A104" s="3" t="inlineStr">
         <is>
-          <t>model-label/new-model-application</t>
+          <t>model-label/model-payment</t>
         </is>
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>New model application</t>
+          <t>Model payment</t>
         </is>
       </c>
       <c r="C104" s="3" t="inlineStr">
@@ -4259,7 +4259,7 @@
       </c>
       <c r="E104" s="3" t="inlineStr">
         <is>
-          <t>Live – BEE service</t>
+          <t>Prototype (preview/sample data)</t>
         </is>
       </c>
       <c r="F104" s="3" t="inlineStr">
@@ -4269,19 +4269,19 @@
       </c>
       <c r="G104" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu roles include: manufacturer, agency. Capabilities today: Create draft; Edit draft; Upload test reports; Submit draft; Edit and resubmit a returned application.</t>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
         <is>
-          <t>model-label/notifications</t>
+          <t>model-label/new-model-application</t>
         </is>
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>New model application</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
@@ -4306,19 +4306,19 @@
       </c>
       <c r="G105" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu roles include: manufacturer, agency. Capabilities today: See updates about your applications; Open the screen to act; Mark one or all as read.</t>
+          <t xml:space="preserve"> Spring menu roles include: manufacturer, agency. Capabilities today: Create draft; Edit draft; Upload test reports; Submit draft; Edit and resubmit a returned application.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="3" t="inlineStr">
         <is>
-          <t>model-label/performance-parameters</t>
+          <t>model-label/notifications</t>
         </is>
       </c>
       <c r="B106" s="3" t="inlineStr">
         <is>
-          <t>Performance parameters</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="C106" s="3" t="inlineStr">
@@ -4333,29 +4333,29 @@
       </c>
       <c r="E106" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F106" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G106" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t xml:space="preserve"> Spring menu roles include: manufacturer, agency. Capabilities today: See updates about your applications; Open the screen to act; Mark one or all as read.</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
         <is>
-          <t>model-label/rating-calculation</t>
+          <t>model-label/performance-parameters</t>
         </is>
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>Rating calculation</t>
+          <t>Performance parameters</t>
         </is>
       </c>
       <c r="C107" s="3" t="inlineStr">
@@ -4370,29 +4370,29 @@
       </c>
       <c r="E107" s="3" t="inlineStr">
         <is>
-          <t>Live – BEE service</t>
+          <t>Prototype (preview/sample data)</t>
         </is>
       </c>
       <c r="F107" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G107" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu roles include: programme. Capabilities today: List applications awaiting a rating; View evidence and test reports; Compute and record a provisional local rating; Reject permanently; See the earlier steps and notes.</t>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
         <is>
-          <t>model-label/renewal-or-degradation</t>
+          <t>model-label/rating-calculation</t>
         </is>
       </c>
       <c r="B108" s="3" t="inlineStr">
         <is>
-          <t>Renewal or degradation</t>
+          <t>Rating calculation</t>
         </is>
       </c>
       <c r="C108" s="3" t="inlineStr">
@@ -4407,7 +4407,7 @@
       </c>
       <c r="E108" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F108" s="3" t="inlineStr">
@@ -4417,19 +4417,19 @@
       </c>
       <c r="G108" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t xml:space="preserve"> Spring menu roles include: programme. Capabilities today: List applications awaiting a rating; View evidence and test reports; Compute and record a provisional local rating; Reject permanently; See the earlier steps and notes.</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
         <is>
-          <t>model-label/secretary-approval</t>
+          <t>model-label/renewal-or-degradation</t>
         </is>
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>Secretary approval</t>
+          <t>Renewal or degradation</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
@@ -4449,7 +4449,7 @@
       </c>
       <c r="F109" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G109" s="3" t="inlineStr">
@@ -4461,12 +4461,12 @@
     <row r="110">
       <c r="A110" s="3" t="inlineStr">
         <is>
-          <t>model-label/test-reports</t>
+          <t>model-label/secretary-approval</t>
         </is>
       </c>
       <c r="B110" s="3" t="inlineStr">
         <is>
-          <t>Test reports</t>
+          <t>Secretary approval</t>
         </is>
       </c>
       <c r="C110" s="3" t="inlineStr">
@@ -4498,17 +4498,17 @@
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t>production/bulk-upload</t>
+          <t>model-label/test-reports</t>
         </is>
       </c>
       <c r="B111" s="3" t="inlineStr">
         <is>
-          <t>Bulk upload</t>
+          <t>Test reports</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Model &amp; Label</t>
         </is>
       </c>
       <c r="D111" s="3" t="inlineStr">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="F111" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G111" s="3" t="inlineStr">
@@ -4535,12 +4535,12 @@
     <row r="112">
       <c r="A112" s="3" t="inlineStr">
         <is>
-          <t>production/ca-evidence</t>
+          <t>production/bulk-upload</t>
         </is>
       </c>
       <c r="B112" s="3" t="inlineStr">
         <is>
-          <t>CA evidence</t>
+          <t>Bulk upload</t>
         </is>
       </c>
       <c r="C112" s="3" t="inlineStr">
@@ -4560,7 +4560,7 @@
       </c>
       <c r="F112" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G112" s="3" t="inlineStr">
@@ -4572,12 +4572,12 @@
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
         <is>
-          <t>production/compliance-exceptions</t>
+          <t>production/ca-evidence</t>
         </is>
       </c>
       <c r="B113" s="3" t="inlineStr">
         <is>
-          <t>Compliance exceptions</t>
+          <t>CA evidence</t>
         </is>
       </c>
       <c r="C113" s="3" t="inlineStr">
@@ -4597,7 +4597,7 @@
       </c>
       <c r="F113" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G113" s="3" t="inlineStr">
@@ -4609,12 +4609,12 @@
     <row r="114">
       <c r="A114" s="3" t="inlineStr">
         <is>
-          <t>production/correction-request</t>
+          <t>production/compliance-exceptions</t>
         </is>
       </c>
       <c r="B114" s="3" t="inlineStr">
         <is>
-          <t>Correction request</t>
+          <t>Compliance exceptions</t>
         </is>
       </c>
       <c r="C114" s="3" t="inlineStr">
@@ -4634,7 +4634,7 @@
       </c>
       <c r="F114" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G114" s="3" t="inlineStr">
@@ -4646,12 +4646,12 @@
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
         <is>
-          <t>production/label-fee</t>
+          <t>production/correction-request</t>
         </is>
       </c>
       <c r="B115" s="3" t="inlineStr">
         <is>
-          <t>Label fee</t>
+          <t>Correction request</t>
         </is>
       </c>
       <c r="C115" s="3" t="inlineStr">
@@ -4683,12 +4683,12 @@
     <row r="116">
       <c r="A116" s="3" t="inlineStr">
         <is>
-          <t>production/production-payment</t>
+          <t>production/label-fee</t>
         </is>
       </c>
       <c r="B116" s="3" t="inlineStr">
         <is>
-          <t>Production payment</t>
+          <t>Label fee</t>
         </is>
       </c>
       <c r="C116" s="3" t="inlineStr">
@@ -4720,12 +4720,12 @@
     <row r="117">
       <c r="A117" s="3" t="inlineStr">
         <is>
-          <t>production/quarterly-submission</t>
+          <t>production/production-payment</t>
         </is>
       </c>
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t>Quarterly submission</t>
+          <t>Production payment</t>
         </is>
       </c>
       <c r="C117" s="3" t="inlineStr">
@@ -4745,7 +4745,7 @@
       </c>
       <c r="F117" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G117" s="3" t="inlineStr">
@@ -4757,12 +4757,12 @@
     <row r="118">
       <c r="A118" s="3" t="inlineStr">
         <is>
-          <t>production/reconciliation</t>
+          <t>production/quarterly-submission</t>
         </is>
       </c>
       <c r="B118" s="3" t="inlineStr">
         <is>
-          <t>Reconciliation</t>
+          <t>Quarterly submission</t>
         </is>
       </c>
       <c r="C118" s="3" t="inlineStr">
@@ -4794,12 +4794,12 @@
     <row r="119">
       <c r="A119" s="3" t="inlineStr">
         <is>
-          <t>production/validation-results</t>
+          <t>production/reconciliation</t>
         </is>
       </c>
       <c r="B119" s="3" t="inlineStr">
         <is>
-          <t>Validation results</t>
+          <t>Reconciliation</t>
         </is>
       </c>
       <c r="C119" s="3" t="inlineStr">
@@ -4819,7 +4819,7 @@
       </c>
       <c r="F119" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G119" s="3" t="inlineStr">
@@ -4831,22 +4831,22 @@
     <row r="120">
       <c r="A120" s="3" t="inlineStr">
         <is>
-          <t>qr-verification/batch-file-download</t>
+          <t>production/validation-results</t>
         </is>
       </c>
       <c r="B120" s="3" t="inlineStr">
         <is>
-          <t>Batch file download</t>
+          <t>Validation results</t>
         </is>
       </c>
       <c r="C120" s="3" t="inlineStr">
         <is>
-          <t>QR &amp; Verification</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="D120" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Helpdesk</t>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance, Helpdesk</t>
         </is>
       </c>
       <c r="E120" s="3" t="inlineStr">
@@ -4868,12 +4868,12 @@
     <row r="121">
       <c r="A121" s="3" t="inlineStr">
         <is>
-          <t>qr-verification/certificate-verification</t>
+          <t>qr-verification/batch-file-download</t>
         </is>
       </c>
       <c r="B121" s="3" t="inlineStr">
         <is>
-          <t>Certificate verification</t>
+          <t>Batch file download</t>
         </is>
       </c>
       <c r="C121" s="3" t="inlineStr">
@@ -4905,12 +4905,12 @@
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>qr-verification/duplicate-exceptions</t>
+          <t>qr-verification/certificate-verification</t>
         </is>
       </c>
       <c r="B122" s="3" t="inlineStr">
         <is>
-          <t>Duplicate exceptions</t>
+          <t>Certificate verification</t>
         </is>
       </c>
       <c r="C122" s="3" t="inlineStr">
@@ -4942,12 +4942,12 @@
     <row r="123">
       <c r="A123" s="3" t="inlineStr">
         <is>
-          <t>qr-verification/public-verification</t>
+          <t>qr-verification/duplicate-exceptions</t>
         </is>
       </c>
       <c r="B123" s="3" t="inlineStr">
         <is>
-          <t>Public verification</t>
+          <t>Duplicate exceptions</t>
         </is>
       </c>
       <c r="C123" s="3" t="inlineStr">
@@ -4967,7 +4967,7 @@
       </c>
       <c r="F123" s="3" t="inlineStr">
         <is>
-          <t>retire</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G123" s="3" t="inlineStr">
@@ -4979,12 +4979,12 @@
     <row r="124">
       <c r="A124" s="3" t="inlineStr">
         <is>
-          <t>qr-verification/qr-batch-request</t>
+          <t>qr-verification/public-verification</t>
         </is>
       </c>
       <c r="B124" s="3" t="inlineStr">
         <is>
-          <t>QR batch request</t>
+          <t>Public verification</t>
         </is>
       </c>
       <c r="C124" s="3" t="inlineStr">
@@ -5004,7 +5004,7 @@
       </c>
       <c r="F124" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>retire</t>
         </is>
       </c>
       <c r="G124" s="3" t="inlineStr">
@@ -5016,12 +5016,12 @@
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
         <is>
-          <t>qr-verification/qr-batch-status</t>
+          <t>qr-verification/qr-batch-request</t>
         </is>
       </c>
       <c r="B125" s="3" t="inlineStr">
         <is>
-          <t>QR batch status</t>
+          <t>QR batch request</t>
         </is>
       </c>
       <c r="C125" s="3" t="inlineStr">
@@ -5053,12 +5053,12 @@
     <row r="126">
       <c r="A126" s="3" t="inlineStr">
         <is>
-          <t>qr-verification/qr-download</t>
+          <t>qr-verification/qr-batch-status</t>
         </is>
       </c>
       <c r="B126" s="3" t="inlineStr">
         <is>
-          <t>QR download</t>
+          <t>QR batch status</t>
         </is>
       </c>
       <c r="C126" s="3" t="inlineStr">
@@ -5090,12 +5090,12 @@
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
         <is>
-          <t>qr-verification/serial-upload</t>
+          <t>qr-verification/qr-download</t>
         </is>
       </c>
       <c r="B127" s="3" t="inlineStr">
         <is>
-          <t>Serial upload</t>
+          <t>QR download</t>
         </is>
       </c>
       <c r="C127" s="3" t="inlineStr">
@@ -5127,49 +5127,49 @@
     <row r="128">
       <c r="A128" s="3" t="inlineStr">
         <is>
-          <t>registrations/new</t>
+          <t>qr-verification/serial-upload</t>
         </is>
       </c>
       <c r="B128" s="3" t="inlineStr">
         <is>
-          <t>New registration request</t>
+          <t>Serial upload</t>
         </is>
       </c>
       <c r="C128" s="3" t="inlineStr">
         <is>
-          <t>registrations</t>
+          <t>QR &amp; Verification</t>
         </is>
       </c>
       <c r="D128" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Helpdesk</t>
         </is>
       </c>
       <c r="E128" s="3" t="inlineStr">
         <is>
-          <t>Live – BEE service</t>
+          <t>Prototype (preview/sample data)</t>
         </is>
       </c>
       <c r="F128" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G128" s="3" t="inlineStr">
         <is>
-          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: File a brand request; Ask to act for a brand; Save a draft.</t>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="3" t="inlineStr">
         <is>
-          <t>registrations/register</t>
+          <t>registrations/new</t>
         </is>
       </c>
       <c r="B129" s="3" t="inlineStr">
         <is>
-          <t>Register</t>
+          <t>New registration request</t>
         </is>
       </c>
       <c r="C129" s="3" t="inlineStr">
@@ -5179,7 +5179,7 @@
       </c>
       <c r="D129" s="3" t="inlineStr">
         <is>
-          <t>programme, director</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E129" s="3" t="inlineStr">
@@ -5194,19 +5194,19 @@
       </c>
       <c r="G129" s="3" t="inlineStr">
         <is>
-          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: See registered brands and authorisations; Propose a closure or revocation; Approve, reject or withdraw a proposal; Read the history.</t>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: File a brand request; Ask to act for a brand; Save a draft.</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="3" t="inlineStr">
         <is>
-          <t>registrations/request</t>
+          <t>registrations/register</t>
         </is>
       </c>
       <c r="B130" s="3" t="inlineStr">
         <is>
-          <t>Registration request</t>
+          <t>Register</t>
         </is>
       </c>
       <c r="C130" s="3" t="inlineStr">
@@ -5216,7 +5216,7 @@
       </c>
       <c r="D130" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>programme, director</t>
         </is>
       </c>
       <c r="E130" s="3" t="inlineStr">
@@ -5231,19 +5231,19 @@
       </c>
       <c r="G130" s="3" t="inlineStr">
         <is>
-          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: See the request; Upload the trade licence; See the fee and submit; Follow the request until Programme review; Recommend or return; Approve, return or reject; See why it was returned and resubmit.</t>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: See registered brands and authorisations; Propose a closure or revocation; Approve, reject or withdraw a proposal; Read the history.</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="3" t="inlineStr">
         <is>
-          <t>registrations/requests</t>
+          <t>registrations/request</t>
         </is>
       </c>
       <c r="B131" s="3" t="inlineStr">
         <is>
-          <t>Registration requests</t>
+          <t>Registration request</t>
         </is>
       </c>
       <c r="C131" s="3" t="inlineStr">
@@ -5253,7 +5253,7 @@
       </c>
       <c r="D131" s="3" t="inlineStr">
         <is>
-          <t>manufacturer, agency</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E131" s="3" t="inlineStr">
@@ -5268,19 +5268,19 @@
       </c>
       <c r="G131" s="3" t="inlineStr">
         <is>
-          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: List your registration requests; Open a request; Start a new request.</t>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: See the request; Upload the trade licence; See the fee and submit; Follow the request until Programme review; Recommend or return; Approve, return or reject; See why it was returned and resubmit.</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="3" t="inlineStr">
         <is>
-          <t>registrations/reviews</t>
+          <t>registrations/requests</t>
         </is>
       </c>
       <c r="B132" s="3" t="inlineStr">
         <is>
-          <t>Registration reviews</t>
+          <t>Registration requests</t>
         </is>
       </c>
       <c r="C132" s="3" t="inlineStr">
@@ -5290,7 +5290,7 @@
       </c>
       <c r="D132" s="3" t="inlineStr">
         <is>
-          <t>programme, director</t>
+          <t>manufacturer, agency</t>
         </is>
       </c>
       <c r="E132" s="3" t="inlineStr">
@@ -5305,34 +5305,34 @@
       </c>
       <c r="G132" s="3" t="inlineStr">
         <is>
-          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: List requests waiting for you; Recommend or return; Approve, return or reject; Read the trail.</t>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: List your registration requests; Open a request; Start a new request.</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/brand-withdrawal</t>
+          <t>registrations/reviews</t>
         </is>
       </c>
       <c r="B133" s="3" t="inlineStr">
         <is>
-          <t>Brand withdrawal</t>
+          <t>Registration reviews</t>
         </is>
       </c>
       <c r="C133" s="3" t="inlineStr">
         <is>
-          <t>Withdrawal</t>
+          <t>registrations</t>
         </is>
       </c>
       <c r="D133" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance</t>
+          <t>programme, director</t>
         </is>
       </c>
       <c r="E133" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F133" s="3" t="inlineStr">
@@ -5342,19 +5342,19 @@
       </c>
       <c r="G133" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: List requests waiting for you; Recommend or return; Approve, return or reject; Read the trail.</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/deposit-release</t>
+          <t>withdrawal/brand-withdrawal</t>
         </is>
       </c>
       <c r="B134" s="3" t="inlineStr">
         <is>
-          <t>Deposit release</t>
+          <t>Brand withdrawal</t>
         </is>
       </c>
       <c r="C134" s="3" t="inlineStr">
@@ -5374,7 +5374,7 @@
       </c>
       <c r="F134" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G134" s="3" t="inlineStr">
@@ -5386,12 +5386,12 @@
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/dues-verification</t>
+          <t>withdrawal/deposit-release</t>
         </is>
       </c>
       <c r="B135" s="3" t="inlineStr">
         <is>
-          <t>Dues verification</t>
+          <t>Deposit release</t>
         </is>
       </c>
       <c r="C135" s="3" t="inlineStr">
@@ -5423,12 +5423,12 @@
     <row r="136">
       <c r="A136" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/model-withdrawal</t>
+          <t>withdrawal/dues-verification</t>
         </is>
       </c>
       <c r="B136" s="3" t="inlineStr">
         <is>
-          <t>Model withdrawal</t>
+          <t>Dues verification</t>
         </is>
       </c>
       <c r="C136" s="3" t="inlineStr">
@@ -5460,12 +5460,12 @@
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/revocation-initiation</t>
+          <t>withdrawal/model-withdrawal</t>
         </is>
       </c>
       <c r="B137" s="3" t="inlineStr">
         <is>
-          <t>Revocation initiation</t>
+          <t>Model withdrawal</t>
         </is>
       </c>
       <c r="C137" s="3" t="inlineStr">
@@ -5497,12 +5497,12 @@
     <row r="138">
       <c r="A138" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/withdrawal-approval</t>
+          <t>withdrawal/revocation-initiation</t>
         </is>
       </c>
       <c r="B138" s="3" t="inlineStr">
         <is>
-          <t>Withdrawal approval</t>
+          <t>Revocation initiation</t>
         </is>
       </c>
       <c r="C138" s="3" t="inlineStr">
@@ -5534,12 +5534,12 @@
     <row r="139">
       <c r="A139" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/withdrawal-letter</t>
+          <t>withdrawal/withdrawal-approval</t>
         </is>
       </c>
       <c r="B139" s="3" t="inlineStr">
         <is>
-          <t>Withdrawal letter</t>
+          <t>Withdrawal approval</t>
         </is>
       </c>
       <c r="C139" s="3" t="inlineStr">
@@ -5571,12 +5571,12 @@
     <row r="140">
       <c r="A140" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/withdrawal-scrutiny</t>
+          <t>withdrawal/withdrawal-letter</t>
         </is>
       </c>
       <c r="B140" s="3" t="inlineStr">
         <is>
-          <t>Withdrawal scrutiny</t>
+          <t>Withdrawal letter</t>
         </is>
       </c>
       <c r="C140" s="3" t="inlineStr">
@@ -5608,27 +5608,27 @@
     <row r="141">
       <c r="A141" s="3" t="inlineStr">
         <is>
-          <t>workflow/application-review</t>
+          <t>withdrawal/withdrawal-scrutiny</t>
         </is>
       </c>
       <c r="B141" s="3" t="inlineStr">
         <is>
-          <t>Application review</t>
+          <t>Withdrawal scrutiny</t>
         </is>
       </c>
       <c r="C141" s="3" t="inlineStr">
         <is>
-          <t>Workflow</t>
+          <t>Withdrawal</t>
         </is>
       </c>
       <c r="D141" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance</t>
         </is>
       </c>
       <c r="E141" s="3" t="inlineStr">
         <is>
-          <t>Live – BEE service</t>
+          <t>Prototype (preview/sample data)</t>
         </is>
       </c>
       <c r="F141" s="3" t="inlineStr">
@@ -5638,19 +5638,19 @@
       </c>
       <c r="G141" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu by role or permission. Capabilities today: List the applications in progress; Link to your next action; Link to the history.</t>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="3" t="inlineStr">
         <is>
-          <t>workflow/approval-note</t>
+          <t>workflow/application-review</t>
         </is>
       </c>
       <c r="B142" s="3" t="inlineStr">
         <is>
-          <t>Approval note</t>
+          <t>Application review</t>
         </is>
       </c>
       <c r="C142" s="3" t="inlineStr">
@@ -5665,7 +5665,7 @@
       </c>
       <c r="E142" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F142" s="3" t="inlineStr">
@@ -5675,19 +5675,19 @@
       </c>
       <c r="G142" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t xml:space="preserve"> Spring menu by role or permission. Capabilities today: List the applications in progress; Link to your next action; Link to the history.</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="3" t="inlineStr">
         <is>
-          <t>workflow/checklist</t>
+          <t>workflow/approval-note</t>
         </is>
       </c>
       <c r="B143" s="3" t="inlineStr">
         <is>
-          <t>Checklist</t>
+          <t>Approval note</t>
         </is>
       </c>
       <c r="C143" s="3" t="inlineStr">
@@ -5719,12 +5719,12 @@
     <row r="144">
       <c r="A144" s="3" t="inlineStr">
         <is>
-          <t>workflow/clarification-and-return</t>
+          <t>workflow/checklist</t>
         </is>
       </c>
       <c r="B144" s="3" t="inlineStr">
         <is>
-          <t>Clarification and return</t>
+          <t>Checklist</t>
         </is>
       </c>
       <c r="C144" s="3" t="inlineStr">
@@ -5756,12 +5756,12 @@
     <row r="145">
       <c r="A145" s="3" t="inlineStr">
         <is>
-          <t>workflow/delegation-and-reassignment</t>
+          <t>workflow/clarification-and-return</t>
         </is>
       </c>
       <c r="B145" s="3" t="inlineStr">
         <is>
-          <t>Delegation and reassignment</t>
+          <t>Clarification and return</t>
         </is>
       </c>
       <c r="C145" s="3" t="inlineStr">
@@ -5793,12 +5793,12 @@
     <row r="146">
       <c r="A146" s="3" t="inlineStr">
         <is>
-          <t>workflow/escalation-dashboard</t>
+          <t>workflow/delegation-and-reassignment</t>
         </is>
       </c>
       <c r="B146" s="3" t="inlineStr">
         <is>
-          <t>Escalation dashboard</t>
+          <t>Delegation and reassignment</t>
         </is>
       </c>
       <c r="C146" s="3" t="inlineStr">
@@ -5813,39 +5813,39 @@
       </c>
       <c r="E146" s="3" t="inlineStr">
         <is>
-          <t>Live – BEE service</t>
+          <t>Prototype (preview/sample data)</t>
         </is>
       </c>
       <c r="F146" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G146" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu by role or permission. Capabilities today: Count the applications waiting at each stage (no time limits are set yet).</t>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="3" t="inlineStr">
         <is>
-          <t>workflow/my-approvals</t>
+          <t>workflow/escalation-dashboard</t>
         </is>
       </c>
       <c r="B147" s="3" t="inlineStr">
         <is>
-          <t>My approvals</t>
+          <t>Escalation dashboard</t>
         </is>
       </c>
       <c r="C147" s="3" t="inlineStr">
         <is>
-          <t>workflow</t>
+          <t>Workflow</t>
         </is>
       </c>
       <c r="D147" s="3" t="inlineStr">
         <is>
-          <t>director, secretary</t>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
         </is>
       </c>
       <c r="E147" s="3" t="inlineStr">
@@ -5860,29 +5860,29 @@
       </c>
       <c r="G147" s="3" t="inlineStr">
         <is>
-          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: List the applications waiting for your decision; Open the approval screen.</t>
+          <t xml:space="preserve"> Spring menu by role or permission. Capabilities today: Count the applications waiting at each stage (no time limits are set yet).</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="3" t="inlineStr">
         <is>
-          <t>workflow/personal-inbox</t>
+          <t>workflow/my-approvals</t>
         </is>
       </c>
       <c r="B148" s="3" t="inlineStr">
         <is>
-          <t>Personal inbox</t>
+          <t>My approvals</t>
         </is>
       </c>
       <c r="C148" s="3" t="inlineStr">
         <is>
-          <t>Workflow</t>
+          <t>workflow</t>
         </is>
       </c>
       <c r="D148" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
+          <t>director, secretary</t>
         </is>
       </c>
       <c r="E148" s="3" t="inlineStr">
@@ -5897,19 +5897,19 @@
       </c>
       <c r="G148" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu roles include: manufacturer, agency, finance, iame, reviewer, programme, director, secretary. Capabilities today: List the applications waiting for you; Open the screen where each is done.</t>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: List the applications waiting for your decision; Open the approval screen.</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="3" t="inlineStr">
         <is>
-          <t>workflow/team-queue</t>
+          <t>workflow/personal-inbox</t>
         </is>
       </c>
       <c r="B149" s="3" t="inlineStr">
         <is>
-          <t>Team queue</t>
+          <t>Personal inbox</t>
         </is>
       </c>
       <c r="C149" s="3" t="inlineStr">
@@ -5924,52 +5924,89 @@
       </c>
       <c r="E149" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F149" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G149" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t xml:space="preserve"> Spring menu roles include: manufacturer, agency, finance, iame, reviewer, programme, director, secretary. Capabilities today: List the applications waiting for you; Open the screen where each is done.</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="3" t="inlineStr">
         <is>
+          <t>workflow/team-queue</t>
+        </is>
+      </c>
+      <c r="B150" s="3" t="inlineStr">
+        <is>
+          <t>Team queue</t>
+        </is>
+      </c>
+      <c r="C150" s="3" t="inlineStr">
+        <is>
+          <t>Workflow</t>
+        </is>
+      </c>
+      <c r="D150" s="3" t="inlineStr">
+        <is>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
+        </is>
+      </c>
+      <c r="E150" s="3" t="inlineStr">
+        <is>
+          <t>Prototype (preview/sample data)</t>
+        </is>
+      </c>
+      <c r="F150" s="3" t="inlineStr">
+        <is>
+          <t>merge</t>
+        </is>
+      </c>
+      <c r="G150" s="3" t="inlineStr">
+        <is>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="3" t="inlineStr">
+        <is>
           <t>workflow/workflow-history</t>
         </is>
       </c>
-      <c r="B150" s="3" t="inlineStr">
+      <c r="B151" s="3" t="inlineStr">
         <is>
           <t>Workflow history</t>
         </is>
       </c>
-      <c r="C150" s="3" t="inlineStr">
+      <c r="C151" s="3" t="inlineStr">
         <is>
           <t>Workflow</t>
         </is>
       </c>
-      <c r="D150" s="3" t="inlineStr">
+      <c r="D151" s="3" t="inlineStr">
         <is>
           <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
         </is>
       </c>
-      <c r="E150" s="3" t="inlineStr">
+      <c r="E151" s="3" t="inlineStr">
         <is>
           <t>Live – BEE service</t>
         </is>
       </c>
-      <c r="F150" s="3" t="inlineStr">
-        <is>
-          <t>merge</t>
-        </is>
-      </c>
-      <c r="G150" s="3" t="inlineStr">
+      <c r="F151" s="3" t="inlineStr">
+        <is>
+          <t>merge</t>
+        </is>
+      </c>
+      <c r="G151" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve"> Spring menu by role or permission. Capabilities today: Choose an application; Read its steps as you are allowed to see them.</t>
         </is>
@@ -6419,11 +6456,11 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
Brief 16: the Delegations screen (ask, approve, revoke, my delegations) (#55)
* Hand over Brief 16 (delegation screen) to Cursor

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

* Brief 16: let an officer ask to delegate a role, and let the Administrator decide.

The screen offers the controls the API allows, and it reads again when a refusal means the record is out of date.

Co-authored-by: Cursor <cursoragent@cursor.com>

* Review fixes for Brief 16: date minimums, the ask form keeps its refusal until edited, the end date is shown as not included, persistent hints, alerts, captions; BL-193 done, BL-199; workbook

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

---------

Co-authored-by: Sameer Khanna <sameerkhanna@Sameers-MacBook-Pro.local>
Co-authored-by: Claude Sonnet 5.5 <noreply@anthropic.com>
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/BEE-portal-status.xlsx
+++ b/docs/tracking/BEE-portal-status.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G150"/>
+  <dimension ref="A1:G151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -1464,49 +1464,49 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>documents/access-rights</t>
+          <t>delegations</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>Access rights</t>
+          <t>Delegations</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Documents</t>
+          <t>delegations</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
+          <t>programme, director, finance, admin</t>
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: Ask to delegate a role; Withdraw or revoke your delegation; Approve or reject a request; See what you hold and until when.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>documents/check-in-or-out</t>
+          <t>documents/access-rights</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Check in or out</t>
+          <t>Access rights</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
@@ -1538,12 +1538,12 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>documents/malware-quarantine</t>
+          <t>documents/check-in-or-out</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>Malware quarantine</t>
+          <t>Check in or out</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G31" s="3" t="inlineStr">
@@ -1575,12 +1575,12 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>documents/preview</t>
+          <t>documents/malware-quarantine</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>Preview</t>
+          <t>Malware quarantine</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -1600,7 +1600,7 @@
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G32" s="3" t="inlineStr">
@@ -1612,12 +1612,12 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>documents/repository</t>
+          <t>documents/preview</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>Repository</t>
+          <t>Preview</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -1637,7 +1637,7 @@
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G33" s="3" t="inlineStr">
@@ -1649,12 +1649,12 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>documents/retention-hold</t>
+          <t>documents/repository</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>Retention hold</t>
+          <t>Repository</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
@@ -1674,7 +1674,7 @@
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G34" s="3" t="inlineStr">
@@ -1686,12 +1686,12 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>documents/search</t>
+          <t>documents/retention-hold</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>Search</t>
+          <t>Retention hold</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
@@ -1723,12 +1723,12 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>documents/version-history</t>
+          <t>documents/search</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Version history</t>
+          <t>Search</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -1760,22 +1760,22 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>enforcement/chain-of-custody</t>
+          <t>documents/version-history</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>Chain of custody</t>
+          <t>Version history</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Enforcement</t>
+          <t>Documents</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary</t>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
@@ -1797,12 +1797,12 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>enforcement/challenge-test</t>
+          <t>enforcement/chain-of-custody</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Challenge test</t>
+          <t>Chain of custody</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -1822,7 +1822,7 @@
       </c>
       <c r="F38" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G38" s="3" t="inlineStr">
@@ -1834,12 +1834,12 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>enforcement/enforcement-decision</t>
+          <t>enforcement/challenge-test</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>Enforcement decision</t>
+          <t>Challenge test</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
@@ -1871,12 +1871,12 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>enforcement/iame-or-sda-assignment</t>
+          <t>enforcement/enforcement-decision</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>IAME or SDA assignment</t>
+          <t>Enforcement decision</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
@@ -1896,7 +1896,7 @@
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G40" s="3" t="inlineStr">
@@ -1908,12 +1908,12 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>enforcement/laboratory-assignment</t>
+          <t>enforcement/iame-or-sda-assignment</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>Laboratory assignment</t>
+          <t>IAME or SDA assignment</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G41" s="3" t="inlineStr">
@@ -1945,12 +1945,12 @@
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>enforcement/manufacturer-response</t>
+          <t>enforcement/laboratory-assignment</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Manufacturer response</t>
+          <t>Laboratory assignment</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
@@ -1970,7 +1970,7 @@
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G42" s="3" t="inlineStr">
@@ -1982,12 +1982,12 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>enforcement/penalty-or-suspension</t>
+          <t>enforcement/manufacturer-response</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>Penalty or suspension</t>
+          <t>Manufacturer response</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
@@ -2019,12 +2019,12 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>enforcement/result-scrutiny</t>
+          <t>enforcement/penalty-or-suspension</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>Result scrutiny</t>
+          <t>Penalty or suspension</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
@@ -2056,12 +2056,12 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>enforcement/sample-plan</t>
+          <t>enforcement/result-scrutiny</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>Sample plan</t>
+          <t>Result scrutiny</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
@@ -2081,7 +2081,7 @@
       </c>
       <c r="F45" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G45" s="3" t="inlineStr">
@@ -2093,12 +2093,12 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>enforcement/sample-plan-approval</t>
+          <t>enforcement/sample-plan</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>Sample plan approval</t>
+          <t>Sample plan</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
@@ -2118,7 +2118,7 @@
       </c>
       <c r="F46" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G46" s="3" t="inlineStr">
@@ -2130,12 +2130,12 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>enforcement/sample-receipt</t>
+          <t>enforcement/sample-plan-approval</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>Sample receipt</t>
+          <t>Sample plan approval</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
@@ -2167,12 +2167,12 @@
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>enforcement/show-cause</t>
+          <t>enforcement/sample-receipt</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>Show cause</t>
+          <t>Sample receipt</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
@@ -2204,12 +2204,12 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>enforcement/test-report</t>
+          <t>enforcement/show-cause</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>Test report</t>
+          <t>Show cause</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
@@ -2241,12 +2241,12 @@
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>enforcement/test-result</t>
+          <t>enforcement/test-report</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>Test result</t>
+          <t>Test report</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
@@ -2278,22 +2278,22 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>finance/failed-or-duplicate-payments</t>
+          <t>enforcement/test-result</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>Failed or duplicate payments</t>
+          <t>Test result</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Finance</t>
+          <t>Enforcement</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance, Auditor</t>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary</t>
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr">
@@ -2315,12 +2315,12 @@
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>finance/fee-and-penalty-ledger</t>
+          <t>finance/failed-or-duplicate-payments</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>Fee and penalty ledger</t>
+          <t>Failed or duplicate payments</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
@@ -2352,12 +2352,12 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>finance/finance-queue</t>
+          <t>finance/fee-and-penalty-ledger</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>Finance queue</t>
+          <t>Fee and penalty ledger</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
@@ -2372,29 +2372,29 @@
       </c>
       <c r="E53" s="3" t="inlineStr">
         <is>
-          <t>Live – BEE service</t>
+          <t>Prototype (preview/sample data)</t>
         </is>
       </c>
       <c r="F53" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G53" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu roles include: finance. Capabilities today: List fee-due applications; View fee and evidence; Confirm fee received.</t>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>finance/payment-reconciliation</t>
+          <t>finance/finance-queue</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>Payment reconciliation</t>
+          <t>Finance queue</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
@@ -2409,7 +2409,7 @@
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F54" s="3" t="inlineStr">
@@ -2419,19 +2419,19 @@
       </c>
       <c r="G54" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t xml:space="preserve"> Spring menu roles include: finance. Capabilities today: List fee-due applications; View fee and evidence; Confirm fee received.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>finance/payment-verification</t>
+          <t>finance/payment-reconciliation</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>Payment verification</t>
+          <t>Payment reconciliation</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
@@ -2451,7 +2451,7 @@
       </c>
       <c r="F55" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G55" s="3" t="inlineStr">
@@ -2463,12 +2463,12 @@
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>finance/receipt</t>
+          <t>finance/payment-verification</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>Receipt</t>
+          <t>Payment verification</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="E56" s="3" t="inlineStr">
         <is>
-          <t>Live – BEE service</t>
+          <t>Prototype (preview/sample data)</t>
         </is>
       </c>
       <c r="F56" s="3" t="inlineStr">
@@ -2493,19 +2493,19 @@
       </c>
       <c r="G56" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Permission: fee_confirmation_correct. Capabilities today: See the fee confirmations and any correction; Propose a correction to a receipt reference or date; Approve or reject a colleague's correction; Withdraw your own correction.</t>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>finance/refund</t>
+          <t>finance/receipt</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>Refund</t>
+          <t>Receipt</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
@@ -2520,29 +2520,29 @@
       </c>
       <c r="E57" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F57" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G57" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t xml:space="preserve"> Permission: fee_confirmation_correct. Capabilities today: See the fee confirmations and any correction; Propose a correction to a receipt reference or date; Approve or reject a colleague's correction; Withdraw your own correction.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>finance/security-deposit-ledger</t>
+          <t>finance/refund</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>Security deposit ledger</t>
+          <t>Refund</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
@@ -2574,12 +2574,12 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>finance/settlement</t>
+          <t>finance/security-deposit-ledger</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>Settlement</t>
+          <t>Security deposit ledger</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
@@ -2599,7 +2599,7 @@
       </c>
       <c r="F59" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G59" s="3" t="inlineStr">
@@ -2611,12 +2611,12 @@
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>finance/transaction-search</t>
+          <t>finance/settlement</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>Transaction search</t>
+          <t>Settlement</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
@@ -2636,7 +2636,7 @@
       </c>
       <c r="F60" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G60" s="3" t="inlineStr">
@@ -2648,22 +2648,22 @@
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>helpdesk/agent-queue</t>
+          <t>finance/transaction-search</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>Agent queue</t>
+          <t>Transaction search</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>Helpdesk</t>
+          <t>Finance</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Helpdesk</t>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance, Auditor</t>
         </is>
       </c>
       <c r="E61" s="3" t="inlineStr">
@@ -2673,7 +2673,7 @@
       </c>
       <c r="F61" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G61" s="3" t="inlineStr">
@@ -2685,12 +2685,12 @@
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>helpdesk/assignment-and-escalation</t>
+          <t>helpdesk/agent-queue</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>Assignment and escalation</t>
+          <t>Agent queue</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
@@ -2722,12 +2722,12 @@
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>helpdesk/classification</t>
+          <t>helpdesk/assignment-and-escalation</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>Classification</t>
+          <t>Assignment and escalation</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
@@ -2759,12 +2759,12 @@
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>helpdesk/communication-history</t>
+          <t>helpdesk/classification</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>Communication history</t>
+          <t>Classification</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
@@ -2796,12 +2796,12 @@
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>helpdesk/feedback</t>
+          <t>helpdesk/communication-history</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>Feedback</t>
+          <t>Communication history</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
@@ -2833,12 +2833,12 @@
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>helpdesk/knowledge-base</t>
+          <t>helpdesk/feedback</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>Knowledge base</t>
+          <t>Feedback</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="F66" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G66" s="3" t="inlineStr">
@@ -2870,12 +2870,12 @@
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>helpdesk/raise-ticket</t>
+          <t>helpdesk/knowledge-base</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
         <is>
-          <t>Raise ticket</t>
+          <t>Knowledge base</t>
         </is>
       </c>
       <c r="C67" s="3" t="inlineStr">
@@ -2907,12 +2907,12 @@
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>helpdesk/resolution-and-closure</t>
+          <t>helpdesk/raise-ticket</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>Resolution and closure</t>
+          <t>Raise ticket</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
@@ -2932,7 +2932,7 @@
       </c>
       <c r="F68" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G68" s="3" t="inlineStr">
@@ -2944,12 +2944,12 @@
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>helpdesk/sla-dashboard</t>
+          <t>helpdesk/resolution-and-closure</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
         <is>
-          <t>SLA dashboard</t>
+          <t>Resolution and closure</t>
         </is>
       </c>
       <c r="C69" s="3" t="inlineStr">
@@ -2969,7 +2969,7 @@
       </c>
       <c r="F69" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G69" s="3" t="inlineStr">
@@ -2981,12 +2981,12 @@
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>helpdesk/track-ticket</t>
+          <t>helpdesk/sla-dashboard</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>Track ticket</t>
+          <t>SLA dashboard</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
@@ -3006,7 +3006,7 @@
       </c>
       <c r="F70" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G70" s="3" t="inlineStr">
@@ -3018,22 +3018,22 @@
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>identity/access-review</t>
+          <t>helpdesk/track-ticket</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
         <is>
-          <t>Access review</t>
+          <t>Track ticket</t>
         </is>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>Helpdesk</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary</t>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Helpdesk</t>
         </is>
       </c>
       <c r="E71" s="3" t="inlineStr">
@@ -3055,12 +3055,12 @@
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>identity/delegation</t>
+          <t>identity/access-review</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>Delegation</t>
+          <t>Access review</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
@@ -3092,12 +3092,12 @@
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>identity/login-and-mfa</t>
+          <t>identity/delegation</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
         <is>
-          <t>Login and MFA</t>
+          <t>Delegation</t>
         </is>
       </c>
       <c r="C73" s="3" t="inlineStr">
@@ -3117,7 +3117,7 @@
       </c>
       <c r="F73" s="3" t="inlineStr">
         <is>
-          <t>retire</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G73" s="3" t="inlineStr">
@@ -3129,12 +3129,12 @@
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>identity/organisation-users</t>
+          <t>identity/login-and-mfa</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>Organisation users</t>
+          <t>Login and MFA</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
@@ -3154,7 +3154,7 @@
       </c>
       <c r="F74" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>retire</t>
         </is>
       </c>
       <c r="G74" s="3" t="inlineStr">
@@ -3166,12 +3166,12 @@
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>identity/role-assignment</t>
+          <t>identity/organisation-users</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
         <is>
-          <t>Role assignment</t>
+          <t>Organisation users</t>
         </is>
       </c>
       <c r="C75" s="3" t="inlineStr">
@@ -3191,7 +3191,7 @@
       </c>
       <c r="F75" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G75" s="3" t="inlineStr">
@@ -3203,12 +3203,12 @@
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>identity/user-profile</t>
+          <t>identity/role-assignment</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>User profile</t>
+          <t>Role assignment</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
@@ -3240,22 +3240,22 @@
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>mis-ai/chatbot-review</t>
+          <t>identity/user-profile</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
         <is>
-          <t>Chatbot review</t>
+          <t>User profile</t>
         </is>
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>MIS &amp; AI</t>
+          <t>Identity</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance, Auditor</t>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary</t>
         </is>
       </c>
       <c r="E77" s="3" t="inlineStr">
@@ -3277,12 +3277,12 @@
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>mis-ai/data-quality</t>
+          <t>mis-ai/chatbot-review</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>Data quality</t>
+          <t>Chatbot review</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
@@ -3302,7 +3302,7 @@
       </c>
       <c r="F78" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G78" s="3" t="inlineStr">
@@ -3314,12 +3314,12 @@
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>mis-ai/enforcement-dashboard</t>
+          <t>mis-ai/data-quality</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
         <is>
-          <t>Enforcement dashboard</t>
+          <t>Data quality</t>
         </is>
       </c>
       <c r="C79" s="3" t="inlineStr">
@@ -3351,12 +3351,12 @@
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>mis-ai/executive-mis</t>
+          <t>mis-ai/enforcement-dashboard</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
         <is>
-          <t>Executive MIS</t>
+          <t>Enforcement dashboard</t>
         </is>
       </c>
       <c r="C80" s="3" t="inlineStr">
@@ -3388,12 +3388,12 @@
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>mis-ai/extraction-review</t>
+          <t>mis-ai/executive-mis</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
         <is>
-          <t>Extraction review</t>
+          <t>Executive MIS</t>
         </is>
       </c>
       <c r="C81" s="3" t="inlineStr">
@@ -3413,7 +3413,7 @@
       </c>
       <c r="F81" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G81" s="3" t="inlineStr">
@@ -3425,12 +3425,12 @@
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>mis-ai/helpdesk-dashboard</t>
+          <t>mis-ai/extraction-review</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
         <is>
-          <t>Helpdesk dashboard</t>
+          <t>Extraction review</t>
         </is>
       </c>
       <c r="C82" s="3" t="inlineStr">
@@ -3462,12 +3462,12 @@
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>mis-ai/model-dashboard</t>
+          <t>mis-ai/helpdesk-dashboard</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
         <is>
-          <t>Model dashboard</t>
+          <t>Helpdesk dashboard</t>
         </is>
       </c>
       <c r="C83" s="3" t="inlineStr">
@@ -3499,12 +3499,12 @@
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>mis-ai/model-monitoring</t>
+          <t>mis-ai/model-dashboard</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>Model monitoring</t>
+          <t>Model dashboard</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
@@ -3524,7 +3524,7 @@
       </c>
       <c r="F84" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G84" s="3" t="inlineStr">
@@ -3536,12 +3536,12 @@
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>mis-ai/production-and-fee-dashboard</t>
+          <t>mis-ai/model-monitoring</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
         <is>
-          <t>Production and fee dashboard</t>
+          <t>Model monitoring</t>
         </is>
       </c>
       <c r="C85" s="3" t="inlineStr">
@@ -3561,7 +3561,7 @@
       </c>
       <c r="F85" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G85" s="3" t="inlineStr">
@@ -3573,12 +3573,12 @@
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>mis-ai/production-anomaly</t>
+          <t>mis-ai/production-and-fee-dashboard</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
         <is>
-          <t>Production anomaly</t>
+          <t>Production and fee dashboard</t>
         </is>
       </c>
       <c r="C86" s="3" t="inlineStr">
@@ -3610,12 +3610,12 @@
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>mis-ai/rating-trends</t>
+          <t>mis-ai/production-anomaly</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
         <is>
-          <t>Rating trends</t>
+          <t>Production anomaly</t>
         </is>
       </c>
       <c r="C87" s="3" t="inlineStr">
@@ -3647,12 +3647,12 @@
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>mis-ai/registration-dashboard</t>
+          <t>mis-ai/rating-trends</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
         <is>
-          <t>Registration dashboard</t>
+          <t>Rating trends</t>
         </is>
       </c>
       <c r="C88" s="3" t="inlineStr">
@@ -3672,7 +3672,7 @@
       </c>
       <c r="F88" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G88" s="3" t="inlineStr">
@@ -3684,12 +3684,12 @@
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>mis-ai/report-builder</t>
+          <t>mis-ai/registration-dashboard</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
         <is>
-          <t>Report builder</t>
+          <t>Registration dashboard</t>
         </is>
       </c>
       <c r="C89" s="3" t="inlineStr">
@@ -3721,12 +3721,12 @@
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>mis-ai/risk-scoring</t>
+          <t>mis-ai/report-builder</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>Risk scoring</t>
+          <t>Report builder</t>
         </is>
       </c>
       <c r="C90" s="3" t="inlineStr">
@@ -3746,7 +3746,7 @@
       </c>
       <c r="F90" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G90" s="3" t="inlineStr">
@@ -3758,12 +3758,12 @@
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>mis-ai/scheduled-reports</t>
+          <t>mis-ai/risk-scoring</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
         <is>
-          <t>Scheduled reports</t>
+          <t>Risk scoring</t>
         </is>
       </c>
       <c r="C91" s="3" t="inlineStr">
@@ -3795,22 +3795,22 @@
     <row r="92">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t>model-label/approval-letter</t>
+          <t>mis-ai/scheduled-reports</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
         <is>
-          <t>Approval letter</t>
+          <t>Scheduled reports</t>
         </is>
       </c>
       <c r="C92" s="3" t="inlineStr">
         <is>
-          <t>Model &amp; Label</t>
+          <t>MIS &amp; AI</t>
         </is>
       </c>
       <c r="D92" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance, Helpdesk</t>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance, Auditor</t>
         </is>
       </c>
       <c r="E92" s="3" t="inlineStr">
@@ -3832,12 +3832,12 @@
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>model-label/approval-note</t>
+          <t>model-label/approval-letter</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
         <is>
-          <t>Approval note</t>
+          <t>Approval letter</t>
         </is>
       </c>
       <c r="C93" s="3" t="inlineStr">
@@ -3869,12 +3869,12 @@
     <row r="94">
       <c r="A94" s="3" t="inlineStr">
         <is>
-          <t>model-label/bee-scrutiny</t>
+          <t>model-label/approval-note</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
         <is>
-          <t>BEE scrutiny</t>
+          <t>Approval note</t>
         </is>
       </c>
       <c r="C94" s="3" t="inlineStr">
@@ -3889,29 +3889,29 @@
       </c>
       <c r="E94" s="3" t="inlineStr">
         <is>
-          <t>Live – BEE service</t>
+          <t>Prototype (preview/sample data)</t>
         </is>
       </c>
       <c r="F94" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G94" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu roles include: reviewer. Capabilities today: List assigned applications; View evidence and test reports; Forward to rating; Return to the applicant; Reject permanently; See the earlier steps and notes.</t>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>model-label/director-approval</t>
+          <t>model-label/bee-scrutiny</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
         <is>
-          <t>Director approval</t>
+          <t>BEE scrutiny</t>
         </is>
       </c>
       <c r="C95" s="3" t="inlineStr">
@@ -3936,19 +3936,19 @@
       </c>
       <c r="G95" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu roles include: director, secretary. Capabilities today: List applications awaiting your decision; View the rating, evidence and test reports; Recommend approval (Director); Give final approval (Secretary); Return to the applicant; Reject permanently; See the earlier steps and notes.</t>
+          <t xml:space="preserve"> Spring menu roles include: reviewer. Capabilities today: List assigned applications; View evidence and test reports; Forward to rating; Return to the applicant; Reject permanently; See the earlier steps and notes.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t>model-label/family-models</t>
+          <t>model-label/director-approval</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
         <is>
-          <t>Family models</t>
+          <t>Director approval</t>
         </is>
       </c>
       <c r="C96" s="3" t="inlineStr">
@@ -3963,29 +3963,29 @@
       </c>
       <c r="E96" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F96" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G96" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t xml:space="preserve"> Spring menu roles include: director, secretary. Capabilities today: List applications awaiting your decision; View the rating, evidence and test reports; Recommend approval (Director); Give final approval (Secretary); Return to the applicant; Reject permanently; See the earlier steps and notes.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>model-label/iame-scrutiny</t>
+          <t>model-label/family-models</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
         <is>
-          <t>IAME scrutiny</t>
+          <t>Family models</t>
         </is>
       </c>
       <c r="C97" s="3" t="inlineStr">
@@ -4000,29 +4000,29 @@
       </c>
       <c r="E97" s="3" t="inlineStr">
         <is>
-          <t>Live – BEE service</t>
+          <t>Prototype (preview/sample data)</t>
         </is>
       </c>
       <c r="F97" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G97" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu roles include: iame. Capabilities today: List assigned applications; View evidence and test reports; Record finding and forward; Return to the applicant; Reject permanently; See the earlier steps and notes.</t>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="3" t="inlineStr">
         <is>
-          <t>model-label/lab-accreditation</t>
+          <t>model-label/iame-scrutiny</t>
         </is>
       </c>
       <c r="B98" s="3" t="inlineStr">
         <is>
-          <t>Lab accreditation</t>
+          <t>IAME scrutiny</t>
         </is>
       </c>
       <c r="C98" s="3" t="inlineStr">
@@ -4037,29 +4037,29 @@
       </c>
       <c r="E98" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F98" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G98" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t xml:space="preserve"> Spring menu roles include: iame. Capabilities today: List assigned applications; View evidence and test reports; Record finding and forward; Return to the applicant; Reject permanently; See the earlier steps and notes.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t>model-label/label-details</t>
+          <t>model-label/lab-accreditation</t>
         </is>
       </c>
       <c r="B99" s="3" t="inlineStr">
         <is>
-          <t>Label details</t>
+          <t>Lab accreditation</t>
         </is>
       </c>
       <c r="C99" s="3" t="inlineStr">
@@ -4091,12 +4091,12 @@
     <row r="100">
       <c r="A100" s="3" t="inlineStr">
         <is>
-          <t>model-label/label-preview</t>
+          <t>model-label/label-details</t>
         </is>
       </c>
       <c r="B100" s="3" t="inlineStr">
         <is>
-          <t>Label preview</t>
+          <t>Label details</t>
         </is>
       </c>
       <c r="C100" s="3" t="inlineStr">
@@ -4111,29 +4111,29 @@
       </c>
       <c r="E100" s="3" t="inlineStr">
         <is>
-          <t>Live – BEE service</t>
+          <t>Prototype (preview/sample data)</t>
         </is>
       </c>
       <c r="F100" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G100" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu roles include: manufacturer, agency. Capabilities today: List your approved applications; Open the printable certificate and star label; Print or save as PDF; A QR code that opens the public verification page.</t>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>model-label/model-dashboard</t>
+          <t>model-label/label-preview</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
         <is>
-          <t>Model dashboard</t>
+          <t>Label preview</t>
         </is>
       </c>
       <c r="C101" s="3" t="inlineStr">
@@ -4158,19 +4158,19 @@
       </c>
       <c r="G101" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu roles include: manufacturer, agency. Capabilities today: List; View detail; Edit draft; Submit draft; See why it was returned; Edit and resubmit; See why it was rejected; See the history.</t>
+          <t xml:space="preserve"> Spring menu roles include: manufacturer, agency. Capabilities today: List your approved applications; Open the printable certificate and star label; Print or save as PDF; A QR code that opens the public verification page.</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="3" t="inlineStr">
         <is>
-          <t>model-label/model-documents</t>
+          <t>model-label/model-dashboard</t>
         </is>
       </c>
       <c r="B102" s="3" t="inlineStr">
         <is>
-          <t>Model documents</t>
+          <t>Model dashboard</t>
         </is>
       </c>
       <c r="C102" s="3" t="inlineStr">
@@ -4185,29 +4185,29 @@
       </c>
       <c r="E102" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F102" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G102" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t xml:space="preserve"> Spring menu roles include: manufacturer, agency. Capabilities today: List; View detail; Edit draft; Submit draft; See why it was returned; Edit and resubmit; See why it was rejected; See the history.</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>model-label/model-payment</t>
+          <t>model-label/model-documents</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
         <is>
-          <t>Model payment</t>
+          <t>Model documents</t>
         </is>
       </c>
       <c r="C103" s="3" t="inlineStr">
@@ -4227,7 +4227,7 @@
       </c>
       <c r="F103" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G103" s="3" t="inlineStr">
@@ -4239,12 +4239,12 @@
     <row r="104">
       <c r="A104" s="3" t="inlineStr">
         <is>
-          <t>model-label/new-model-application</t>
+          <t>model-label/model-payment</t>
         </is>
       </c>
       <c r="B104" s="3" t="inlineStr">
         <is>
-          <t>New model application</t>
+          <t>Model payment</t>
         </is>
       </c>
       <c r="C104" s="3" t="inlineStr">
@@ -4259,7 +4259,7 @@
       </c>
       <c r="E104" s="3" t="inlineStr">
         <is>
-          <t>Live – BEE service</t>
+          <t>Prototype (preview/sample data)</t>
         </is>
       </c>
       <c r="F104" s="3" t="inlineStr">
@@ -4269,19 +4269,19 @@
       </c>
       <c r="G104" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu roles include: manufacturer, agency. Capabilities today: Create draft; Edit draft; Upload test reports; Submit draft; Edit and resubmit a returned application.</t>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
         <is>
-          <t>model-label/notifications</t>
+          <t>model-label/new-model-application</t>
         </is>
       </c>
       <c r="B105" s="3" t="inlineStr">
         <is>
-          <t>Notifications</t>
+          <t>New model application</t>
         </is>
       </c>
       <c r="C105" s="3" t="inlineStr">
@@ -4306,19 +4306,19 @@
       </c>
       <c r="G105" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu roles include: manufacturer, agency. Capabilities today: See updates about your applications; Open the screen to act; Mark one or all as read.</t>
+          <t xml:space="preserve"> Spring menu roles include: manufacturer, agency. Capabilities today: Create draft; Edit draft; Upload test reports; Submit draft; Edit and resubmit a returned application.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="3" t="inlineStr">
         <is>
-          <t>model-label/performance-parameters</t>
+          <t>model-label/notifications</t>
         </is>
       </c>
       <c r="B106" s="3" t="inlineStr">
         <is>
-          <t>Performance parameters</t>
+          <t>Notifications</t>
         </is>
       </c>
       <c r="C106" s="3" t="inlineStr">
@@ -4333,29 +4333,29 @@
       </c>
       <c r="E106" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F106" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G106" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t xml:space="preserve"> Spring menu roles include: manufacturer, agency. Capabilities today: See updates about your applications; Open the screen to act; Mark one or all as read.</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
         <is>
-          <t>model-label/rating-calculation</t>
+          <t>model-label/performance-parameters</t>
         </is>
       </c>
       <c r="B107" s="3" t="inlineStr">
         <is>
-          <t>Rating calculation</t>
+          <t>Performance parameters</t>
         </is>
       </c>
       <c r="C107" s="3" t="inlineStr">
@@ -4370,29 +4370,29 @@
       </c>
       <c r="E107" s="3" t="inlineStr">
         <is>
-          <t>Live – BEE service</t>
+          <t>Prototype (preview/sample data)</t>
         </is>
       </c>
       <c r="F107" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G107" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu roles include: programme. Capabilities today: List applications awaiting a rating; View evidence and test reports; Compute and record a provisional local rating; Reject permanently; See the earlier steps and notes.</t>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
         <is>
-          <t>model-label/renewal-or-degradation</t>
+          <t>model-label/rating-calculation</t>
         </is>
       </c>
       <c r="B108" s="3" t="inlineStr">
         <is>
-          <t>Renewal or degradation</t>
+          <t>Rating calculation</t>
         </is>
       </c>
       <c r="C108" s="3" t="inlineStr">
@@ -4407,7 +4407,7 @@
       </c>
       <c r="E108" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F108" s="3" t="inlineStr">
@@ -4417,19 +4417,19 @@
       </c>
       <c r="G108" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t xml:space="preserve"> Spring menu roles include: programme. Capabilities today: List applications awaiting a rating; View evidence and test reports; Compute and record a provisional local rating; Reject permanently; See the earlier steps and notes.</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
         <is>
-          <t>model-label/secretary-approval</t>
+          <t>model-label/renewal-or-degradation</t>
         </is>
       </c>
       <c r="B109" s="3" t="inlineStr">
         <is>
-          <t>Secretary approval</t>
+          <t>Renewal or degradation</t>
         </is>
       </c>
       <c r="C109" s="3" t="inlineStr">
@@ -4449,7 +4449,7 @@
       </c>
       <c r="F109" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G109" s="3" t="inlineStr">
@@ -4461,12 +4461,12 @@
     <row r="110">
       <c r="A110" s="3" t="inlineStr">
         <is>
-          <t>model-label/test-reports</t>
+          <t>model-label/secretary-approval</t>
         </is>
       </c>
       <c r="B110" s="3" t="inlineStr">
         <is>
-          <t>Test reports</t>
+          <t>Secretary approval</t>
         </is>
       </c>
       <c r="C110" s="3" t="inlineStr">
@@ -4498,17 +4498,17 @@
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t>production/bulk-upload</t>
+          <t>model-label/test-reports</t>
         </is>
       </c>
       <c r="B111" s="3" t="inlineStr">
         <is>
-          <t>Bulk upload</t>
+          <t>Test reports</t>
         </is>
       </c>
       <c r="C111" s="3" t="inlineStr">
         <is>
-          <t>Production</t>
+          <t>Model &amp; Label</t>
         </is>
       </c>
       <c r="D111" s="3" t="inlineStr">
@@ -4523,7 +4523,7 @@
       </c>
       <c r="F111" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G111" s="3" t="inlineStr">
@@ -4535,12 +4535,12 @@
     <row r="112">
       <c r="A112" s="3" t="inlineStr">
         <is>
-          <t>production/ca-evidence</t>
+          <t>production/bulk-upload</t>
         </is>
       </c>
       <c r="B112" s="3" t="inlineStr">
         <is>
-          <t>CA evidence</t>
+          <t>Bulk upload</t>
         </is>
       </c>
       <c r="C112" s="3" t="inlineStr">
@@ -4560,7 +4560,7 @@
       </c>
       <c r="F112" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G112" s="3" t="inlineStr">
@@ -4572,12 +4572,12 @@
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
         <is>
-          <t>production/compliance-exceptions</t>
+          <t>production/ca-evidence</t>
         </is>
       </c>
       <c r="B113" s="3" t="inlineStr">
         <is>
-          <t>Compliance exceptions</t>
+          <t>CA evidence</t>
         </is>
       </c>
       <c r="C113" s="3" t="inlineStr">
@@ -4597,7 +4597,7 @@
       </c>
       <c r="F113" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G113" s="3" t="inlineStr">
@@ -4609,12 +4609,12 @@
     <row r="114">
       <c r="A114" s="3" t="inlineStr">
         <is>
-          <t>production/correction-request</t>
+          <t>production/compliance-exceptions</t>
         </is>
       </c>
       <c r="B114" s="3" t="inlineStr">
         <is>
-          <t>Correction request</t>
+          <t>Compliance exceptions</t>
         </is>
       </c>
       <c r="C114" s="3" t="inlineStr">
@@ -4634,7 +4634,7 @@
       </c>
       <c r="F114" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G114" s="3" t="inlineStr">
@@ -4646,12 +4646,12 @@
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
         <is>
-          <t>production/label-fee</t>
+          <t>production/correction-request</t>
         </is>
       </c>
       <c r="B115" s="3" t="inlineStr">
         <is>
-          <t>Label fee</t>
+          <t>Correction request</t>
         </is>
       </c>
       <c r="C115" s="3" t="inlineStr">
@@ -4683,12 +4683,12 @@
     <row r="116">
       <c r="A116" s="3" t="inlineStr">
         <is>
-          <t>production/production-payment</t>
+          <t>production/label-fee</t>
         </is>
       </c>
       <c r="B116" s="3" t="inlineStr">
         <is>
-          <t>Production payment</t>
+          <t>Label fee</t>
         </is>
       </c>
       <c r="C116" s="3" t="inlineStr">
@@ -4720,12 +4720,12 @@
     <row r="117">
       <c r="A117" s="3" t="inlineStr">
         <is>
-          <t>production/quarterly-submission</t>
+          <t>production/production-payment</t>
         </is>
       </c>
       <c r="B117" s="3" t="inlineStr">
         <is>
-          <t>Quarterly submission</t>
+          <t>Production payment</t>
         </is>
       </c>
       <c r="C117" s="3" t="inlineStr">
@@ -4745,7 +4745,7 @@
       </c>
       <c r="F117" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G117" s="3" t="inlineStr">
@@ -4757,12 +4757,12 @@
     <row r="118">
       <c r="A118" s="3" t="inlineStr">
         <is>
-          <t>production/reconciliation</t>
+          <t>production/quarterly-submission</t>
         </is>
       </c>
       <c r="B118" s="3" t="inlineStr">
         <is>
-          <t>Reconciliation</t>
+          <t>Quarterly submission</t>
         </is>
       </c>
       <c r="C118" s="3" t="inlineStr">
@@ -4794,12 +4794,12 @@
     <row r="119">
       <c r="A119" s="3" t="inlineStr">
         <is>
-          <t>production/validation-results</t>
+          <t>production/reconciliation</t>
         </is>
       </c>
       <c r="B119" s="3" t="inlineStr">
         <is>
-          <t>Validation results</t>
+          <t>Reconciliation</t>
         </is>
       </c>
       <c r="C119" s="3" t="inlineStr">
@@ -4819,7 +4819,7 @@
       </c>
       <c r="F119" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G119" s="3" t="inlineStr">
@@ -4831,22 +4831,22 @@
     <row r="120">
       <c r="A120" s="3" t="inlineStr">
         <is>
-          <t>qr-verification/batch-file-download</t>
+          <t>production/validation-results</t>
         </is>
       </c>
       <c r="B120" s="3" t="inlineStr">
         <is>
-          <t>Batch file download</t>
+          <t>Validation results</t>
         </is>
       </c>
       <c r="C120" s="3" t="inlineStr">
         <is>
-          <t>QR &amp; Verification</t>
+          <t>Production</t>
         </is>
       </c>
       <c r="D120" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Helpdesk</t>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance, Helpdesk</t>
         </is>
       </c>
       <c r="E120" s="3" t="inlineStr">
@@ -4868,12 +4868,12 @@
     <row r="121">
       <c r="A121" s="3" t="inlineStr">
         <is>
-          <t>qr-verification/certificate-verification</t>
+          <t>qr-verification/batch-file-download</t>
         </is>
       </c>
       <c r="B121" s="3" t="inlineStr">
         <is>
-          <t>Certificate verification</t>
+          <t>Batch file download</t>
         </is>
       </c>
       <c r="C121" s="3" t="inlineStr">
@@ -4905,12 +4905,12 @@
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>qr-verification/duplicate-exceptions</t>
+          <t>qr-verification/certificate-verification</t>
         </is>
       </c>
       <c r="B122" s="3" t="inlineStr">
         <is>
-          <t>Duplicate exceptions</t>
+          <t>Certificate verification</t>
         </is>
       </c>
       <c r="C122" s="3" t="inlineStr">
@@ -4942,12 +4942,12 @@
     <row r="123">
       <c r="A123" s="3" t="inlineStr">
         <is>
-          <t>qr-verification/public-verification</t>
+          <t>qr-verification/duplicate-exceptions</t>
         </is>
       </c>
       <c r="B123" s="3" t="inlineStr">
         <is>
-          <t>Public verification</t>
+          <t>Duplicate exceptions</t>
         </is>
       </c>
       <c r="C123" s="3" t="inlineStr">
@@ -4967,7 +4967,7 @@
       </c>
       <c r="F123" s="3" t="inlineStr">
         <is>
-          <t>retire</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G123" s="3" t="inlineStr">
@@ -4979,12 +4979,12 @@
     <row r="124">
       <c r="A124" s="3" t="inlineStr">
         <is>
-          <t>qr-verification/qr-batch-request</t>
+          <t>qr-verification/public-verification</t>
         </is>
       </c>
       <c r="B124" s="3" t="inlineStr">
         <is>
-          <t>QR batch request</t>
+          <t>Public verification</t>
         </is>
       </c>
       <c r="C124" s="3" t="inlineStr">
@@ -5004,7 +5004,7 @@
       </c>
       <c r="F124" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>retire</t>
         </is>
       </c>
       <c r="G124" s="3" t="inlineStr">
@@ -5016,12 +5016,12 @@
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
         <is>
-          <t>qr-verification/qr-batch-status</t>
+          <t>qr-verification/qr-batch-request</t>
         </is>
       </c>
       <c r="B125" s="3" t="inlineStr">
         <is>
-          <t>QR batch status</t>
+          <t>QR batch request</t>
         </is>
       </c>
       <c r="C125" s="3" t="inlineStr">
@@ -5053,12 +5053,12 @@
     <row r="126">
       <c r="A126" s="3" t="inlineStr">
         <is>
-          <t>qr-verification/qr-download</t>
+          <t>qr-verification/qr-batch-status</t>
         </is>
       </c>
       <c r="B126" s="3" t="inlineStr">
         <is>
-          <t>QR download</t>
+          <t>QR batch status</t>
         </is>
       </c>
       <c r="C126" s="3" t="inlineStr">
@@ -5090,12 +5090,12 @@
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
         <is>
-          <t>qr-verification/serial-upload</t>
+          <t>qr-verification/qr-download</t>
         </is>
       </c>
       <c r="B127" s="3" t="inlineStr">
         <is>
-          <t>Serial upload</t>
+          <t>QR download</t>
         </is>
       </c>
       <c r="C127" s="3" t="inlineStr">
@@ -5127,49 +5127,49 @@
     <row r="128">
       <c r="A128" s="3" t="inlineStr">
         <is>
-          <t>registrations/new</t>
+          <t>qr-verification/serial-upload</t>
         </is>
       </c>
       <c r="B128" s="3" t="inlineStr">
         <is>
-          <t>New registration request</t>
+          <t>Serial upload</t>
         </is>
       </c>
       <c r="C128" s="3" t="inlineStr">
         <is>
-          <t>registrations</t>
+          <t>QR &amp; Verification</t>
         </is>
       </c>
       <c r="D128" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Helpdesk</t>
         </is>
       </c>
       <c r="E128" s="3" t="inlineStr">
         <is>
-          <t>Live – BEE service</t>
+          <t>Prototype (preview/sample data)</t>
         </is>
       </c>
       <c r="F128" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G128" s="3" t="inlineStr">
         <is>
-          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: File a brand request; Ask to act for a brand; Save a draft.</t>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="3" t="inlineStr">
         <is>
-          <t>registrations/register</t>
+          <t>registrations/new</t>
         </is>
       </c>
       <c r="B129" s="3" t="inlineStr">
         <is>
-          <t>Register</t>
+          <t>New registration request</t>
         </is>
       </c>
       <c r="C129" s="3" t="inlineStr">
@@ -5179,7 +5179,7 @@
       </c>
       <c r="D129" s="3" t="inlineStr">
         <is>
-          <t>programme, director</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E129" s="3" t="inlineStr">
@@ -5194,19 +5194,19 @@
       </c>
       <c r="G129" s="3" t="inlineStr">
         <is>
-          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: See registered brands and authorisations; Propose a closure or revocation; Approve, reject or withdraw a proposal; Read the history.</t>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: File a brand request; Ask to act for a brand; Save a draft.</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="3" t="inlineStr">
         <is>
-          <t>registrations/request</t>
+          <t>registrations/register</t>
         </is>
       </c>
       <c r="B130" s="3" t="inlineStr">
         <is>
-          <t>Registration request</t>
+          <t>Register</t>
         </is>
       </c>
       <c r="C130" s="3" t="inlineStr">
@@ -5216,7 +5216,7 @@
       </c>
       <c r="D130" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>programme, director</t>
         </is>
       </c>
       <c r="E130" s="3" t="inlineStr">
@@ -5231,19 +5231,19 @@
       </c>
       <c r="G130" s="3" t="inlineStr">
         <is>
-          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: See the request; Upload the trade licence; See the fee and submit; Follow the request until Programme review; Recommend or return; Approve, return or reject; See why it was returned and resubmit.</t>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: See registered brands and authorisations; Propose a closure or revocation; Approve, reject or withdraw a proposal; Read the history.</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="3" t="inlineStr">
         <is>
-          <t>registrations/requests</t>
+          <t>registrations/request</t>
         </is>
       </c>
       <c r="B131" s="3" t="inlineStr">
         <is>
-          <t>Registration requests</t>
+          <t>Registration request</t>
         </is>
       </c>
       <c r="C131" s="3" t="inlineStr">
@@ -5253,7 +5253,7 @@
       </c>
       <c r="D131" s="3" t="inlineStr">
         <is>
-          <t>manufacturer, agency</t>
+          <t>—</t>
         </is>
       </c>
       <c r="E131" s="3" t="inlineStr">
@@ -5268,19 +5268,19 @@
       </c>
       <c r="G131" s="3" t="inlineStr">
         <is>
-          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: List your registration requests; Open a request; Start a new request.</t>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: See the request; Upload the trade licence; See the fee and submit; Follow the request until Programme review; Recommend or return; Approve, return or reject; See why it was returned and resubmit.</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="3" t="inlineStr">
         <is>
-          <t>registrations/reviews</t>
+          <t>registrations/requests</t>
         </is>
       </c>
       <c r="B132" s="3" t="inlineStr">
         <is>
-          <t>Registration reviews</t>
+          <t>Registration requests</t>
         </is>
       </c>
       <c r="C132" s="3" t="inlineStr">
@@ -5290,7 +5290,7 @@
       </c>
       <c r="D132" s="3" t="inlineStr">
         <is>
-          <t>programme, director</t>
+          <t>manufacturer, agency</t>
         </is>
       </c>
       <c r="E132" s="3" t="inlineStr">
@@ -5305,34 +5305,34 @@
       </c>
       <c r="G132" s="3" t="inlineStr">
         <is>
-          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: List requests waiting for you; Recommend or return; Approve, return or reject; Read the trail.</t>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: List your registration requests; Open a request; Start a new request.</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/brand-withdrawal</t>
+          <t>registrations/reviews</t>
         </is>
       </c>
       <c r="B133" s="3" t="inlineStr">
         <is>
-          <t>Brand withdrawal</t>
+          <t>Registration reviews</t>
         </is>
       </c>
       <c r="C133" s="3" t="inlineStr">
         <is>
-          <t>Withdrawal</t>
+          <t>registrations</t>
         </is>
       </c>
       <c r="D133" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance</t>
+          <t>programme, director</t>
         </is>
       </c>
       <c r="E133" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F133" s="3" t="inlineStr">
@@ -5342,19 +5342,19 @@
       </c>
       <c r="G133" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: List requests waiting for you; Recommend or return; Approve, return or reject; Read the trail.</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/deposit-release</t>
+          <t>withdrawal/brand-withdrawal</t>
         </is>
       </c>
       <c r="B134" s="3" t="inlineStr">
         <is>
-          <t>Deposit release</t>
+          <t>Brand withdrawal</t>
         </is>
       </c>
       <c r="C134" s="3" t="inlineStr">
@@ -5374,7 +5374,7 @@
       </c>
       <c r="F134" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G134" s="3" t="inlineStr">
@@ -5386,12 +5386,12 @@
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/dues-verification</t>
+          <t>withdrawal/deposit-release</t>
         </is>
       </c>
       <c r="B135" s="3" t="inlineStr">
         <is>
-          <t>Dues verification</t>
+          <t>Deposit release</t>
         </is>
       </c>
       <c r="C135" s="3" t="inlineStr">
@@ -5423,12 +5423,12 @@
     <row r="136">
       <c r="A136" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/model-withdrawal</t>
+          <t>withdrawal/dues-verification</t>
         </is>
       </c>
       <c r="B136" s="3" t="inlineStr">
         <is>
-          <t>Model withdrawal</t>
+          <t>Dues verification</t>
         </is>
       </c>
       <c r="C136" s="3" t="inlineStr">
@@ -5460,12 +5460,12 @@
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/revocation-initiation</t>
+          <t>withdrawal/model-withdrawal</t>
         </is>
       </c>
       <c r="B137" s="3" t="inlineStr">
         <is>
-          <t>Revocation initiation</t>
+          <t>Model withdrawal</t>
         </is>
       </c>
       <c r="C137" s="3" t="inlineStr">
@@ -5497,12 +5497,12 @@
     <row r="138">
       <c r="A138" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/withdrawal-approval</t>
+          <t>withdrawal/revocation-initiation</t>
         </is>
       </c>
       <c r="B138" s="3" t="inlineStr">
         <is>
-          <t>Withdrawal approval</t>
+          <t>Revocation initiation</t>
         </is>
       </c>
       <c r="C138" s="3" t="inlineStr">
@@ -5534,12 +5534,12 @@
     <row r="139">
       <c r="A139" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/withdrawal-letter</t>
+          <t>withdrawal/withdrawal-approval</t>
         </is>
       </c>
       <c r="B139" s="3" t="inlineStr">
         <is>
-          <t>Withdrawal letter</t>
+          <t>Withdrawal approval</t>
         </is>
       </c>
       <c r="C139" s="3" t="inlineStr">
@@ -5571,12 +5571,12 @@
     <row r="140">
       <c r="A140" s="3" t="inlineStr">
         <is>
-          <t>withdrawal/withdrawal-scrutiny</t>
+          <t>withdrawal/withdrawal-letter</t>
         </is>
       </c>
       <c r="B140" s="3" t="inlineStr">
         <is>
-          <t>Withdrawal scrutiny</t>
+          <t>Withdrawal letter</t>
         </is>
       </c>
       <c r="C140" s="3" t="inlineStr">
@@ -5608,27 +5608,27 @@
     <row r="141">
       <c r="A141" s="3" t="inlineStr">
         <is>
-          <t>workflow/application-review</t>
+          <t>withdrawal/withdrawal-scrutiny</t>
         </is>
       </c>
       <c r="B141" s="3" t="inlineStr">
         <is>
-          <t>Application review</t>
+          <t>Withdrawal scrutiny</t>
         </is>
       </c>
       <c r="C141" s="3" t="inlineStr">
         <is>
-          <t>Workflow</t>
+          <t>Withdrawal</t>
         </is>
       </c>
       <c r="D141" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Finance</t>
         </is>
       </c>
       <c r="E141" s="3" t="inlineStr">
         <is>
-          <t>Live – BEE service</t>
+          <t>Prototype (preview/sample data)</t>
         </is>
       </c>
       <c r="F141" s="3" t="inlineStr">
@@ -5638,19 +5638,19 @@
       </c>
       <c r="G141" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu by role or permission. Capabilities today: List the applications in progress; Link to your next action; Link to the history.</t>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="3" t="inlineStr">
         <is>
-          <t>workflow/approval-note</t>
+          <t>workflow/application-review</t>
         </is>
       </c>
       <c r="B142" s="3" t="inlineStr">
         <is>
-          <t>Approval note</t>
+          <t>Application review</t>
         </is>
       </c>
       <c r="C142" s="3" t="inlineStr">
@@ -5665,7 +5665,7 @@
       </c>
       <c r="E142" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F142" s="3" t="inlineStr">
@@ -5675,19 +5675,19 @@
       </c>
       <c r="G142" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t xml:space="preserve"> Spring menu by role or permission. Capabilities today: List the applications in progress; Link to your next action; Link to the history.</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="3" t="inlineStr">
         <is>
-          <t>workflow/checklist</t>
+          <t>workflow/approval-note</t>
         </is>
       </c>
       <c r="B143" s="3" t="inlineStr">
         <is>
-          <t>Checklist</t>
+          <t>Approval note</t>
         </is>
       </c>
       <c r="C143" s="3" t="inlineStr">
@@ -5719,12 +5719,12 @@
     <row r="144">
       <c r="A144" s="3" t="inlineStr">
         <is>
-          <t>workflow/clarification-and-return</t>
+          <t>workflow/checklist</t>
         </is>
       </c>
       <c r="B144" s="3" t="inlineStr">
         <is>
-          <t>Clarification and return</t>
+          <t>Checklist</t>
         </is>
       </c>
       <c r="C144" s="3" t="inlineStr">
@@ -5756,12 +5756,12 @@
     <row r="145">
       <c r="A145" s="3" t="inlineStr">
         <is>
-          <t>workflow/delegation-and-reassignment</t>
+          <t>workflow/clarification-and-return</t>
         </is>
       </c>
       <c r="B145" s="3" t="inlineStr">
         <is>
-          <t>Delegation and reassignment</t>
+          <t>Clarification and return</t>
         </is>
       </c>
       <c r="C145" s="3" t="inlineStr">
@@ -5793,12 +5793,12 @@
     <row r="146">
       <c r="A146" s="3" t="inlineStr">
         <is>
-          <t>workflow/escalation-dashboard</t>
+          <t>workflow/delegation-and-reassignment</t>
         </is>
       </c>
       <c r="B146" s="3" t="inlineStr">
         <is>
-          <t>Escalation dashboard</t>
+          <t>Delegation and reassignment</t>
         </is>
       </c>
       <c r="C146" s="3" t="inlineStr">
@@ -5813,39 +5813,39 @@
       </c>
       <c r="E146" s="3" t="inlineStr">
         <is>
-          <t>Live – BEE service</t>
+          <t>Prototype (preview/sample data)</t>
         </is>
       </c>
       <c r="F146" s="3" t="inlineStr">
         <is>
-          <t>keep</t>
+          <t>merge</t>
         </is>
       </c>
       <c r="G146" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu by role or permission. Capabilities today: Count the applications waiting at each stage (no time limits are set yet).</t>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="3" t="inlineStr">
         <is>
-          <t>workflow/my-approvals</t>
+          <t>workflow/escalation-dashboard</t>
         </is>
       </c>
       <c r="B147" s="3" t="inlineStr">
         <is>
-          <t>My approvals</t>
+          <t>Escalation dashboard</t>
         </is>
       </c>
       <c r="C147" s="3" t="inlineStr">
         <is>
-          <t>workflow</t>
+          <t>Workflow</t>
         </is>
       </c>
       <c r="D147" s="3" t="inlineStr">
         <is>
-          <t>director, secretary</t>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
         </is>
       </c>
       <c r="E147" s="3" t="inlineStr">
@@ -5860,29 +5860,29 @@
       </c>
       <c r="G147" s="3" t="inlineStr">
         <is>
-          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: List the applications waiting for your decision; Open the approval screen.</t>
+          <t xml:space="preserve"> Spring menu by role or permission. Capabilities today: Count the applications waiting at each stage (no time limits are set yet).</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="3" t="inlineStr">
         <is>
-          <t>workflow/personal-inbox</t>
+          <t>workflow/my-approvals</t>
         </is>
       </c>
       <c r="B148" s="3" t="inlineStr">
         <is>
-          <t>Personal inbox</t>
+          <t>My approvals</t>
         </is>
       </c>
       <c r="C148" s="3" t="inlineStr">
         <is>
-          <t>Workflow</t>
+          <t>workflow</t>
         </is>
       </c>
       <c r="D148" s="3" t="inlineStr">
         <is>
-          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
+          <t>director, secretary</t>
         </is>
       </c>
       <c r="E148" s="3" t="inlineStr">
@@ -5897,19 +5897,19 @@
       </c>
       <c r="G148" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Spring menu roles include: manufacturer, agency, finance, iame, reviewer, programme, director, secretary. Capabilities today: List the applications waiting for you; Open the screen where each is done.</t>
+          <t>Runtime screen (not in the 141-screen catalogue). Capabilities: List the applications waiting for your decision; Open the approval screen.</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="3" t="inlineStr">
         <is>
-          <t>workflow/team-queue</t>
+          <t>workflow/personal-inbox</t>
         </is>
       </c>
       <c r="B149" s="3" t="inlineStr">
         <is>
-          <t>Team queue</t>
+          <t>Personal inbox</t>
         </is>
       </c>
       <c r="C149" s="3" t="inlineStr">
@@ -5924,52 +5924,89 @@
       </c>
       <c r="E149" s="3" t="inlineStr">
         <is>
-          <t>Prototype (preview/sample data)</t>
+          <t>Live – BEE service</t>
         </is>
       </c>
       <c r="F149" s="3" t="inlineStr">
         <is>
-          <t>merge</t>
+          <t>keep</t>
         </is>
       </c>
       <c r="G149" s="3" t="inlineStr">
         <is>
-          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+          <t xml:space="preserve"> Spring menu roles include: manufacturer, agency, finance, iame, reviewer, programme, director, secretary. Capabilities today: List the applications waiting for you; Open the screen where each is done.</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="3" t="inlineStr">
         <is>
+          <t>workflow/team-queue</t>
+        </is>
+      </c>
+      <c r="B150" s="3" t="inlineStr">
+        <is>
+          <t>Team queue</t>
+        </is>
+      </c>
+      <c r="C150" s="3" t="inlineStr">
+        <is>
+          <t>Workflow</t>
+        </is>
+      </c>
+      <c r="D150" s="3" t="inlineStr">
+        <is>
+          <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
+        </is>
+      </c>
+      <c r="E150" s="3" t="inlineStr">
+        <is>
+          <t>Prototype (preview/sample data)</t>
+        </is>
+      </c>
+      <c r="F150" s="3" t="inlineStr">
+        <is>
+          <t>merge</t>
+        </is>
+      </c>
+      <c r="G150" s="3" t="inlineStr">
+        <is>
+          <t>Catalogue / preview screen; not wired to the live BEE service list for this feature.</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="3" t="inlineStr">
+        <is>
           <t>workflow/workflow-history</t>
         </is>
       </c>
-      <c r="B150" s="3" t="inlineStr">
+      <c r="B151" s="3" t="inlineStr">
         <is>
           <t>Workflow history</t>
         </is>
       </c>
-      <c r="C150" s="3" t="inlineStr">
+      <c r="C151" s="3" t="inlineStr">
         <is>
           <t>Workflow</t>
         </is>
       </c>
-      <c r="D150" s="3" t="inlineStr">
+      <c r="D151" s="3" t="inlineStr">
         <is>
           <t>BEE Admin, Programme, Reviewer, Director, Secretary, Auditor</t>
         </is>
       </c>
-      <c r="E150" s="3" t="inlineStr">
+      <c r="E151" s="3" t="inlineStr">
         <is>
           <t>Live – BEE service</t>
         </is>
       </c>
-      <c r="F150" s="3" t="inlineStr">
-        <is>
-          <t>merge</t>
-        </is>
-      </c>
-      <c r="G150" s="3" t="inlineStr">
+      <c r="F151" s="3" t="inlineStr">
+        <is>
+          <t>merge</t>
+        </is>
+      </c>
+      <c r="G151" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve"> Spring menu by role or permission. Capabilities today: Choose an application; Read its steps as you are allowed to see them.</t>
         </is>
@@ -6419,11 +6456,11 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="18">

</xml_diff>

<commit_message>
WP02 accepted as a local package: gate 2175/0 recorded; workbook
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/BEE-portal-status.xlsx
+++ b/docs/tracking/BEE-portal-status.xlsx
@@ -6476,16 +6476,16 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Identity, session, MFA, model-application policy</t>
+          <t>Identity, session, MFA, delegation, policy (package accepted 14 Oct 2026; escalation R12 waits for BEE B14)</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E18" s="3" t="n">
-        <v>92</v>
+        <v>100</v>
       </c>
     </row>
     <row r="19">

</xml_diff>

<commit_message>
WP02 package review: corrections, a second denial matrix, WP02 accepted as a local package (#56)
* WP02 package review: corrections (acceptance map, policy and MFA notes, plan, denial evidence incl. a matrix over the other routes), BL-200..204

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

* WP02 package review fixes: an entitled writer is not exercised, the delegation request joins the matrix, stale status lines, counts

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

* WP02 accepted as a local package: gate 2175/0 recorded; workbook

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

---------

Co-authored-by: Sameer Khanna <sameerkhanna@Sameers-MacBook-Pro.local>
Co-authored-by: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/BEE-portal-status.xlsx
+++ b/docs/tracking/BEE-portal-status.xlsx
@@ -6476,16 +6476,16 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Identity, session, MFA, model-application policy</t>
+          <t>Identity, session, MFA, delegation, policy (package accepted 14 Oct 2026; escalation R12 waits for BEE B14)</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E18" s="3" t="n">
-        <v>92</v>
+        <v>100</v>
       </c>
     </row>
     <row r="19">

</xml_diff>

<commit_message>
WP05 package review: scope reconciled, resubmit snapshot, model-application guard (V51), intake accessibility, stale text; WP05 accepted
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/BEE-portal-status.xlsx
+++ b/docs/tracking/BEE-portal-status.xlsx
@@ -6026,7 +6026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6601,7 +6601,7 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>OpenAPI contract, BFF, contract tests</t>
+          <t>OpenAPI contract, BFF, contract tests (package accepted 14 Oct 2026)</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -6871,12 +6871,12 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>WP06.1a</t>
+          <t>WP05</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Document intake and storage</t>
+          <t>Package review: model application intake, evidence, fee and state (rating formula placeholder; renewal not built)</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -6896,21 +6896,21 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>WP06.2</t>
+          <t>WP06.1a</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Blob retention, orphans, limits (BL-001–003)</t>
+          <t>Document intake and storage</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E35" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="36">
@@ -6921,21 +6921,21 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>WP07.1a</t>
+          <t>WP06.2</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Finance fee confirmation</t>
+          <t>Blob retention, orphans, limits (BL-001–003)</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E36" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -6946,12 +6946,12 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>WP07.1b–f</t>
+          <t>WP07.1a</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>IAME, Reviewer, Rating, Director, Secretary stages</t>
+          <t>Finance fee confirmation</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -6971,12 +6971,12 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>WP07.1g–h</t>
+          <t>WP07.1b–f</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Return, resubmit, rejection</t>
+          <t>IAME, Reviewer, Rating, Director, Secretary stages</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -6996,12 +6996,12 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>WP07.1i–k</t>
+          <t>WP07.1g–h</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>History, inbox, workflow views</t>
+          <t>Return, resubmit, rejection</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -7021,12 +7021,12 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>WP08.1a</t>
+          <t>WP07.1i–k</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Fee rule administration</t>
+          <t>History, inbox, workflow views</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -7046,12 +7046,12 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>WP08.1b</t>
+          <t>WP08.1a</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Tax line on fee rules</t>
+          <t>Fee rule administration</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -7071,12 +7071,12 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>WP08.1c</t>
+          <t>WP08.1b</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Rating schemes administration</t>
+          <t>Tax line on fee rules</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -7096,12 +7096,12 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>WP08.1d</t>
+          <t>WP08.1c</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Permission-based admin menu</t>
+          <t>Rating schemes administration</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -7121,12 +7121,12 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>WP08.1e</t>
+          <t>WP08.1d</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Fee confirmation correction proposals</t>
+          <t>Permission-based admin menu</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -7146,12 +7146,12 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>WP08.1f</t>
+          <t>WP08.1e</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Fee reversal</t>
+          <t>Fee confirmation correction proposals</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -7171,12 +7171,12 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>WP08.1g</t>
+          <t>WP08.1f</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Born-pending and notification proof</t>
+          <t>Fee reversal</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -7196,12 +7196,12 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>WP08.1h</t>
+          <t>WP08.1g</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Business settings (propose/approve numbers)</t>
+          <t>Born-pending and notification proof</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
@@ -7221,12 +7221,12 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>WP09.1a</t>
+          <t>WP08.1h</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Certificate record</t>
+          <t>Business settings (propose/approve numbers)</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
@@ -7246,12 +7246,12 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>WP09.1b</t>
+          <t>WP09.1a</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Printable certificate and label</t>
+          <t>Certificate record</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -7271,12 +7271,12 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>WP09.1c</t>
+          <t>WP09.1b</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Public verification page</t>
+          <t>Printable certificate and label</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
@@ -7296,12 +7296,12 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>WP09.1d</t>
+          <t>WP09.1c</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Verification rate limit</t>
+          <t>Public verification page</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -7321,12 +7321,12 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>WP10.1a</t>
+          <t>WP09.1d</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>In-portal notifications (API)</t>
+          <t>Verification rate limit</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -7346,12 +7346,12 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>WP10.1b</t>
+          <t>WP10.1a</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Notification bell and page</t>
+          <t>In-portal notifications (API)</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
@@ -7371,71 +7371,71 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>WP11</t>
+          <t>WP10.1b</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>AI demonstrations (local)</t>
+          <t>Notification bell and page</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E54" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>Platform</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>WP01</t>
+          <t>WP11</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Documentation and design evidence</t>
+          <t>AI demonstrations (local)</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E55" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>Backlog theme</t>
+          <t>Platform</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>BL-024/025</t>
+          <t>WP01</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>Feature template and OpenAPI split</t>
+          <t>Documentation and design evidence</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E56" s="3" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
     </row>
     <row r="57">
@@ -7446,45 +7446,70 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>BL-040–042</t>
+          <t>BL-024/025</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+          <t>Feature template and OpenAPI split</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="E57" s="3" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
+          <t>Backlog theme</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>BL-040–042</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
           <t>Owner decision</t>
         </is>
       </c>
-      <c r="B58" s="3" t="inlineStr">
+      <c r="B59" s="3" t="inlineStr">
         <is>
           <t>D10</t>
         </is>
       </c>
-      <c r="C58" s="3" t="inlineStr">
+      <c r="C59" s="3" t="inlineStr">
         <is>
           <t>Provisional local rules for notifications (portal only)</t>
         </is>
       </c>
-      <c r="D58" s="3" t="inlineStr">
+      <c r="D59" s="3" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
-      <c r="E58" s="3" t="n">
+      <c r="E59" s="3" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
WP05 package review: scope reconciled, resubmit snapshot, model-application guard (V51), intake accessibility, stale text; WP05 accepted (#58)
Co-authored-by: Sameer Khanna <sameerkhanna@Sameers-MacBook-Pro.local>
Co-authored-by: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/BEE-portal-status.xlsx
+++ b/docs/tracking/BEE-portal-status.xlsx
@@ -6026,7 +6026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E58"/>
+  <dimension ref="A1:E59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6601,7 +6601,7 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>OpenAPI contract, BFF, contract tests</t>
+          <t>OpenAPI contract, BFF, contract tests (package accepted 14 Oct 2026)</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -6871,12 +6871,12 @@
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>WP06.1a</t>
+          <t>WP05</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Document intake and storage</t>
+          <t>Package review: model application intake, evidence, fee and state (rating formula placeholder; renewal not built)</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -6896,21 +6896,21 @@
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>WP06.2</t>
+          <t>WP06.1a</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Blob retention, orphans, limits (BL-001–003)</t>
+          <t>Document intake and storage</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E35" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="36">
@@ -6921,21 +6921,21 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>WP07.1a</t>
+          <t>WP06.2</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Finance fee confirmation</t>
+          <t>Blob retention, orphans, limits (BL-001–003)</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E36" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
@@ -6946,12 +6946,12 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>WP07.1b–f</t>
+          <t>WP07.1a</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>IAME, Reviewer, Rating, Director, Secretary stages</t>
+          <t>Finance fee confirmation</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -6971,12 +6971,12 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>WP07.1g–h</t>
+          <t>WP07.1b–f</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Return, resubmit, rejection</t>
+          <t>IAME, Reviewer, Rating, Director, Secretary stages</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -6996,12 +6996,12 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>WP07.1i–k</t>
+          <t>WP07.1g–h</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>History, inbox, workflow views</t>
+          <t>Return, resubmit, rejection</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -7021,12 +7021,12 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>WP08.1a</t>
+          <t>WP07.1i–k</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Fee rule administration</t>
+          <t>History, inbox, workflow views</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -7046,12 +7046,12 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>WP08.1b</t>
+          <t>WP08.1a</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Tax line on fee rules</t>
+          <t>Fee rule administration</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -7071,12 +7071,12 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>WP08.1c</t>
+          <t>WP08.1b</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Rating schemes administration</t>
+          <t>Tax line on fee rules</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -7096,12 +7096,12 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>WP08.1d</t>
+          <t>WP08.1c</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Permission-based admin menu</t>
+          <t>Rating schemes administration</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -7121,12 +7121,12 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>WP08.1e</t>
+          <t>WP08.1d</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Fee confirmation correction proposals</t>
+          <t>Permission-based admin menu</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -7146,12 +7146,12 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>WP08.1f</t>
+          <t>WP08.1e</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Fee reversal</t>
+          <t>Fee confirmation correction proposals</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -7171,12 +7171,12 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>WP08.1g</t>
+          <t>WP08.1f</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Born-pending and notification proof</t>
+          <t>Fee reversal</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -7196,12 +7196,12 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>WP08.1h</t>
+          <t>WP08.1g</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Business settings (propose/approve numbers)</t>
+          <t>Born-pending and notification proof</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
@@ -7221,12 +7221,12 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>WP09.1a</t>
+          <t>WP08.1h</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Certificate record</t>
+          <t>Business settings (propose/approve numbers)</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
@@ -7246,12 +7246,12 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>WP09.1b</t>
+          <t>WP09.1a</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Printable certificate and label</t>
+          <t>Certificate record</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -7271,12 +7271,12 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>WP09.1c</t>
+          <t>WP09.1b</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Public verification page</t>
+          <t>Printable certificate and label</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
@@ -7296,12 +7296,12 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>WP09.1d</t>
+          <t>WP09.1c</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Verification rate limit</t>
+          <t>Public verification page</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -7321,12 +7321,12 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>WP10.1a</t>
+          <t>WP09.1d</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>In-portal notifications (API)</t>
+          <t>Verification rate limit</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -7346,12 +7346,12 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>WP10.1b</t>
+          <t>WP10.1a</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Notification bell and page</t>
+          <t>In-portal notifications (API)</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
@@ -7371,71 +7371,71 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>WP11</t>
+          <t>WP10.1b</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>AI demonstrations (local)</t>
+          <t>Notification bell and page</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E54" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>Platform</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>WP01</t>
+          <t>WP11</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Documentation and design evidence</t>
+          <t>AI demonstrations (local)</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E55" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>Backlog theme</t>
+          <t>Platform</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>BL-024/025</t>
+          <t>WP01</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>Feature template and OpenAPI split</t>
+          <t>Documentation and design evidence</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E56" s="3" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
     </row>
     <row r="57">
@@ -7446,45 +7446,70 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>BL-040–042</t>
+          <t>BL-024/025</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+          <t>Feature template and OpenAPI split</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="E57" s="3" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
+          <t>Backlog theme</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>BL-040–042</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
+        <is>
           <t>Owner decision</t>
         </is>
       </c>
-      <c r="B58" s="3" t="inlineStr">
+      <c r="B59" s="3" t="inlineStr">
         <is>
           <t>D10</t>
         </is>
       </c>
-      <c r="C58" s="3" t="inlineStr">
+      <c r="C59" s="3" t="inlineStr">
         <is>
           <t>Provisional local rules for notifications (portal only)</t>
         </is>
       </c>
-      <c r="D58" s="3" t="inlineStr">
+      <c r="D59" s="3" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
-      <c r="E58" s="3" t="n">
+      <c r="E59" s="3" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Count WP06 and WP07 on narrowed scopes (7/11) at the owner's direction
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/BEE-portal-status.xlsx
+++ b/docs/tracking/BEE-portal-status.xlsx
@@ -6026,7 +6026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6921,21 +6921,21 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>WP06.2</t>
+          <t>WP06</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Blob retention, orphans, limits (BL-001–003)</t>
+          <t>Package review: accepted on narrowed scope (test-report intake, versions, scoped retrieval for drafts)</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E36" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="37">
@@ -6946,21 +6946,21 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>WP07.1a</t>
+          <t>WP06.2</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Finance fee confirmation</t>
+          <t>Blob retention, orphans, limits (BL-001–003)</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E37" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
@@ -6971,12 +6971,12 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>WP07.1b–f</t>
+          <t>WP07</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>IAME, Reviewer, Rating, Director, Secretary stages</t>
+          <t>Package review: accepted on narrowed scope (stage workflow, manual fee confirmation/correction/reversal); payment simulation, production, CA not built</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -6996,12 +6996,12 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>WP07.1g–h</t>
+          <t>WP07.1a</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Return, resubmit, rejection</t>
+          <t>Finance fee confirmation</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -7021,12 +7021,12 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>WP07.1i–k</t>
+          <t>WP07.1b–f</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>History, inbox, workflow views</t>
+          <t>IAME, Reviewer, Rating, Director, Secretary stages</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -7046,12 +7046,12 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>WP08.1a</t>
+          <t>WP07.1g–h</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Fee rule administration</t>
+          <t>Return, resubmit, rejection</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -7071,12 +7071,12 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>WP08.1b</t>
+          <t>WP07.1i–k</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Tax line on fee rules</t>
+          <t>History, inbox, workflow views</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -7096,12 +7096,12 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>WP08.1c</t>
+          <t>WP08.1a</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Rating schemes administration</t>
+          <t>Fee rule administration</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -7121,12 +7121,12 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>WP08.1d</t>
+          <t>WP08.1b</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Permission-based admin menu</t>
+          <t>Tax line on fee rules</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -7146,12 +7146,12 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>WP08.1e</t>
+          <t>WP08.1c</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Fee confirmation correction proposals</t>
+          <t>Rating schemes administration</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -7171,12 +7171,12 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>WP08.1f</t>
+          <t>WP08.1d</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Fee reversal</t>
+          <t>Permission-based admin menu</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -7196,12 +7196,12 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>WP08.1g</t>
+          <t>WP08.1e</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Born-pending and notification proof</t>
+          <t>Fee confirmation correction proposals</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
@@ -7221,12 +7221,12 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>WP08.1h</t>
+          <t>WP08.1f</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Business settings (propose/approve numbers)</t>
+          <t>Fee reversal</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
@@ -7246,12 +7246,12 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>WP09.1a</t>
+          <t>WP08.1g</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Certificate record</t>
+          <t>Born-pending and notification proof</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -7271,12 +7271,12 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>WP09.1b</t>
+          <t>WP08.1h</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Printable certificate and label</t>
+          <t>Business settings (propose/approve numbers)</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
@@ -7296,12 +7296,12 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>WP09.1c</t>
+          <t>WP09.1a</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Public verification page</t>
+          <t>Certificate record</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -7321,12 +7321,12 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>WP09.1d</t>
+          <t>WP09.1b</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Verification rate limit</t>
+          <t>Printable certificate and label</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -7346,12 +7346,12 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>WP10.1a</t>
+          <t>WP09.1c</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>In-portal notifications (API)</t>
+          <t>Public verification page</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
@@ -7371,12 +7371,12 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>WP10.1b</t>
+          <t>WP09.1d</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Notification bell and page</t>
+          <t>Verification rate limit</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
@@ -7396,37 +7396,37 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>WP11</t>
+          <t>WP10.1a</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>AI demonstrations (local)</t>
+          <t>In-portal notifications (API)</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E55" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>Platform</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>WP01</t>
+          <t>WP10.1b</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>Documentation and design evidence</t>
+          <t>Notification bell and page</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
@@ -7441,75 +7441,125 @@
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>Backlog theme</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>BL-024/025</t>
+          <t>WP11</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Feature template and OpenAPI split</t>
+          <t>AI demonstrations (local)</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E57" s="3" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>Backlog theme</t>
+          <t>Platform</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>BL-040–042</t>
+          <t>WP01</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+          <t>Documentation and design evidence</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E58" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
+          <t>Backlog theme</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>BL-024/025</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>Feature template and OpenAPI split</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>Backlog theme</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>BL-040–042</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
           <t>Owner decision</t>
         </is>
       </c>
-      <c r="B59" s="3" t="inlineStr">
+      <c r="B61" s="3" t="inlineStr">
         <is>
           <t>D10</t>
         </is>
       </c>
-      <c r="C59" s="3" t="inlineStr">
+      <c r="C61" s="3" t="inlineStr">
         <is>
           <t>Provisional local rules for notifications (portal only)</t>
         </is>
       </c>
-      <c r="D59" s="3" t="inlineStr">
+      <c r="D61" s="3" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
-      <c r="E59" s="3" t="n">
+      <c r="E61" s="3" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
WP06 to WP11 package review: WP06 and WP07 accepted on narrowed scopes (7/11) (#59)
* Package review of WP06 to WP11: none accepted, count stays 5/11; findings, reconciliation, BL-210 to BL-218

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

* Count WP06 and WP07 on narrowed scopes (7/11) at the owner's direction

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

---------

Co-authored-by: Sameer Khanna <sameerkhanna@Sameers-MacBook-Pro.local>
Co-authored-by: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/BEE-portal-status.xlsx
+++ b/docs/tracking/BEE-portal-status.xlsx
@@ -6026,7 +6026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E59"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6921,21 +6921,21 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>WP06.2</t>
+          <t>WP06</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Blob retention, orphans, limits (BL-001–003)</t>
+          <t>Package review: accepted on narrowed scope (test-report intake, versions, scoped retrieval for drafts)</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E36" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="37">
@@ -6946,21 +6946,21 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>WP07.1a</t>
+          <t>WP06.2</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Finance fee confirmation</t>
+          <t>Blob retention, orphans, limits (BL-001–003)</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E37" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
@@ -6971,12 +6971,12 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>WP07.1b–f</t>
+          <t>WP07</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>IAME, Reviewer, Rating, Director, Secretary stages</t>
+          <t>Package review: accepted on narrowed scope (stage workflow, manual fee confirmation/correction/reversal); payment simulation, production, CA not built</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
@@ -6996,12 +6996,12 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>WP07.1g–h</t>
+          <t>WP07.1a</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Return, resubmit, rejection</t>
+          <t>Finance fee confirmation</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -7021,12 +7021,12 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>WP07.1i–k</t>
+          <t>WP07.1b–f</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>History, inbox, workflow views</t>
+          <t>IAME, Reviewer, Rating, Director, Secretary stages</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -7046,12 +7046,12 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>WP08.1a</t>
+          <t>WP07.1g–h</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Fee rule administration</t>
+          <t>Return, resubmit, rejection</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -7071,12 +7071,12 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>WP08.1b</t>
+          <t>WP07.1i–k</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Tax line on fee rules</t>
+          <t>History, inbox, workflow views</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -7096,12 +7096,12 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>WP08.1c</t>
+          <t>WP08.1a</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Rating schemes administration</t>
+          <t>Fee rule administration</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -7121,12 +7121,12 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>WP08.1d</t>
+          <t>WP08.1b</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Permission-based admin menu</t>
+          <t>Tax line on fee rules</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -7146,12 +7146,12 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>WP08.1e</t>
+          <t>WP08.1c</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Fee confirmation correction proposals</t>
+          <t>Rating schemes administration</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -7171,12 +7171,12 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>WP08.1f</t>
+          <t>WP08.1d</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Fee reversal</t>
+          <t>Permission-based admin menu</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -7196,12 +7196,12 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>WP08.1g</t>
+          <t>WP08.1e</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Born-pending and notification proof</t>
+          <t>Fee confirmation correction proposals</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
@@ -7221,12 +7221,12 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>WP08.1h</t>
+          <t>WP08.1f</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Business settings (propose/approve numbers)</t>
+          <t>Fee reversal</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
@@ -7246,12 +7246,12 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>WP09.1a</t>
+          <t>WP08.1g</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Certificate record</t>
+          <t>Born-pending and notification proof</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -7271,12 +7271,12 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>WP09.1b</t>
+          <t>WP08.1h</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Printable certificate and label</t>
+          <t>Business settings (propose/approve numbers)</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
@@ -7296,12 +7296,12 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>WP09.1c</t>
+          <t>WP09.1a</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Public verification page</t>
+          <t>Certificate record</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -7321,12 +7321,12 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>WP09.1d</t>
+          <t>WP09.1b</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Verification rate limit</t>
+          <t>Printable certificate and label</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -7346,12 +7346,12 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>WP10.1a</t>
+          <t>WP09.1c</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>In-portal notifications (API)</t>
+          <t>Public verification page</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
@@ -7371,12 +7371,12 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>WP10.1b</t>
+          <t>WP09.1d</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Notification bell and page</t>
+          <t>Verification rate limit</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
@@ -7396,37 +7396,37 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>WP11</t>
+          <t>WP10.1a</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>AI demonstrations (local)</t>
+          <t>In-portal notifications (API)</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E55" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>Platform</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>WP01</t>
+          <t>WP10.1b</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>Documentation and design evidence</t>
+          <t>Notification bell and page</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
@@ -7441,75 +7441,125 @@
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>Backlog theme</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>BL-024/025</t>
+          <t>WP11</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Feature template and OpenAPI split</t>
+          <t>AI demonstrations (local)</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E57" s="3" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>Backlog theme</t>
+          <t>Platform</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>BL-040–042</t>
+          <t>WP01</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+          <t>Documentation and design evidence</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E58" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
+          <t>Backlog theme</t>
+        </is>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>BL-024/025</t>
+        </is>
+      </c>
+      <c r="C59" s="3" t="inlineStr">
+        <is>
+          <t>Feature template and OpenAPI split</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>Backlog theme</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>BL-040–042</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="3" t="inlineStr">
+        <is>
           <t>Owner decision</t>
         </is>
       </c>
-      <c r="B59" s="3" t="inlineStr">
+      <c r="B61" s="3" t="inlineStr">
         <is>
           <t>D10</t>
         </is>
       </c>
-      <c r="C59" s="3" t="inlineStr">
+      <c r="C61" s="3" t="inlineStr">
         <is>
           <t>Provisional local rules for notifications (portal only)</t>
         </is>
       </c>
-      <c r="D59" s="3" t="inlineStr">
+      <c r="D61" s="3" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
-      <c r="E59" s="3" t="n">
+      <c r="E61" s="3" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Workbook: hardening row and the unbuilt WP07 to WP10 scope
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/BEE-portal-status.xlsx
+++ b/docs/tracking/BEE-portal-status.xlsx
@@ -6026,7 +6026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6946,21 +6946,21 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>WP06.2</t>
+          <t>HARDEN-1</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Blob retention, orphans, limits (BL-001–003)</t>
+          <t>Review hardening: nosniff on PDF downloads, /verify status region, certificate heading, two repaired WebMvc test classes (BL-216 to BL-219)</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E37" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="38">
@@ -6971,21 +6971,21 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>WP07</t>
+          <t>WP06.2</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Package review: accepted on narrowed scope (stage workflow, manual fee confirmation/correction/reversal); payment simulation, production, CA not built</t>
+          <t>Blob retention, orphans, limits (BL-001–003)</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E38" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -6996,12 +6996,12 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>WP07.1a</t>
+          <t>WP07</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Finance fee confirmation</t>
+          <t>Package review: accepted on narrowed scope (stage workflow, manual fee confirmation/correction/reversal); payment simulation, production, CA not built</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -7021,12 +7021,12 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>WP07.1b–f</t>
+          <t>WP07.1a</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>IAME, Reviewer, Rating, Director, Secretary stages</t>
+          <t>Finance fee confirmation</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -7046,12 +7046,12 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>WP07.1g–h</t>
+          <t>WP07.1b–f</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Return, resubmit, rejection</t>
+          <t>IAME, Reviewer, Rating, Director, Secretary stages</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -7071,12 +7071,12 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>WP07.1i–k</t>
+          <t>WP07.1g–h</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>History, inbox, workflow views</t>
+          <t>Return, resubmit, rejection</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -7096,12 +7096,12 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>WP08.1a</t>
+          <t>WP07.1i–k</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Fee rule administration</t>
+          <t>History, inbox, workflow views</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -7121,12 +7121,12 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>WP08.1b</t>
+          <t>WP08.1a</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Tax line on fee rules</t>
+          <t>Fee rule administration</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -7146,12 +7146,12 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>WP08.1c</t>
+          <t>WP08.1b</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Rating schemes administration</t>
+          <t>Tax line on fee rules</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -7171,12 +7171,12 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>WP08.1d</t>
+          <t>WP08.1c</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Permission-based admin menu</t>
+          <t>Rating schemes administration</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -7196,12 +7196,12 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>WP08.1e</t>
+          <t>WP08.1d</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Fee confirmation correction proposals</t>
+          <t>Permission-based admin menu</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
@@ -7221,12 +7221,12 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>WP08.1f</t>
+          <t>WP08.1e</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Fee reversal</t>
+          <t>Fee confirmation correction proposals</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
@@ -7246,12 +7246,12 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>WP08.1g</t>
+          <t>WP08.1f</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Born-pending and notification proof</t>
+          <t>Fee reversal</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -7271,12 +7271,12 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>WP08.1h</t>
+          <t>WP08.1g</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Business settings (propose/approve numbers)</t>
+          <t>Born-pending and notification proof</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
@@ -7296,12 +7296,12 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>WP09.1a</t>
+          <t>WP08.1h</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Certificate record</t>
+          <t>Business settings (propose/approve numbers)</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -7321,12 +7321,12 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>WP09.1b</t>
+          <t>WP09.1a</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Printable certificate and label</t>
+          <t>Certificate record</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -7346,12 +7346,12 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>WP09.1c</t>
+          <t>WP09.1b</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Public verification page</t>
+          <t>Printable certificate and label</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
@@ -7371,12 +7371,12 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>WP09.1d</t>
+          <t>WP09.1c</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Verification rate limit</t>
+          <t>Public verification page</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
@@ -7396,12 +7396,12 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>WP10.1a</t>
+          <t>WP09.1d</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>In-portal notifications (API)</t>
+          <t>Verification rate limit</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
@@ -7421,12 +7421,12 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>WP10.1b</t>
+          <t>WP10.1a</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>Notification bell and page</t>
+          <t>In-portal notifications (API)</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
@@ -7446,92 +7446,92 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>WP11</t>
+          <t>WP10.1b</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>AI demonstrations (local)</t>
+          <t>Notification bell and page</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E57" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>Platform</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>WP01</t>
+          <t>WP11</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>Documentation and design evidence</t>
+          <t>AI demonstrations (local)</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E58" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>Backlog theme</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>BL-024/025</t>
+          <t>WP07.x</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>Feature template and OpenAPI split</t>
+          <t>Payment simulation, reconciliation, production, bulk, CA evidence, refunds (BL-211)</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E59" s="3" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>Backlog theme</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>BL-040–042</t>
+          <t>WP08.x</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+          <t>QR batch, serial and duplicate control (BL-212); package not accepted</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E60" s="3" t="n">
@@ -7541,25 +7541,150 @@
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
+          <t>Work package</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>WP09.x</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>Fabric adapter, hash proof, pending/amend/revoke (BL-213); package not accepted</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>Work package</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>WP10.x</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>Cases, sampling, partner assignment, tickets (BL-214); package not accepted</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>WP01</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>Documentation and design evidence</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>Backlog theme</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>BL-024/025</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>Feature template and OpenAPI split</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>Backlog theme</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>BL-040–042</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
           <t>Owner decision</t>
         </is>
       </c>
-      <c r="B61" s="3" t="inlineStr">
+      <c r="B66" s="3" t="inlineStr">
         <is>
           <t>D10</t>
         </is>
       </c>
-      <c r="C61" s="3" t="inlineStr">
+      <c r="C66" s="3" t="inlineStr">
         <is>
           <t>Provisional local rules for notifications (portal only)</t>
         </is>
       </c>
-      <c r="D61" s="3" t="inlineStr">
+      <c r="D66" s="3" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
-      <c r="E61" s="3" t="n">
+      <c r="E66" s="3" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Hardening from the WP06 to WP11 review; fix two broken WebMvc tests (#60)
* Hardening from the WP06 to WP11 review: nosniff on PDF downloads, verify result as status region, certificate heading; fix two broken WebMvc tests; BL-216/217/218/219

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

* Workbook: hardening row and the unbuilt WP07 to WP10 scope

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>

---------

Co-authored-by: Sameer Khanna <sameerkhanna@Sameers-MacBook-Pro.local>
Co-authored-by: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/BEE-portal-status.xlsx
+++ b/docs/tracking/BEE-portal-status.xlsx
@@ -6026,7 +6026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6946,21 +6946,21 @@
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>WP06.2</t>
+          <t>HARDEN-1</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Blob retention, orphans, limits (BL-001–003)</t>
+          <t>Review hardening: nosniff on PDF downloads, /verify status region, certificate heading, two repaired WebMvc test classes (BL-216 to BL-219)</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E37" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="38">
@@ -6971,21 +6971,21 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>WP07</t>
+          <t>WP06.2</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Package review: accepted on narrowed scope (stage workflow, manual fee confirmation/correction/reversal); payment simulation, production, CA not built</t>
+          <t>Blob retention, orphans, limits (BL-001–003)</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E38" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="39">
@@ -6996,12 +6996,12 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>WP07.1a</t>
+          <t>WP07</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Finance fee confirmation</t>
+          <t>Package review: accepted on narrowed scope (stage workflow, manual fee confirmation/correction/reversal); payment simulation, production, CA not built</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -7021,12 +7021,12 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>WP07.1b–f</t>
+          <t>WP07.1a</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>IAME, Reviewer, Rating, Director, Secretary stages</t>
+          <t>Finance fee confirmation</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -7046,12 +7046,12 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>WP07.1g–h</t>
+          <t>WP07.1b–f</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>Return, resubmit, rejection</t>
+          <t>IAME, Reviewer, Rating, Director, Secretary stages</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -7071,12 +7071,12 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>WP07.1i–k</t>
+          <t>WP07.1g–h</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>History, inbox, workflow views</t>
+          <t>Return, resubmit, rejection</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -7096,12 +7096,12 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>WP08.1a</t>
+          <t>WP07.1i–k</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>Fee rule administration</t>
+          <t>History, inbox, workflow views</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -7121,12 +7121,12 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>WP08.1b</t>
+          <t>WP08.1a</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Tax line on fee rules</t>
+          <t>Fee rule administration</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -7146,12 +7146,12 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>WP08.1c</t>
+          <t>WP08.1b</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Rating schemes administration</t>
+          <t>Tax line on fee rules</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -7171,12 +7171,12 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>WP08.1d</t>
+          <t>WP08.1c</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Permission-based admin menu</t>
+          <t>Rating schemes administration</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -7196,12 +7196,12 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>WP08.1e</t>
+          <t>WP08.1d</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Fee confirmation correction proposals</t>
+          <t>Permission-based admin menu</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
@@ -7221,12 +7221,12 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>WP08.1f</t>
+          <t>WP08.1e</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Fee reversal</t>
+          <t>Fee confirmation correction proposals</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
@@ -7246,12 +7246,12 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>WP08.1g</t>
+          <t>WP08.1f</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Born-pending and notification proof</t>
+          <t>Fee reversal</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -7271,12 +7271,12 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>WP08.1h</t>
+          <t>WP08.1g</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Business settings (propose/approve numbers)</t>
+          <t>Born-pending and notification proof</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
@@ -7296,12 +7296,12 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>WP09.1a</t>
+          <t>WP08.1h</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Certificate record</t>
+          <t>Business settings (propose/approve numbers)</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -7321,12 +7321,12 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>WP09.1b</t>
+          <t>WP09.1a</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Printable certificate and label</t>
+          <t>Certificate record</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -7346,12 +7346,12 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>WP09.1c</t>
+          <t>WP09.1b</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Public verification page</t>
+          <t>Printable certificate and label</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
@@ -7371,12 +7371,12 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>WP09.1d</t>
+          <t>WP09.1c</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Verification rate limit</t>
+          <t>Public verification page</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
@@ -7396,12 +7396,12 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>WP10.1a</t>
+          <t>WP09.1d</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>In-portal notifications (API)</t>
+          <t>Verification rate limit</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
@@ -7421,12 +7421,12 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>WP10.1b</t>
+          <t>WP10.1a</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>Notification bell and page</t>
+          <t>In-portal notifications (API)</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
@@ -7446,92 +7446,92 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>WP11</t>
+          <t>WP10.1b</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>AI demonstrations (local)</t>
+          <t>Notification bell and page</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E57" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>Platform</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>WP01</t>
+          <t>WP11</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>Documentation and design evidence</t>
+          <t>AI demonstrations (local)</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E58" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>Backlog theme</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>BL-024/025</t>
+          <t>WP07.x</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>Feature template and OpenAPI split</t>
+          <t>Payment simulation, reconciliation, production, bulk, CA evidence, refunds (BL-211)</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E59" s="3" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>Backlog theme</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>BL-040–042</t>
+          <t>WP08.x</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+          <t>QR batch, serial and duplicate control (BL-212); package not accepted</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E60" s="3" t="n">
@@ -7541,25 +7541,150 @@
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
+          <t>Work package</t>
+        </is>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>WP09.x</t>
+        </is>
+      </c>
+      <c r="C61" s="3" t="inlineStr">
+        <is>
+          <t>Fabric adapter, hash proof, pending/amend/revoke (BL-213); package not accepted</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>Work package</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>WP10.x</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>Cases, sampling, partner assignment, tickets (BL-214); package not accepted</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="B63" s="3" t="inlineStr">
+        <is>
+          <t>WP01</t>
+        </is>
+      </c>
+      <c r="C63" s="3" t="inlineStr">
+        <is>
+          <t>Documentation and design evidence</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>Backlog theme</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>BL-024/025</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>Feature template and OpenAPI split</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="3" t="inlineStr">
+        <is>
+          <t>Backlog theme</t>
+        </is>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>BL-040–042</t>
+        </is>
+      </c>
+      <c r="C65" s="3" t="inlineStr">
+        <is>
+          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
           <t>Owner decision</t>
         </is>
       </c>
-      <c r="B61" s="3" t="inlineStr">
+      <c r="B66" s="3" t="inlineStr">
         <is>
           <t>D10</t>
         </is>
       </c>
-      <c r="C61" s="3" t="inlineStr">
+      <c r="C66" s="3" t="inlineStr">
         <is>
           <t>Provisional local rules for notifications (portal only)</t>
         </is>
       </c>
-      <c r="D61" s="3" t="inlineStr">
+      <c r="D66" s="3" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
-      <c r="E61" s="3" t="n">
+      <c r="E66" s="3" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Demo Phase 0: /api/demo dispatcher (DemoModule), BFF catch-all, demo client, placeholder screens and menu entries, BL-220
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/BEE-portal-status.xlsx
+++ b/docs/tracking/BEE-portal-status.xlsx
@@ -6026,7 +6026,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E66"/>
+  <dimension ref="A1:E67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -6971,21 +6971,21 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>WP06.2</t>
+          <t>BL-219</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Blob retention, orphans, limits (BL-001–003)</t>
+          <t>Gate runs the default backend suite (backend.unit-tests); gate 2176 passed, 0 failed</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E38" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="39">
@@ -6996,21 +6996,21 @@
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>WP07</t>
+          <t>WP06.2</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Package review: accepted on narrowed scope (stage workflow, manual fee confirmation/correction/reversal); payment simulation, production, CA not built</t>
+          <t>Blob retention, orphans, limits (BL-001–003)</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E39" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40">
@@ -7021,12 +7021,12 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>WP07.1a</t>
+          <t>WP07</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>Finance fee confirmation</t>
+          <t>Package review: accepted on narrowed scope (stage workflow, manual fee confirmation/correction/reversal); payment simulation, production, CA not built</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
@@ -7046,12 +7046,12 @@
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>WP07.1b–f</t>
+          <t>WP07.1a</t>
         </is>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>IAME, Reviewer, Rating, Director, Secretary stages</t>
+          <t>Finance fee confirmation</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
@@ -7071,12 +7071,12 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>WP07.1g–h</t>
+          <t>WP07.1b–f</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Return, resubmit, rejection</t>
+          <t>IAME, Reviewer, Rating, Director, Secretary stages</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
@@ -7096,12 +7096,12 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>WP07.1i–k</t>
+          <t>WP07.1g–h</t>
         </is>
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>History, inbox, workflow views</t>
+          <t>Return, resubmit, rejection</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
@@ -7121,12 +7121,12 @@
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>WP08.1a</t>
+          <t>WP07.1i–k</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>Fee rule administration</t>
+          <t>History, inbox, workflow views</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
@@ -7146,12 +7146,12 @@
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>WP08.1b</t>
+          <t>WP08.1a</t>
         </is>
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>Tax line on fee rules</t>
+          <t>Fee rule administration</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
@@ -7171,12 +7171,12 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>WP08.1c</t>
+          <t>WP08.1b</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>Rating schemes administration</t>
+          <t>Tax line on fee rules</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
@@ -7196,12 +7196,12 @@
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>WP08.1d</t>
+          <t>WP08.1c</t>
         </is>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>Permission-based admin menu</t>
+          <t>Rating schemes administration</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
@@ -7221,12 +7221,12 @@
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>WP08.1e</t>
+          <t>WP08.1d</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Fee confirmation correction proposals</t>
+          <t>Permission-based admin menu</t>
         </is>
       </c>
       <c r="D48" s="3" t="inlineStr">
@@ -7246,12 +7246,12 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>WP08.1f</t>
+          <t>WP08.1e</t>
         </is>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>Fee reversal</t>
+          <t>Fee confirmation correction proposals</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
@@ -7271,12 +7271,12 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>WP08.1g</t>
+          <t>WP08.1f</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>Born-pending and notification proof</t>
+          <t>Fee reversal</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
@@ -7296,12 +7296,12 @@
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>WP08.1h</t>
+          <t>WP08.1g</t>
         </is>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>Business settings (propose/approve numbers)</t>
+          <t>Born-pending and notification proof</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
@@ -7321,12 +7321,12 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>WP09.1a</t>
+          <t>WP08.1h</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>Certificate record</t>
+          <t>Business settings (propose/approve numbers)</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
@@ -7346,12 +7346,12 @@
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>WP09.1b</t>
+          <t>WP09.1a</t>
         </is>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
-          <t>Printable certificate and label</t>
+          <t>Certificate record</t>
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr">
@@ -7371,12 +7371,12 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>WP09.1c</t>
+          <t>WP09.1b</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>Public verification page</t>
+          <t>Printable certificate and label</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
@@ -7396,12 +7396,12 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>WP09.1d</t>
+          <t>WP09.1c</t>
         </is>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>Verification rate limit</t>
+          <t>Public verification page</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
@@ -7421,12 +7421,12 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>WP10.1a</t>
+          <t>WP09.1d</t>
         </is>
       </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
-          <t>In-portal notifications (API)</t>
+          <t>Verification rate limit</t>
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr">
@@ -7446,12 +7446,12 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>WP10.1b</t>
+          <t>WP10.1a</t>
         </is>
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>Notification bell and page</t>
+          <t>In-portal notifications (API)</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
@@ -7471,21 +7471,21 @@
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>WP11</t>
+          <t>WP10.1b</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>AI demonstrations (local)</t>
+          <t>Notification bell and page</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E58" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="59">
@@ -7496,12 +7496,12 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>WP07.x</t>
+          <t>WP11</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>Payment simulation, reconciliation, production, bulk, CA evidence, refunds (BL-211)</t>
+          <t>AI demonstrations (local)</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
@@ -7521,12 +7521,12 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>WP08.x</t>
+          <t>WP07.x</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>QR batch, serial and duplicate control (BL-212); package not accepted</t>
+          <t>Payment simulation, reconciliation, production, bulk, CA evidence, refunds (BL-211)</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
@@ -7546,12 +7546,12 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>WP09.x</t>
+          <t>WP08.x</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>Fabric adapter, hash proof, pending/amend/revoke (BL-213); package not accepted</t>
+          <t>QR batch, serial and duplicate control (BL-212); package not accepted</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
@@ -7571,12 +7571,12 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>WP10.x</t>
+          <t>WP09.x</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>Cases, sampling, partner assignment, tickets (BL-214); package not accepted</t>
+          <t>Fabric adapter, hash proof, pending/amend/revoke (BL-213); package not accepted</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
@@ -7591,51 +7591,51 @@
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>Platform</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>WP01</t>
+          <t>WP10.x</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>Documentation and design evidence</t>
+          <t>Cases, sampling, partner assignment, tickets (BL-214); package not accepted</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Done</t>
+          <t>Not started</t>
         </is>
       </c>
       <c r="E63" s="3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>Backlog theme</t>
+          <t>Platform</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>BL-024/025</t>
+          <t>WP01</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>Feature template and OpenAPI split</t>
+          <t>Documentation and design evidence</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E64" s="3" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
     </row>
     <row r="65">
@@ -7646,45 +7646,70 @@
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>BL-040–042</t>
+          <t>BL-024/025</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+          <t>Feature template and OpenAPI split</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="E65" s="3" t="n">
-        <v>0</v>
+        <v>40</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
+          <t>Backlog theme</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>BL-040–042</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="3" t="inlineStr">
+        <is>
           <t>Owner decision</t>
         </is>
       </c>
-      <c r="B66" s="3" t="inlineStr">
+      <c r="B67" s="3" t="inlineStr">
         <is>
           <t>D10</t>
         </is>
       </c>
-      <c r="C66" s="3" t="inlineStr">
+      <c r="C67" s="3" t="inlineStr">
         <is>
           <t>Provisional local rules for notifications (portal only)</t>
         </is>
       </c>
-      <c r="D66" s="3" t="inlineStr">
+      <c r="D67" s="3" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
-      <c r="E66" s="3" t="n">
+      <c r="E67" s="3" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
BL-220 demo API reference and drift test, BL-223 status workbook, BL-229, seeded production times at working hours
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/BEE-portal-status.xlsx
+++ b/docs/tracking/BEE-portal-status.xlsx
@@ -6026,11 +6026,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E67"/>
+  <dimension ref="A1:E77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
     <col width="48" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
@@ -7496,21 +7496,21 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>WP11</t>
+          <t>DEMO-S1</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>AI demonstrations (local)</t>
+          <t>Demo: payment simulation (V52-V53); built, not independently reviewed</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E59" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="60">
@@ -7521,21 +7521,21 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>WP07.x</t>
+          <t>DEMO-S2</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>Payment simulation, reconciliation, production, bulk, CA evidence, refunds (BL-211)</t>
+          <t>Demo: QR batch and serial with duplicate control (V54-V55); built, not independently reviewed</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E60" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="61">
@@ -7546,21 +7546,21 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>WP08.x</t>
+          <t>DEMO-S3</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>QR batch, serial and duplicate control (BL-212); package not accepted</t>
+          <t>Demo: simulated Fabric ledger, hash chain, revoke/amend (V56-V58); built, not independently reviewed</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E61" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="62">
@@ -7571,21 +7571,21 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>WP09.x</t>
+          <t>DEMO-S4</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>Fabric adapter, hash proof, pending/amend/revoke (BL-213); package not accepted</t>
+          <t>Demo: quarterly production submission (V59-V60); built, not independently reviewed</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E62" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="63">
@@ -7596,37 +7596,37 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>WP10.x</t>
+          <t>DEMO-S5</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>Cases, sampling, partner assignment, tickets (BL-214); package not accepted</t>
+          <t>Demo: MIS dashboard (V61); built, not independently reviewed</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E63" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>Platform</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>WP01</t>
+          <t>DEMO-S6</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>Documentation and design evidence</t>
+          <t>Demo: five AI use cases, advisory only (V62-V64); built, not independently reviewed</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
@@ -7641,75 +7641,325 @@
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>Backlog theme</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>BL-024/025</t>
+          <t>DEMO-LOGIN</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>Feature template and OpenAPI split</t>
+          <t>Demo-only username and password sign-in (off by default), role landing, offline fonts; gate 2176 passed, 0 failed</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E65" s="3" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>Backlog theme</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>BL-040–042</t>
+          <t>DEMO-NOTIFY</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+          <t>Demo: simulated email and SMS notifications from payment, ledger and production events (V66), Notifications screen and unread badge; gate 2176 passed, 0 failed</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E66" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
+          <t>Work package</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>DEMO-EXPORT</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>Demo: Download CSV on every list, QR serial file, printable certificate with QR code; gate 2176 passed, 0 failed</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>Work package</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>DEMO-POLISH</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>Demo: IST times, realistic seeded dates and anomaly data, helpdesk model card text (V65); built, not independently reviewed</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>Work package</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>WP11</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>AI demonstrations (local)</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>Work package</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>WP07.x</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>Payment simulation, reconciliation, production, bulk, CA evidence, refunds (BL-211)</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>Work package</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>WP08.x</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>QR batch, serial and duplicate control (BL-212); package not accepted</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>Work package</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>WP09.x</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>Fabric adapter, hash proof, pending/amend/revoke (BL-213); package not accepted</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>Work package</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>WP10.x</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>Cases, sampling, partner assignment, tickets (BL-214); package not accepted</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>WP01</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>Documentation and design evidence</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>Backlog theme</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>BL-024/025</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>Feature template and OpenAPI split</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>Backlog theme</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>BL-040–042</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
           <t>Owner decision</t>
         </is>
       </c>
-      <c r="B67" s="3" t="inlineStr">
+      <c r="B77" s="3" t="inlineStr">
         <is>
           <t>D10</t>
         </is>
       </c>
-      <c r="C67" s="3" t="inlineStr">
+      <c r="C77" s="3" t="inlineStr">
         <is>
           <t>Provisional local rules for notifications (portal only)</t>
         </is>
       </c>
-      <c r="D67" s="3" t="inlineStr">
+      <c r="D77" s="3" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
-      <c r="E67" s="3" t="n">
+      <c r="E77" s="3" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
BL-220 demo API reference and drift test, BL-223 status workbook, BL-229, seeded production times at working hours (#68)
Co-authored-by: Sameer Khanna <sameerkhanna@Sameers-MacBook-Pro.local>
Co-authored-by: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tracking/BEE-portal-status.xlsx
+++ b/docs/tracking/BEE-portal-status.xlsx
@@ -6026,11 +6026,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E67"/>
+  <dimension ref="A1:E77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
     <col width="48" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="13" customWidth="1" min="5" max="5"/>
@@ -7496,21 +7496,21 @@
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>WP11</t>
+          <t>DEMO-S1</t>
         </is>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>AI demonstrations (local)</t>
+          <t>Demo: payment simulation (V52-V53); built, not independently reviewed</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E59" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="60">
@@ -7521,21 +7521,21 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>WP07.x</t>
+          <t>DEMO-S2</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>Payment simulation, reconciliation, production, bulk, CA evidence, refunds (BL-211)</t>
+          <t>Demo: QR batch and serial with duplicate control (V54-V55); built, not independently reviewed</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E60" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="61">
@@ -7546,21 +7546,21 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>WP08.x</t>
+          <t>DEMO-S3</t>
         </is>
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>QR batch, serial and duplicate control (BL-212); package not accepted</t>
+          <t>Demo: simulated Fabric ledger, hash chain, revoke/amend (V56-V58); built, not independently reviewed</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E61" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="62">
@@ -7571,21 +7571,21 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>WP09.x</t>
+          <t>DEMO-S4</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>Fabric adapter, hash proof, pending/amend/revoke (BL-213); package not accepted</t>
+          <t>Demo: quarterly production submission (V59-V60); built, not independently reviewed</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E62" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="63">
@@ -7596,37 +7596,37 @@
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>WP10.x</t>
+          <t>DEMO-S5</t>
         </is>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>Cases, sampling, partner assignment, tickets (BL-214); package not accepted</t>
+          <t>Demo: MIS dashboard (V61); built, not independently reviewed</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E63" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>Platform</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>WP01</t>
+          <t>DEMO-S6</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>Documentation and design evidence</t>
+          <t>Demo: five AI use cases, advisory only (V62-V64); built, not independently reviewed</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
@@ -7641,75 +7641,325 @@
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>Backlog theme</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>BL-024/025</t>
+          <t>DEMO-LOGIN</t>
         </is>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>Feature template and OpenAPI split</t>
+          <t>Demo-only username and password sign-in (off by default), role landing, offline fonts; gate 2176 passed, 0 failed</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E65" s="3" t="n">
-        <v>40</v>
+        <v>100</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>Backlog theme</t>
+          <t>Work package</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>BL-040–042</t>
+          <t>DEMO-NOTIFY</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+          <t>Demo: simulated email and SMS notifications from payment, ledger and production events (V66), Notifications screen and unread badge; gate 2176 passed, 0 failed</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="E66" s="3" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
+          <t>Work package</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>DEMO-EXPORT</t>
+        </is>
+      </c>
+      <c r="C67" s="3" t="inlineStr">
+        <is>
+          <t>Demo: Download CSV on every list, QR serial file, printable certificate with QR code; gate 2176 passed, 0 failed</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>Work package</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>DEMO-POLISH</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>Demo: IST times, realistic seeded dates and anomaly data, helpdesk model card text (V65); built, not independently reviewed</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="3" t="inlineStr">
+        <is>
+          <t>Work package</t>
+        </is>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>WP11</t>
+        </is>
+      </c>
+      <c r="C69" s="3" t="inlineStr">
+        <is>
+          <t>AI demonstrations (local)</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>Work package</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>WP07.x</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>Payment simulation, reconciliation, production, bulk, CA evidence, refunds (BL-211)</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="3" t="inlineStr">
+        <is>
+          <t>Work package</t>
+        </is>
+      </c>
+      <c r="B71" s="3" t="inlineStr">
+        <is>
+          <t>WP08.x</t>
+        </is>
+      </c>
+      <c r="C71" s="3" t="inlineStr">
+        <is>
+          <t>QR batch, serial and duplicate control (BL-212); package not accepted</t>
+        </is>
+      </c>
+      <c r="D71" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="E71" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>Work package</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>WP09.x</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>Fabric adapter, hash proof, pending/amend/revoke (BL-213); package not accepted</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="3" t="inlineStr">
+        <is>
+          <t>Work package</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="inlineStr">
+        <is>
+          <t>WP10.x</t>
+        </is>
+      </c>
+      <c r="C73" s="3" t="inlineStr">
+        <is>
+          <t>Cases, sampling, partner assignment, tickets (BL-214); package not accepted</t>
+        </is>
+      </c>
+      <c r="D73" s="3" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="E73" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>Platform</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>WP01</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>Documentation and design evidence</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="3" t="inlineStr">
+        <is>
+          <t>Backlog theme</t>
+        </is>
+      </c>
+      <c r="B75" s="3" t="inlineStr">
+        <is>
+          <t>BL-024/025</t>
+        </is>
+      </c>
+      <c r="C75" s="3" t="inlineStr">
+        <is>
+          <t>Feature template and OpenAPI split</t>
+        </is>
+      </c>
+      <c r="D75" s="3" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="E75" s="3" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>Backlog theme</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>BL-040–042</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>BEE owner decisions (fees, masters, evidence gates)</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
+        <is>
           <t>Owner decision</t>
         </is>
       </c>
-      <c r="B67" s="3" t="inlineStr">
+      <c r="B77" s="3" t="inlineStr">
         <is>
           <t>D10</t>
         </is>
       </c>
-      <c r="C67" s="3" t="inlineStr">
+      <c r="C77" s="3" t="inlineStr">
         <is>
           <t>Provisional local rules for notifications (portal only)</t>
         </is>
       </c>
-      <c r="D67" s="3" t="inlineStr">
+      <c r="D77" s="3" t="inlineStr">
         <is>
           <t>Accepted</t>
         </is>
       </c>
-      <c r="E67" s="3" t="n">
+      <c r="E77" s="3" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>